<commit_message>
Add long-term and short-term profiles in one combined report
- Rename Profile A to LT (profile_long_term.yaml) and add ST
  (profile_short_term.yaml); both share profiles/weighted_profile.py.
- run_ci.py / main.py (press Enter) score every profile and write one
  report, results_profile_LT_ST_..., with each profile's score, rank and
  flag columns. Yahoo downloads are reused across profiles.
- New Resilience concept (yearly / volatile-period consistency, worst
  3-month return); risk-adjusted and volatility use 1Y/5Y/10Y too.
- Fix: Maximum Drawdown is negative, so it is no longer inverted.
- Headers keep "LT"/"ST" uppercase; alerts, database, compare_results
  and the column dictionary handle the combined report.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_screener/docs/report_column_dictionary.xlsx
+++ b/etf_screener/docs/report_column_dictionary.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volatile Periods" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$113</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$252</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scoring Concepts'!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$258</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scoring Concepts'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volatile Periods'!$A$1:$H$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -489,7 +489,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Used In Profile A Score</t>
+          <t>Used In Profile LT Score</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Yes - 1W: YAML weight 0.05 = 5% of Short-term Return (≈0.5% of Profile A); 1M: YAML weight 0.15 = 16% of Short-term Return (≈1.6% of Profile A); 2M: YAML weight 0.15 = 16% of Short-term Return (≈1.6% of Profile A); QTD: YAML weight 0.15 = 16% of Short-term Return (≈1.6% of Profile A); 3M: YAML weight 0.15 = 16% of Short-term Return (≈1.6% of Profile A); 6M: YAML weight 0.12 = 13% of Short-term Return (≈1.2% of Profile A); 9M: YAML weight 0.1 = 11% of Short-term Return (≈1.0% of Profile A); YTD: YAML weight 0.05 = 5% of Short-term Return (≈0.5% of Profile A). Short-term Return = 9.5% of Profile A  |  Yes - 1Y: YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile A); 2Y: YAML weight 0.1 = 10% of Long-term Return (≈2.4% of Profile A); 3Y: YAML weight 0.095 = 10% of Long-term Return (≈2.3% of Profile A); 4Y: YAML weight 0.085 = 9% of Long-term Return (≈2.0% of Profile A); 5Y: YAML weight 0.075 = 8% of Long-term Return (≈1.8% of Profile A); 6Y: YAML weight 0.06 = 6% of Long-term Return (≈1.4% of Profile A); 7Y: YAML weight 0.06 = 6% of Long-term Return (≈1.4% of Profile A); 8Y: YAML weight 0.06 = 6% of Long-term Return (≈1.4% of Profile A); 9Y: YAML weight 0.065 = 7% of Long-term Return (≈1.6% of Profile A); 10Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile A); 15Y: YAML weight 0.085 = 9% of Long-term Return (≈2.0% of Profile A); 20Y: YAML weight 0.09 = 9% of Long-term Return (≈2.2% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - 1W: YAML weight 0.05 = 5% of Short-term Return (≈0.3% of Profile LT); 1M: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); 2M: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); QTD: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); 3M: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); 6M: YAML weight 0.12 = 13% of Short-term Return (≈0.6% of Profile LT); 9M: YAML weight 0.1 = 11% of Short-term Return (≈0.5% of Profile LT); YTD: YAML weight 0.05 = 5% of Short-term Return (≈0.3% of Profile LT). Short-term Return = 4.8% of Profile LT  |  Yes - 1Y: YAML weight 0.03 = 3% of Long-term Return (≈0.7% of Profile LT); 2Y: YAML weight 0.04 = 4% of Long-term Return (≈1.0% of Profile LT); 3Y: YAML weight 0.08 = 8% of Long-term Return (≈1.9% of Profile LT); 4Y: YAML weight 0.08 = 8% of Long-term Return (≈1.9% of Profile LT); 5Y: YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile LT); 6Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT); 7Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT); 8Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT); 9Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT); 10Y: YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile LT); 15Y: YAML weight 0.12 = 12% of Long-term Return (≈2.9% of Profile LT); 20Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈2.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈1.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1610,7 +1610,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈2.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈1.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1823,7 +1823,7 @@
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.45 = 30% of Risk-adjusted (≈5.7% of Profile A); 1Y: YAML weight 0.1 = 7% of Risk-adjusted (≈1.3% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - 1Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 3Y: YAML weight 0.2 = 20% of Risk-adjusted (≈3.8% of Profile LT); 5Y: YAML weight 0.15 = 15% of Risk-adjusted (≈2.9% of Profile LT); 10Y: YAML weight 0.1 = 10% of Risk-adjusted (≈1.9% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -1880,7 +1880,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.35 = 35% of Volatility (≈5.0% of Profile A). Volatility = 14.3% of Profile A</t>
+          <t>Yes - 3Y: YAML weight 0.2 = 20% of Volatility (≈2.9% of Profile LT); 5Y: YAML weight 0.15 = 15% of Volatility (≈2.1% of Profile LT); 10Y: YAML weight 0.05 = 5% of Volatility (≈0.7% of Profile LT). Volatility = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.2 = 20% of Resilience (≈1.9% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2092,7 +2092,7 @@
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.25 = 17% of Risk-adjusted (≈3.2% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - 3Y: YAML weight 0.1 = 10% of Risk-adjusted (≈1.9% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.2 = 13% of Risk-adjusted (≈2.5% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - 3Y: YAML weight 0.1 = 10% of Risk-adjusted (≈1.9% of Profile LT); 5Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 10Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>The worst pain an investor would have felt. 5Y includes the 2022 bear market. HIGH sector distortion (cyclical semis vs software).</t>
+          <t>The worst pain an investor would have felt. 5Y includes the 2022 bear market. HIGH sector distortion (cyclical semis vs software). Scored as-is (not inverted): the higher, less negative value scores better.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.35 = 35% of Volatility (≈5.0% of Profile A); 5Y: YAML weight 0.3 = 30% of Volatility (≈4.3% of Profile A). Volatility = 14.3% of Profile A</t>
+          <t>Yes - 3Y: YAML weight 0.2 = 20% of Volatility (≈2.9% of Profile LT); 5Y: YAML weight 0.25 = 25% of Volatility (≈3.6% of Profile LT); 10Y: YAML weight 0.15 = 15% of Volatility (≈2.1% of Profile LT). Volatility = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2479,7 +2479,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 1 = 100% of Costs (≈9.5% of Profile A). Costs = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 1 = 100% of Costs (≈9.5% of Profile LT). Costs = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -2585,7 +2585,7 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.6 = 100% of Liquidity/Size (≈4.8% of Profile A). Liquidity/Size = 4.8% of Profile A</t>
+          <t>Yes - YAML weight 0.6 = 100% of Liquidity/Size (≈4.8% of Profile LT). Liquidity/Size = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 20% of Quality/Valuation (≈2.9% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.2 = 20% of Quality/Valuation (≈1.9% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="H49" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I49" s="2" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>Yes - Wide: YAML weight 0.05 = 5% of Quality/Valuation (≈0.7% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - Wide: YAML weight 0.05 = 5% of Quality/Valuation (≈0.5% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I56" s="2" t="inlineStr">
@@ -3282,7 +3282,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.55 = 55% of Tracking (≈2.6% of Profile A); 1Y: YAML weight 0.45 = 45% of Tracking (≈2.1% of Profile A). Tracking = 4.8% of Profile A</t>
+          <t>Yes - 3Y: YAML weight 0.55 = 55% of Tracking (≈2.6% of Profile LT); 1Y: YAML weight 0.45 = 45% of Tracking (≈2.1% of Profile LT). Tracking = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
@@ -3388,7 +3388,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>Yes - Overall: YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - Overall: YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>Yes - Overall: YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - Overall: YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
@@ -3559,7 +3559,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>No - Tax/Income has 0 weight in Profile A (inputs: 1Y: YAML weight 0.2 = 29% of Tax/Income (≈0.0% of Profile A); 2Y: YAML weight 0.15 = 21% of Tax/Income (≈0.0% of Profile A))</t>
+          <t>No - Tax/Income has 0 weight in Profile LT (inputs: 1Y: YAML weight 0.2 = 29% of Tax/Income (≈0.0% of Profile LT); 2Y: YAML weight 0.15 = 21% of Tax/Income (≈0.0% of Profile LT))</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>No - Tax/Income has 0 weight in Profile A (inputs: YAML weight 0.25 = 36% of Tax/Income (≈0.0% of Profile A))</t>
+          <t>No - Tax/Income has 0 weight in Profile LT (inputs: YAML weight 0.25 = 36% of Tax/Income (≈0.0% of Profile LT))</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr">
@@ -3775,7 +3775,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>No - Tax/Income has 0 weight in Profile A (inputs: Trailing Annual: YAML weight 0.1 = 14% of Tax/Income (≈0.0% of Profile A))</t>
+          <t>No - Tax/Income has 0 weight in Profile LT (inputs: Trailing Annual: YAML weight 0.1 = 14% of Tax/Income (≈0.0% of Profile LT))</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -4683,7 +4683,7 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.1 = 7% of Risk-adjusted (≈1.3% of Profile A); 1Y: YAML weight 0.15 = 10% of Risk-adjusted (≈1.9% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - 3Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 1Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr"/>
@@ -4728,7 +4728,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.1 = 7% of Risk-adjusted (≈1.3% of Profile A); 1Y: YAML weight 0.15 = 10% of Risk-adjusted (≈1.9% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - 3Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 1Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr"/>
@@ -4822,7 +4822,7 @@
       <c r="B91" s="2" t="inlineStr"/>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1Y-20Y (1Y 15%, 2Y 10%, 3Y 9.5%, 4Y 8.5%, 5Y 7.5%, 6-8Y 6% each, 9Y 6.5%, 10Y 7%, 15Y 8.5%, 20Y 9%).</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1Y 3%, Total Return 2Y 4%, Total Return 3Y 8%, Total Return 4Y 8%, Total Return 5Y 15%, Total Return 6Y 7%, Total Return 7Y 7%, Total Return 8Y 7%, Total Return 9Y 7%, Total Return 10Y 15%, Total Return 15Y 12%, Total Return 20Y 7%.</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -4847,7 +4847,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr"/>
@@ -4863,7 +4863,7 @@
       <c r="B92" s="2" t="inlineStr"/>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1W 5%, 1M / 2M / QTD / 3M 15% each, 6M 12%, 9M 10%, YTD 5%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1W 5%, Total Return 1M 16%, Total Return 2M 16%, Total Return QTD 16%, Total Return 3M 16%, Total Return 6M 13%, Total Return 9M 11%, Total Return YTD 5%.</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -4888,7 +4888,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr"/>
@@ -4904,7 +4904,7 @@
       <c r="B93" s="2" t="inlineStr"/>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Morningstar Sharpe 3Y 45% / 1Y 10%, Upside Capture 3Y 25%, Downside Capture 3Y 20% (inverted), Yahoo Sharpe 3Y 10% / 1Y 15%, Z Score 3Y 10% / 1Y 15%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Morningstar Sharpe 1Y 5%, Morningstar Sharpe 3Y 20%, Morningstar Sharpe 5Y 15%, Morningstar Sharpe 10Y 10%, Upside Capture 3Y 10%, Downside Capture 3Y 10% (inverted), Downside Capture 5Y 5% (inverted), Downside Capture 10Y 5% (inverted), Yahoo Sharpe 1Y 5%, Yahoo Sharpe 3Y 5%, Z Score 1Y 5%, Z Score 3Y 5%.</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -4929,7 +4929,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr"/>
@@ -4945,7 +4945,7 @@
       <c r="B94" s="2" t="inlineStr"/>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Standard Deviation 3Y 35%, Max Drawdown 3Y 35%, 5Y 30% (all inverted).</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Standard Deviation 3Y 20% (inverted), Standard Deviation 5Y 15% (inverted), Standard Deviation 10Y 5% (inverted), Max Drawdown 3Y 20%, Max Drawdown 5Y 25%, Max Drawdown 10Y 15%.</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Blank for funds younger than 3 years.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Blank for funds younger than 3 years. Max drawdown is negative, so it is NOT inverted: closer to 0 scores higher.</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -4970,7 +4970,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr"/>
@@ -4980,13 +4980,13 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Tracking Score</t>
+          <t>Resilience Score</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr"/>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tracking Error 3Y 55%, 1Y 45% (inverted).</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Yearly Beat % 25%, Yearly Bottom 10% Count / Yearly Periods With Data 15% (inverted), Volatile Beat % 25%, Volatile Bottom 10% Count / Volatile Periods With Data 15% (inverted), Worst Three Month Return 20%.</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Good for index funds; for active funds low tracking error just means 'close to the index'.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. How consistently the fund beat the indexes: calendar years and the S&amp;P 500's volatile periods (crashes and recoveries). Bottom-10% counts are divided by the periods the fund has data for, so older funds aren't penalized for having more periods.</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile A</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr"/>
@@ -5021,13 +5021,13 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Liquidity Size Score</t>
+          <t>Tracking Score</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr"/>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Fund Size with fixed cutoffs ($10M → 0, $500M target, $5B → 100).</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tracking Error 3Y 55% (inverted), Tracking Error 1Y 45% (inverted).</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Not within category.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Good for index funds; for active funds low tracking error just means 'close to the index'.</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr"/>
@@ -5062,13 +5062,13 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Quality Valuation Score</t>
+          <t>Liquidity Size Score</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr"/>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Growth Grade 20%, Financial Health 15%, Profitability 15%, Price/Fair Value 15% (inverted), Medalist 15%, Star rating 15%, Wide moat 5%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Fund Size with fixed cutoffs ($10M → 0, $500M target, $5B → 100) 100%.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -5083,7 +5083,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Mostly equity data; bond funds rely on Medalist and stars.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Not within category.</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -5093,7 +5093,7 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr"/>
@@ -5103,13 +5103,13 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Costs Score</t>
+          <t>Quality Valuation Score</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr"/>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Adjusted Expense Ratio 100% (inverted).</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Growth Grade 20%, Financial Health 15%, Profitability 15%, Price/Fair Value 15% (inverted), Medalist 15%, Star rating 15%, Wide moat 5%.</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -5124,7 +5124,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Mostly equity data; bond funds rely on Medalist and stars.</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr"/>
@@ -5144,13 +5144,13 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Tax Income Score</t>
+          <t>Costs Score</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr"/>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tax Cost Ratio 1Y 20% / 2Y 15% (inverted), Dividend per Share 10% each x4, SEC 30-Day Yield 25%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Adjusted Expense Ratio 100% (inverted).</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>No - 0 weight in Profile A</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr"/>
@@ -5185,32 +5185,28 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Return Rank</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>1W, 1M, 2M, QTD, 3M, 6M, 9M, YTD, 1Y, 2Y, 3Y, 4Y, 5Y, 6Y, 7Y, 8Y, 9Y, 10Y, 15Y, 20Y</t>
-        </is>
-      </c>
+          <t>Tax Income Score</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr"/>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Rank of the matching 'Total Return' column across ALL funds in the report (1 = highest return).</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tax Cost Ratio 1Y 29% (inverted), Tax Cost Ratio 2Y 21% (inverted), Dividend per Share (Trailing) 14%, SEC 30-Day Yield 36%.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Rank = position when all funds are sorted by that period's return, highest first (ties share the lowest rank)</t>
+          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (1 = best)</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Across all categories, not within category - leveraged / sector funds dominate both ends. Used for the 1W &amp; 1M momentum tabs.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type.</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -5220,7 +5216,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - 0 weight in Profile LT</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr"/>
@@ -5230,28 +5226,32 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Profile A Score</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr"/>
+          <t>Return Rank</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>1W, 1M, 2M, QTD, 3M, 6M, 9M, YTD, 1Y, 2Y, 3Y, 4Y, 5Y, 6Y, 7Y, 8Y, 9Y, 10Y, 15Y, 20Y</t>
+        </is>
+      </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Final 0-100 score combining the nine concept scores with the weights in input_profile_a.yaml.</t>
+          <t>Rank of the matching 'Total Return' column across ALL funds in the report (1 = highest return).</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Profile A Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Long-term Return 0.25, Short-term Return 0.1, Risk-adjusted 0.2, Volatility 0.15, Tracking 0.05, Liquidity/Size 0.05, Quality/Valuation 0.15, Costs 0.1, Tax/Income 0 (sum 1.05, so each effective share = weight / 1.05)</t>
+          <t>Rank = position when all funds are sorted by that period's return, highest first (ties share the lowest rank)</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Higher is better</t>
+          <t>Lower is better (1 = best)</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'.</t>
+          <t>Across all categories, not within category - leveraged / sector funds dominate both ends. Used for the 1W &amp; 1M momentum tabs.</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -5261,7 +5261,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>This IS the Profile A score</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr"/>
@@ -5271,24 +5271,28 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Profile A Rank In Category</t>
+          <t>Profile LT Score</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr"/>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Rank of the Profile A Score within the fund's Morningstar Category (1 = best).</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr"/>
+          <t>Final 0-100 score combining the concept scores with the weights in profile_long_term.yaml.</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Profile LT Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Long-term Return 0.25, Short-term Return 0.05, Risk-adjusted 0.2, Volatility 0.15, Resilience 0.1, Tracking 0.05, Liquidity/Size 0.05, Quality/Valuation 0.1, Costs 0.1, Tax/Income 0 (sum 1.05, so each effective share = weight / 1.05)</t>
+        </is>
+      </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent.</t>
+          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'.</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -5298,7 +5302,7 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>This IS the Profile LT score</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr"/>
@@ -5308,28 +5312,24 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Profile A Selected Flag</t>
+          <t>Profile LT Rank In Category</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr"/>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is in the top 5 of its Morningstar Category by Profile A Score.</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr">
-        <is>
-          <t>Rank In Category ≤ top_n_per_category (5)</t>
-        </is>
-      </c>
+          <t>Rank of the Profile LT Score within the fund's Morningstar Category (1 = best).</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr"/>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>top_n_per_category is set in the YAML.</t>
+          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -5349,24 +5349,28 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Profile A Rank Overall</t>
+          <t>Profile LT Selected Flag</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr"/>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Rank of the Profile A Score across all funds (1 = best).</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr"/>
+          <t>1 if the fund is in the top 5 of its Morningstar Category by Profile LT Score.</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Rank In Category ≤ top_n_per_category (5)</t>
+        </is>
+      </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
+          <t>top_n_per_category is set in profile_long_term.yaml.</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -5386,26 +5390,26 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Profile A Selected Overall Flag</t>
+          <t>Profile LT Rank Overall</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr"/>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is in the top 5 overall.</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>Rank Overall ≤ 5</t>
-        </is>
-      </c>
+          <t>Rank of the Profile LT Score across all funds (1 = best).</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr"/>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr"/>
+          <t>Lower is better</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
+        </is>
+      </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
           <t>Screener (calculated)</t>
@@ -5423,26 +5427,26 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Missing From Yahoo</t>
+          <t>Profile LT Selected Overall Flag</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr"/>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>('No Yahoo Data' tab only) Which Yahoo-based results are missing: Sharpe / Z-score, yearly returns, volatile periods.</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr"/>
+          <t>1 if the fund is in the top 5 overall.</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Rank Overall ≤ 5</t>
+        </is>
+      </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>These funds are taken off the overview; all their Morningstar columns are still on that tab.</t>
-        </is>
-      </c>
+          <t>1 = selected</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr"/>
       <c r="G106" s="2" t="inlineStr">
         <is>
           <t>Screener (calculated)</t>
@@ -5460,28 +5464,28 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Top K Cutoff (rows needed)</t>
+          <t>Profile ST Score</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr"/>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>(Momentum tab) Smallest K such that at least 50 funds are within the best K funds for BOTH 1W and 1M return.</t>
+          <t>Final 0-100 score combining the concept scores with the weights in profile_short_term.yaml.</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>K = smallest number with ≥ 50 funds having 1W position ≤ K AND 1M position ≤ K</t>
+          <t>Profile ST Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Long-term Return 0.05, Short-term Return 0.4, Risk-adjusted 0.2, Volatility 0.1, Resilience 0, Tracking 0, Liquidity/Size 0.1, Quality/Valuation 0.05, Costs 0.1, Tax/Income 0 (sum 1, so each effective share = weight / 1)</t>
         </is>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Same value on every row.</t>
+          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'. Uses ST's own concept weights, so it can't be recomputed from the concept score columns in this report (those use LT's). Blank for funds profile_short_term.yaml filters out.</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -5491,7 +5495,7 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - this is the Profile ST score</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr"/>
@@ -5501,26 +5505,26 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Top Position</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr">
-        <is>
-          <t>1W, 1M</t>
-        </is>
-      </c>
+          <t>Profile ST Rank In Category</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr"/>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>(Momentum tab) Fund's position counted from the best 1-week (1W) or 1-month (1M) return (1 = best).</t>
+          <t>Rank of the Profile ST Score within the fund's Morningstar Category (1 = best).</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr"/>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Lower = stronger signal</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="inlineStr"/>
+          <t>Lower is better</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
+        </is>
+      </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
           <t>Screener (calculated)</t>
@@ -5538,28 +5542,28 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Bottom K Cutoff (rows needed)</t>
+          <t>Profile ST Selected Flag</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr"/>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>(Momentum tab) Smallest K such that at least 50 funds are within the worst K funds for BOTH 1W and 1M return.</t>
+          <t>1 if the fund is in the top 5 of its Morningstar Category by Profile ST Score.</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>K = smallest number with ≥ 50 funds having 1W position ≤ K AND 1M position ≤ K</t>
+          <t>Rank In Category ≤ top_n_per_category (5)</t>
         </is>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>Same value on every row.</t>
+          <t>top_n_per_category is set in profile_short_term.yaml.</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -5579,26 +5583,26 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Bottom Position</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr">
-        <is>
-          <t>1W, 1M</t>
-        </is>
-      </c>
+          <t>Profile ST Rank Overall</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr"/>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>(Momentum tab) Fund's position counted from the worst 1-week (1W) or 1-month (1M) return (1 = worst).</t>
+          <t>Rank of the Profile ST Score across all funds (1 = best).</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr"/>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Lower = stronger signal</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr"/>
+          <t>Lower is better</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
+        </is>
+      </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
           <t>Screener (calculated)</t>
@@ -5616,66 +5620,50 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Trading Volume</t>
+          <t>Profile ST Selected Overall Flag</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr"/>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window.</t>
+          <t>1 if the fund is in the top 5 overall.</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Reported directly from exchange data</t>
+          <t>Rank Overall ≤ 5</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>Higher = easier to trade at a fair price</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="inlineStr">
-        <is>
-          <t>Not in the current eTrade export. The YAML still gives it weight 0.4 in Liquidity/Size; since the column is missing, Fund Size gets the whole Liquidity/Size weight. Add it to the export to use it.</t>
-        </is>
-      </c>
+          <t>1 = selected</t>
+        </is>
+      </c>
+      <c r="F111" s="2" t="inlineStr"/>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>Morningstar (not in current data)</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>No effect: weighted 0.4 in the YAML, but the column is missing</t>
-        </is>
-      </c>
-      <c r="I111" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window. Key facts: Unit is shares, not dollars. Single-day volume and average volume are distinct fields; which one an export column holds depends on the data point chosen.</t>
-        </is>
-      </c>
-      <c r="J111" s="2" t="inlineStr">
-        <is>
-          <t>Corrected to Morningstar's definition</t>
-        </is>
-      </c>
-      <c r="K111" s="2" t="inlineStr">
-        <is>
-          <t>http://quote.morningstar.com/ETFdefinition.html</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I111" s="2" t="inlineStr"/>
+      <c r="J111" s="2" t="inlineStr"/>
+      <c r="K111" s="2" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Management Style</t>
+          <t>Missing From Yahoo</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr"/>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Whether the fund is run by a single manager, a team, or a committee.</t>
+          <t>('No Yahoo Data' tab only) Which Yahoo-based results are missing: Sharpe / Z-score, yearly returns, volatile periods.</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr"/>
@@ -5686,12 +5674,12 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>Mentioned in column_glossary.md; not in the current export and not used in scoring.</t>
+          <t>These funds are taken off the overview; all their Morningstar columns are still on that tab.</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>Morningstar (not in current data)</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -5699,77 +5687,323 @@
           <t>No</t>
         </is>
       </c>
-      <c r="I112" s="2" t="inlineStr">
-        <is>
-          <t>Not found. The closest Morningstar definitions: 'Management Team' is used when more than two people manage the fund together or the fund strongly promotes a team approach; 'Multiple Managers' is used when people manage portions independently. Key facts: When a fund lists only 'Management Team' without names, Morningstar shows manager tenure as a dash.</t>
-        </is>
-      </c>
-      <c r="J112" s="2" t="inlineStr">
-        <is>
-          <t>No Morningstar definition found</t>
-        </is>
-      </c>
-      <c r="K112" s="2" t="inlineStr">
-        <is>
-          <t>https://awgmain.morningstar.com/webhelp/glossary_definitions/mutual_fund/Manager_Tenure_(Longest).htm</t>
-        </is>
-      </c>
+      <c r="I112" s="2" t="inlineStr"/>
+      <c r="J112" s="2" t="inlineStr"/>
+      <c r="K112" s="2" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>3Y Return Rank in Category</t>
+          <t>Top K Cutoff (rows needed)</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr"/>
       <c r="C113" s="2" t="inlineStr">
         <is>
+          <t>(Momentum tab) Smallest K such that at least 50 funds are within the best K funds for BOTH 1W and 1M return.</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>K = smallest number with ≥ 50 funds having 1W position ≤ K AND 1M position ≤ K</t>
+        </is>
+      </c>
+      <c r="E113" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>Same value on every row.</t>
+        </is>
+      </c>
+      <c r="G113" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="H113" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr"/>
+      <c r="J113" s="2" t="inlineStr"/>
+      <c r="K113" s="2" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Top Position</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>1W, 1M</t>
+        </is>
+      </c>
+      <c r="C114" s="2" t="inlineStr">
+        <is>
+          <t>(Momentum tab) Fund's position counted from the best 1-week (1W) or 1-month (1M) return (1 = best).</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr"/>
+      <c r="E114" s="2" t="inlineStr">
+        <is>
+          <t>Lower = stronger signal</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr"/>
+      <c r="G114" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I114" s="2" t="inlineStr"/>
+      <c r="J114" s="2" t="inlineStr"/>
+      <c r="K114" s="2" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Bottom K Cutoff (rows needed)</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr"/>
+      <c r="C115" s="2" t="inlineStr">
+        <is>
+          <t>(Momentum tab) Smallest K such that at least 50 funds are within the worst K funds for BOTH 1W and 1M return.</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>K = smallest number with ≥ 50 funds having 1W position ≤ K AND 1M position ≤ K</t>
+        </is>
+      </c>
+      <c r="E115" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>Same value on every row.</t>
+        </is>
+      </c>
+      <c r="G115" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I115" s="2" t="inlineStr"/>
+      <c r="J115" s="2" t="inlineStr"/>
+      <c r="K115" s="2" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Bottom Position</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>1W, 1M</t>
+        </is>
+      </c>
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>(Momentum tab) Fund's position counted from the worst 1-week (1W) or 1-month (1M) return (1 = worst).</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr"/>
+      <c r="E116" s="2" t="inlineStr">
+        <is>
+          <t>Lower = stronger signal</t>
+        </is>
+      </c>
+      <c r="F116" s="2" t="inlineStr"/>
+      <c r="G116" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="inlineStr"/>
+      <c r="J116" s="2" t="inlineStr"/>
+      <c r="K116" s="2" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Trading Volume</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr"/>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window.</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>Reported directly from exchange data</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>Higher = easier to trade at a fair price</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>Not in the current eTrade export. The YAML still gives it weight 0.4 in Liquidity/Size; since the column is missing, Fund Size gets the whole Liquidity/Size weight. Add it to the export to use it.</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>Morningstar (not in current data)</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>No effect: weighted 0.4 in the YAML, but the column is missing</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
+        <is>
+          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window. Key facts: Unit is shares, not dollars. Single-day volume and average volume are distinct fields; which one an export column holds depends on the data point chosen.</t>
+        </is>
+      </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>Corrected to Morningstar's definition</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr">
+        <is>
+          <t>http://quote.morningstar.com/ETFdefinition.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>Management Style</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr"/>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Whether the fund is run by a single manager, a team, or a committee.</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr"/>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>Mentioned in column_glossary.md; not in the current export and not used in scoring.</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>Morningstar (not in current data)</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
+        <is>
+          <t>Not found. The closest Morningstar definitions: 'Management Team' is used when more than two people manage the fund together or the fund strongly promotes a team approach; 'Multiple Managers' is used when people manage portions independently. Key facts: When a fund lists only 'Management Team' without names, Morningstar shows manager tenure as a dash.</t>
+        </is>
+      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>No Morningstar definition found</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr">
+        <is>
+          <t>https://awgmain.morningstar.com/webhelp/glossary_definitions/mutual_fund/Manager_Tenure_(Longest).htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>3Y Return Rank in Category</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr"/>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
           <t>Morningstar's percentile rank of the fund's 3-year return within its category (1 = best).</t>
         </is>
       </c>
-      <c r="D113" s="2" t="inlineStr">
+      <c r="D119" s="2" t="inlineStr">
         <is>
           <t>Morningstar computes this; lower rank = better</t>
         </is>
       </c>
-      <c r="E113" s="2" t="inlineStr">
+      <c r="E119" s="2" t="inlineStr">
         <is>
           <t>Lower is better</t>
         </is>
       </c>
-      <c r="F113" s="2" t="inlineStr">
+      <c r="F119" s="2" t="inlineStr">
         <is>
           <t>Used by the old single 'Performance' concept, which has since been split into Long-term and Short-term Return. Not in the current export.</t>
         </is>
       </c>
-      <c r="G113" s="2" t="inlineStr">
+      <c r="G119" s="2" t="inlineStr">
         <is>
           <t>Morningstar (not in current data)</t>
         </is>
       </c>
-      <c r="H113" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I113" s="2" t="inlineStr">
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I119" s="2" t="inlineStr">
         <is>
           <t>The fund's 3-year total-return percentile rank among all funds in the same Morningstar Category, on a 1-100 scale where 1 is the best (highest return) and 100 the worst. Key facts: Based on total return, not adjusted for sales loads (Morningstar publishes load-adjusted ranks separately). Only funds with a full 3-year history are ranked. Lower = better for returns.</t>
         </is>
       </c>
-      <c r="J113" s="2" t="inlineStr">
+      <c r="J119" s="2" t="inlineStr">
         <is>
           <t>Matches Morningstar</t>
         </is>
       </c>
-      <c r="K113" s="2" t="inlineStr">
+      <c r="K119" s="2" t="inlineStr">
         <is>
           <t>https://awgmain.morningstar.com/webhelp/glossary_definitions/mutual_fund/mfglossary_PercentileRankCategory.html</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K113"/>
+  <autoFilter ref="A1:K119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5780,7 +6014,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G252"/>
+  <dimension ref="A1:G258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -5825,7 +6059,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Used In Profile A Score</t>
+          <t>Used In Profile LT Score</t>
         </is>
       </c>
     </row>
@@ -6159,7 +6393,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 5% of Short-term Return (≈0.5% of Profile A). Short-term Return = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 5% of Short-term Return (≈0.3% of Profile LT). Short-term Return = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6196,7 +6430,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 16% of Short-term Return (≈1.6% of Profile A). Short-term Return = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT). Short-term Return = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6467,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 16% of Short-term Return (≈1.6% of Profile A). Short-term Return = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT). Short-term Return = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6270,7 +6504,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 16% of Short-term Return (≈1.6% of Profile A). Short-term Return = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT). Short-term Return = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6541,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 16% of Short-term Return (≈1.6% of Profile A). Short-term Return = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT). Short-term Return = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6344,7 +6578,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.12 = 13% of Short-term Return (≈1.2% of Profile A). Short-term Return = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.12 = 13% of Short-term Return (≈0.6% of Profile LT). Short-term Return = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6381,7 +6615,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 11% of Short-term Return (≈1.0% of Profile A). Short-term Return = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.1 = 11% of Short-term Return (≈0.5% of Profile LT). Short-term Return = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6418,7 +6652,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 5% of Short-term Return (≈0.5% of Profile A). Short-term Return = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 5% of Short-term Return (≈0.3% of Profile LT). Short-term Return = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6455,7 +6689,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.03 = 3% of Long-term Return (≈0.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6492,7 +6726,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 10% of Long-term Return (≈2.4% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.04 = 4% of Long-term Return (≈1.0% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6763,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.095 = 10% of Long-term Return (≈2.3% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.08 = 8% of Long-term Return (≈1.9% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6566,7 +6800,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.085 = 9% of Long-term Return (≈2.0% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.08 = 8% of Long-term Return (≈1.9% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6603,7 +6837,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.075 = 8% of Long-term Return (≈1.8% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6640,7 +6874,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.06 = 6% of Long-term Return (≈1.4% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6677,7 +6911,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.06 = 6% of Long-term Return (≈1.4% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6714,7 +6948,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.06 = 6% of Long-term Return (≈1.4% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6751,7 +6985,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.065 = 7% of Long-term Return (≈1.6% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6788,7 +7022,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6825,7 +7059,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.085 = 9% of Long-term Return (≈2.0% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.12 = 12% of Long-term Return (≈2.9% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6862,7 +7096,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.09 = 9% of Long-term Return (≈2.2% of Profile A). Long-term Return = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7635,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈2.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -7833,7 +8067,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈1.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9297,7 +9531,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈2.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9729,7 +9963,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈1.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9766,7 +10000,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 7% of Risk-adjusted (≈1.3% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9803,7 +10037,7 @@
       </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.45 = 30% of Risk-adjusted (≈5.7% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.2 = 20% of Risk-adjusted (≈3.8% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9840,7 +10074,7 @@
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.15 = 15% of Risk-adjusted (≈2.9% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9877,7 +10111,7 @@
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.1 = 10% of Risk-adjusted (≈1.9% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9951,7 +10185,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.35 = 35% of Volatility (≈5.0% of Profile A). Volatility = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.2 = 20% of Volatility (≈2.9% of Profile LT). Volatility = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9988,7 +10222,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.15 = 15% of Volatility (≈2.1% of Profile LT). Volatility = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10025,7 +10259,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.05 = 5% of Volatility (≈0.7% of Profile LT). Volatility = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10058,7 +10292,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.2 = 20% of Resilience (≈1.9% of Profile LT). Resilience = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10313,7 +10547,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 17% of Risk-adjusted (≈3.2% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.1 = 10% of Risk-adjusted (≈1.9% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10461,7 +10695,7 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 13% of Risk-adjusted (≈2.5% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.1 = 10% of Risk-adjusted (≈1.9% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10498,7 +10732,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10535,7 +10769,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10609,7 +10843,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.35 = 35% of Volatility (≈5.0% of Profile A). Volatility = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.2 = 20% of Volatility (≈2.9% of Profile LT). Volatility = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10646,7 +10880,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.3 = 30% of Volatility (≈4.3% of Profile A). Volatility = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.25 = 25% of Volatility (≈3.6% of Profile LT). Volatility = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10683,7 +10917,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.15 = 15% of Volatility (≈2.1% of Profile LT). Volatility = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10856,7 +11090,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 1 = 100% of Costs (≈9.5% of Profile A). Costs = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 1 = 100% of Costs (≈9.5% of Profile LT). Costs = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10922,7 +11156,7 @@
       </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.6 = 100% of Liquidity/Size (≈4.8% of Profile A). Liquidity/Size = 4.8% of Profile A</t>
+          <t>Yes - YAML weight 0.6 = 100% of Liquidity/Size (≈4.8% of Profile LT). Liquidity/Size = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -11025,7 +11259,7 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 20% of Quality/Valuation (≈2.9% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.2 = 20% of Quality/Valuation (≈1.9% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -11058,7 +11292,7 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -11091,7 +11325,7 @@
       </c>
       <c r="G147" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -11128,7 +11362,7 @@
       </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 5% of Quality/Valuation (≈0.7% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 5% of Quality/Valuation (≈0.5% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -11400,7 +11634,7 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -11470,7 +11704,7 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.45 = 45% of Tracking (≈2.1% of Profile A). Tracking = 4.8% of Profile A</t>
+          <t>Yes - YAML weight 0.45 = 45% of Tracking (≈2.1% of Profile LT). Tracking = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -11507,7 +11741,7 @@
       </c>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.55 = 55% of Tracking (≈2.6% of Profile A). Tracking = 4.8% of Profile A</t>
+          <t>Yes - YAML weight 0.55 = 55% of Tracking (≈2.6% of Profile LT). Tracking = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -11651,7 +11885,7 @@
       </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -11799,7 +12033,7 @@
       </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈2.1% of Profile A). Quality/Valuation = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 15% of Quality/Valuation (≈1.4% of Profile LT). Quality/Valuation = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -12095,7 +12329,7 @@
       </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>No - Tax/Income has 0 weight in Profile A (inputs: YAML weight 0.2 = 29% of Tax/Income (≈0.0% of Profile A))</t>
+          <t>No - Tax/Income has 0 weight in Profile LT (inputs: YAML weight 0.2 = 29% of Tax/Income (≈0.0% of Profile LT))</t>
         </is>
       </c>
     </row>
@@ -12132,7 +12366,7 @@
       </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>No - Tax/Income has 0 weight in Profile A (inputs: YAML weight 0.15 = 21% of Tax/Income (≈0.0% of Profile A))</t>
+          <t>No - Tax/Income has 0 weight in Profile LT (inputs: YAML weight 0.15 = 21% of Tax/Income (≈0.0% of Profile LT))</t>
         </is>
       </c>
     </row>
@@ -12309,7 +12543,7 @@
       </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>No - Tax/Income has 0 weight in Profile A (inputs: YAML weight 0.25 = 36% of Tax/Income (≈0.0% of Profile A))</t>
+          <t>No - Tax/Income has 0 weight in Profile LT (inputs: YAML weight 0.25 = 36% of Tax/Income (≈0.0% of Profile LT))</t>
         </is>
       </c>
     </row>
@@ -12379,7 +12613,7 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>No - Tax/Income has 0 weight in Profile A (inputs: YAML weight 0.1 = 14% of Tax/Income (≈0.0% of Profile A))</t>
+          <t>No - Tax/Income has 0 weight in Profile LT (inputs: YAML weight 0.1 = 14% of Tax/Income (≈0.0% of Profile LT))</t>
         </is>
       </c>
     </row>
@@ -13154,7 +13388,7 @@
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 10% of Risk-adjusted (≈1.9% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13191,7 +13425,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 7% of Risk-adjusted (≈1.3% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13228,7 +13462,7 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 10% of Risk-adjusted (≈1.9% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13265,7 +13499,7 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 7% of Risk-adjusted (≈1.3% of Profile A). Risk-adjusted = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13364,7 +13598,7 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 23.8% of Profile A</t>
+          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13397,7 +13631,7 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13430,7 +13664,7 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 19.0% of Profile A</t>
+          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13463,14 +13697,14 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Tracking Score</t>
+          <t>Resilience Score</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -13480,7 +13714,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Tracking Score</t>
+          <t>Resilience Score</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr"/>
@@ -13496,14 +13730,14 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile A</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Liquidity Size Score</t>
+          <t>Tracking Score</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -13513,7 +13747,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>Liquidity Size Score</t>
+          <t>Tracking Score</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr"/>
@@ -13529,14 +13763,14 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Quality Valuation Score</t>
+          <t>Liquidity Size Score</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -13546,7 +13780,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Quality Valuation Score</t>
+          <t>Liquidity Size Score</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr"/>
@@ -13562,14 +13796,14 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile A</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Costs Score</t>
+          <t>Quality Valuation Score</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -13579,7 +13813,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>Costs Score</t>
+          <t>Quality Valuation Score</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr"/>
@@ -13595,14 +13829,14 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile A</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Tax Income Score</t>
+          <t>Costs Score</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -13612,7 +13846,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Tax Income Score</t>
+          <t>Costs Score</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr"/>
@@ -13628,14 +13862,14 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>No - 0 weight in Profile A</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (1W)</t>
+          <t>Tax Income Score</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -13645,17 +13879,13 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>Return Rank</t>
-        </is>
-      </c>
-      <c r="D221" s="2" t="inlineStr">
-        <is>
-          <t>1W</t>
-        </is>
-      </c>
+          <t>Tax Income Score</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr"/>
       <c r="E221" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (1 = best)</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F221" s="2" t="inlineStr">
@@ -13665,14 +13895,14 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - 0 weight in Profile LT</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (1M)</t>
+          <t>Return Rank (1W)</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -13687,7 +13917,7 @@
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>1W</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
@@ -13709,7 +13939,7 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (2M)</t>
+          <t>Return Rank (1M)</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -13724,7 +13954,7 @@
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>2M</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr">
@@ -13746,7 +13976,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (QTD)</t>
+          <t>Return Rank (2M)</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -13761,7 +13991,7 @@
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>QTD</t>
+          <t>2M</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
@@ -13783,7 +14013,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (3M)</t>
+          <t>Return Rank (QTD)</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -13798,7 +14028,7 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>3M</t>
+          <t>QTD</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
@@ -13820,7 +14050,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (6M)</t>
+          <t>Return Rank (3M)</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -13835,7 +14065,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>6M</t>
+          <t>3M</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
@@ -13857,7 +14087,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (9M)</t>
+          <t>Return Rank (6M)</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -13872,7 +14102,7 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>9M</t>
+          <t>6M</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
@@ -13894,7 +14124,7 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (YTD)</t>
+          <t>Return Rank (9M)</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -13909,7 +14139,7 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>YTD</t>
+          <t>9M</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
@@ -13931,7 +14161,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (1Y)</t>
+          <t>Return Rank (YTD)</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -13946,7 +14176,7 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>1Y</t>
+          <t>YTD</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
@@ -13968,7 +14198,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (2Y)</t>
+          <t>Return Rank (1Y)</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -13983,7 +14213,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2Y</t>
+          <t>1Y</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
@@ -14005,7 +14235,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (3Y)</t>
+          <t>Return Rank (2Y)</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -14020,7 +14250,7 @@
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>3Y</t>
+          <t>2Y</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
@@ -14042,7 +14272,7 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (4Y)</t>
+          <t>Return Rank (3Y)</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -14057,7 +14287,7 @@
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>4Y</t>
+          <t>3Y</t>
         </is>
       </c>
       <c r="E232" s="2" t="inlineStr">
@@ -14079,7 +14309,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (5Y)</t>
+          <t>Return Rank (4Y)</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -14094,7 +14324,7 @@
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>5Y</t>
+          <t>4Y</t>
         </is>
       </c>
       <c r="E233" s="2" t="inlineStr">
@@ -14116,7 +14346,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (6Y)</t>
+          <t>Return Rank (5Y)</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -14131,7 +14361,7 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>6Y</t>
+          <t>5Y</t>
         </is>
       </c>
       <c r="E234" s="2" t="inlineStr">
@@ -14153,7 +14383,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (7Y)</t>
+          <t>Return Rank (6Y)</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -14168,7 +14398,7 @@
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>7Y</t>
+          <t>6Y</t>
         </is>
       </c>
       <c r="E235" s="2" t="inlineStr">
@@ -14190,7 +14420,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (8Y)</t>
+          <t>Return Rank (7Y)</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -14205,7 +14435,7 @@
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>8Y</t>
+          <t>7Y</t>
         </is>
       </c>
       <c r="E236" s="2" t="inlineStr">
@@ -14227,7 +14457,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (9Y)</t>
+          <t>Return Rank (8Y)</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -14242,7 +14472,7 @@
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>9Y</t>
+          <t>8Y</t>
         </is>
       </c>
       <c r="E237" s="2" t="inlineStr">
@@ -14264,7 +14494,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (10Y)</t>
+          <t>Return Rank (9Y)</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -14279,7 +14509,7 @@
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>10Y</t>
+          <t>9Y</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr">
@@ -14301,7 +14531,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (15Y)</t>
+          <t>Return Rank (10Y)</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -14316,7 +14546,7 @@
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>15Y</t>
+          <t>10Y</t>
         </is>
       </c>
       <c r="E239" s="2" t="inlineStr">
@@ -14338,7 +14568,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (20Y)</t>
+          <t>Return Rank (15Y)</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -14353,7 +14583,7 @@
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>20Y</t>
+          <t>15Y</t>
         </is>
       </c>
       <c r="E240" s="2" t="inlineStr">
@@ -14375,7 +14605,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Profile A Score</t>
+          <t>Return Rank (20Y)</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -14385,13 +14615,17 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Profile A Score</t>
-        </is>
-      </c>
-      <c r="D241" s="2" t="inlineStr"/>
+          <t>Return Rank</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>20Y</t>
+        </is>
+      </c>
       <c r="E241" s="2" t="inlineStr">
         <is>
-          <t>Higher is better</t>
+          <t>Lower is better (1 = best)</t>
         </is>
       </c>
       <c r="F241" s="2" t="inlineStr">
@@ -14401,14 +14635,14 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>This IS the Profile A score</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>Profile A Rank In Category</t>
+          <t>Profile LT Score</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -14418,13 +14652,13 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Profile A Rank In Category</t>
+          <t>Profile LT Score</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr"/>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F242" s="2" t="inlineStr">
@@ -14434,14 +14668,14 @@
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>This IS the Profile LT score</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Profile A Selected Flag</t>
+          <t>Profile LT Rank In Category</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -14451,13 +14685,13 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>Profile A Selected Flag</t>
+          <t>Profile LT Rank In Category</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr"/>
       <c r="E243" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F243" s="2" t="inlineStr">
@@ -14474,7 +14708,7 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>Profile A Rank Overall</t>
+          <t>Profile LT Selected Flag</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -14484,13 +14718,13 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Profile A Rank Overall</t>
+          <t>Profile LT Selected Flag</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr"/>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F244" s="2" t="inlineStr">
@@ -14507,7 +14741,7 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>Profile A Selected Overall Flag</t>
+          <t>Profile LT Rank Overall</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -14517,13 +14751,13 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>Profile A Selected Overall Flag</t>
+          <t>Profile LT Rank Overall</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr"/>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F245" s="2" t="inlineStr">
@@ -14540,23 +14774,23 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>Missing From Yahoo</t>
+          <t>Profile LT Selected Overall Flag</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>No Yahoo Data</t>
+          <t>Overview (also on the extra tabs)</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Missing From Yahoo</t>
+          <t>Profile LT Selected Overall Flag</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr"/>
       <c r="E246" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F246" s="2" t="inlineStr">
@@ -14573,23 +14807,23 @@
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>Top K Cutoff (rows needed)</t>
+          <t>Profile ST Score</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>Top 50 / Bottom 50 momentum</t>
+          <t>Overview (also on the extra tabs)</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>Top K Cutoff (rows needed)</t>
+          <t>Profile ST Score</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr"/>
       <c r="E247" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F247" s="2" t="inlineStr">
@@ -14599,34 +14833,30 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - this is the Profile ST score</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>Top Position 1W</t>
+          <t>Profile ST Rank In Category</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>Top 50 / Bottom 50 momentum</t>
+          <t>Overview (also on the extra tabs)</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Top Position</t>
-        </is>
-      </c>
-      <c r="D248" s="2" t="inlineStr">
-        <is>
-          <t>1W</t>
-        </is>
-      </c>
+          <t>Profile ST Rank In Category</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr"/>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>Lower = stronger signal</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F248" s="2" t="inlineStr">
@@ -14643,27 +14873,23 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>Top Position 1M</t>
+          <t>Profile ST Selected Flag</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>Top 50 / Bottom 50 momentum</t>
+          <t>Overview (also on the extra tabs)</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>Top Position</t>
-        </is>
-      </c>
-      <c r="D249" s="2" t="inlineStr">
-        <is>
-          <t>1M</t>
-        </is>
-      </c>
+          <t>Profile ST Selected Flag</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr"/>
       <c r="E249" s="2" t="inlineStr">
         <is>
-          <t>Lower = stronger signal</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F249" s="2" t="inlineStr">
@@ -14680,23 +14906,23 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>Bottom K Cutoff (rows needed)</t>
+          <t>Profile ST Rank Overall</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>Top 50 / Bottom 50 momentum</t>
+          <t>Overview (also on the extra tabs)</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>Bottom K Cutoff (rows needed)</t>
+          <t>Profile ST Rank Overall</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr"/>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F250" s="2" t="inlineStr">
@@ -14713,27 +14939,23 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>Bottom Position 1W</t>
+          <t>Profile ST Selected Overall Flag</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>Top 50 / Bottom 50 momentum</t>
+          <t>Overview (also on the extra tabs)</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>Bottom Position</t>
-        </is>
-      </c>
-      <c r="D251" s="2" t="inlineStr">
-        <is>
-          <t>1W</t>
-        </is>
-      </c>
+          <t>Profile ST Selected Overall Flag</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr"/>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>Lower = stronger signal</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F251" s="2" t="inlineStr">
@@ -14750,42 +14972,252 @@
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
         <is>
+          <t>Missing From Yahoo</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>No Yahoo Data</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>Missing From Yahoo</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr"/>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>Top K Cutoff (rows needed)</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>Top 50 / Bottom 50 momentum</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>Top K Cutoff (rows needed)</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr"/>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>Top Position 1W</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>Top 50 / Bottom 50 momentum</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>Top Position</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>Lower = stronger signal</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>Top Position 1M</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>Top 50 / Bottom 50 momentum</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>Top Position</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>Lower = stronger signal</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>Bottom K Cutoff (rows needed)</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>Top 50 / Bottom 50 momentum</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>Bottom K Cutoff (rows needed)</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr"/>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>Bottom Position 1W</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>Top 50 / Bottom 50 momentum</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>Bottom Position</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>Lower = stronger signal</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>Screener (calculated)</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
           <t>Bottom Position 1M</t>
         </is>
       </c>
-      <c r="B252" s="2" t="inlineStr">
+      <c r="B258" s="2" t="inlineStr">
         <is>
           <t>Top 50 / Bottom 50 momentum</t>
         </is>
       </c>
-      <c r="C252" s="2" t="inlineStr">
+      <c r="C258" s="2" t="inlineStr">
         <is>
           <t>Bottom Position</t>
         </is>
       </c>
-      <c r="D252" s="2" t="inlineStr">
+      <c r="D258" s="2" t="inlineStr">
         <is>
           <t>1M</t>
         </is>
       </c>
-      <c r="E252" s="2" t="inlineStr">
+      <c r="E258" s="2" t="inlineStr">
         <is>
           <t>Lower = stronger signal</t>
         </is>
       </c>
-      <c r="F252" s="2" t="inlineStr">
+      <c r="F258" s="2" t="inlineStr">
         <is>
           <t>Screener (calculated)</t>
         </is>
       </c>
-      <c r="G252" s="2" t="inlineStr">
+      <c r="G258" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G252"/>
+  <autoFilter ref="A1:G258"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14796,7 +15228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -14821,7 +15253,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Effective share of Profile A</t>
+          <t>Effective share of Profile LT</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -14887,11 +15319,11 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>4.8%</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -14966,7 +15398,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Standard Deviation 3Y, Max Drawdown 3Y/5Y</t>
+          <t>Standard Deviation and Max Drawdown 1Y/3Y/5Y/10Y</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -14988,42 +15420,42 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>Resilience</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>4.8%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Tracking Error 1Y/3Y</t>
+          <t>Yearly / Volatile Beat %, share of years / periods in the bottom 10%, Worst Three Month Return</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Low-Medium</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Yes / Low</t>
+          <t>No / Moderate</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Benchmark-relative, so partly self-correcting.</t>
+          <t>Beating ALL the broad indexes favours whatever led the market (e.g. tech in 2023-24); defensive funds shine in the crash periods instead.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Liquidity/Size</t>
+          <t>Tracking</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
@@ -15036,64 +15468,64 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Fund Size</t>
+          <t>Tracking Error 1Y/3Y</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Low-Medium</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>No / No</t>
+          <t>Yes / Low</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Driven by popularity and age, not holdings.</t>
+          <t>Benchmark-relative, so partly self-correcting.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Quality/Valuation</t>
+          <t>Liquidity/Size</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>4.8%</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Grades, Price/Fair Value, Medalist, stars, moat</t>
+          <t>Fund Size</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Yes / High</t>
+          <t>No / No</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Growth grade and Price/Fair Value differ systematically software vs hardware.</t>
+          <t>Driven by popularity and age, not holdings.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Costs</t>
+          <t>Quality/Valuation</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
@@ -15106,62 +15538,97 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Adjusted Expense Ratio</t>
+          <t>Grades, Price/Fair Value, Medalist, stars, moat</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>No / No</t>
+          <t>Yes / High</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Driven by passive vs active, not composition.</t>
+          <t>Growth grade and Price/Fair Value differ systematically software vs hardware.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Costs</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>9.5%</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Adjusted Expense Ratio</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>No / No</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Driven by passive vs active, not composition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Tax/Income</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>Tax Cost Ratio, dividends, SEC yield</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Yes / Moderate</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Yield and distributions differ by sector maturity.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G10"/>
+  <autoFilter ref="A1:G11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add DuckDB query tool and top_n_overall; remove SQLite database and unused code
- profile YAMLs: new top-level top_n_overall controls the Selected Overall Flag
  separately from top_n_per_category; run_recorder now records top_n
- db_access/query.py: query any report, eTrade export or returns cache with SQL
  (DuckDB), with column search, saved queries and Excel export
- Top / Bottom 50 1W & 1M momentum tabs replaced by momentum_top / momentum_bottom queries
- Remove the SQLite database (database.py, import/query scripts, schema doc);
  history now comes from the saved reports
- Remove the older eTrade merge script, unused functions and config presets,
  and 22 expected columns the data doesn't have
- Fix requirements.txt (colorama and duckdb on separate lines)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_screener/docs/report_column_dictionary.xlsx
+++ b/etf_screener/docs/report_column_dictionary.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volatile Periods" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$119</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$258</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$252</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scoring Concepts'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volatile Periods'!$A$1:$H$25</definedName>
   </definedNames>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K119"/>
+  <dimension ref="A1:K115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -957,7 +957,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Compare within category - a 5% year is great for a bond fund and poor for a tech fund. Blank when the fund is younger than the period. 1W/1M feed the Top/Bottom 50 momentum tabs. Sector caveat: multi-year returns are strongly driven by sub-sector timing (e.g. AI semiconductors vs software), which within-category ranking does not correct for. 'Since Inception' is not comparable across funds with different start dates.</t>
+          <t>Compare within category - a 5% year is great for a bond fund and poor for a tech fund. Blank when the fund is younger than the period. Sector caveat: multi-year returns are strongly driven by sub-sector timing (e.g. AI semiconductors vs software), which within-category ranking does not correct for. 'Since Inception' is not comparable across funds with different start dates.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -5251,7 +5251,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Across all categories, not within category - leveraged / sector funds dominate both ends. Used for the 1W &amp; 1M momentum tabs.</t>
+          <t>Across all categories, not within category - leveraged / sector funds dominate both ends. For momentum lists use python db_access/query.py momentum_top / momentum_bottom.</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -5433,12 +5433,12 @@
       <c r="B106" s="2" t="inlineStr"/>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is in the top 5 overall.</t>
+          <t>1 if the fund is in the top 100 overall.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Rank Overall ≤ 5</t>
+          <t>Rank Overall ≤ top_n_overall (100)</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
@@ -5446,7 +5446,11 @@
           <t>1 = selected</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>top_n_overall is set in profile_long_term.yaml (if left out, top_n_per_category is used).</t>
+        </is>
+      </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
           <t>Screener (calculated)</t>
@@ -5626,12 +5630,12 @@
       <c r="B111" s="2" t="inlineStr"/>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is in the top 5 overall.</t>
+          <t>1 if the fund is in the top 25 overall.</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Rank Overall ≤ 5</t>
+          <t>Rank Overall ≤ top_n_overall (25)</t>
         </is>
       </c>
       <c r="E111" s="2" t="inlineStr">
@@ -5639,7 +5643,11 @@
           <t>1 = selected</t>
         </is>
       </c>
-      <c r="F111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>top_n_overall is set in profile_short_term.yaml (if left out, top_n_per_category is used).</t>
+        </is>
+      </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
           <t>Screener (calculated)</t>
@@ -5694,70 +5702,82 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>Top K Cutoff (rows needed)</t>
+          <t>Trading Volume</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr"/>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>(Momentum tab) Smallest K such that at least 50 funds are within the best K funds for BOTH 1W and 1M return.</t>
+          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window.</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>K = smallest number with ≥ 50 funds having 1W position ≤ K AND 1M position ≤ K</t>
+          <t>Reported directly from exchange data</t>
         </is>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Higher = easier to trade at a fair price</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>Same value on every row.</t>
+          <t>Not in the current eTrade export. The YAML still gives it weight 0.4 in Liquidity/Size; since the column is missing, Fund Size gets the whole Liquidity/Size weight. Add it to the export to use it.</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Morningstar (not in current data)</t>
         </is>
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I113" s="2" t="inlineStr"/>
-      <c r="J113" s="2" t="inlineStr"/>
-      <c r="K113" s="2" t="inlineStr"/>
+          <t>No effect: weighted 0.4 in the YAML, but the column is missing</t>
+        </is>
+      </c>
+      <c r="I113" s="2" t="inlineStr">
+        <is>
+          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window. Key facts: Unit is shares, not dollars. Single-day volume and average volume are distinct fields; which one an export column holds depends on the data point chosen.</t>
+        </is>
+      </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>Corrected to Morningstar's definition</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr">
+        <is>
+          <t>http://quote.morningstar.com/ETFdefinition.html</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>Top Position</t>
-        </is>
-      </c>
-      <c r="B114" s="2" t="inlineStr">
-        <is>
-          <t>1W, 1M</t>
-        </is>
-      </c>
+          <t>Management Style</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr"/>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>(Momentum tab) Fund's position counted from the best 1-week (1W) or 1-month (1M) return (1 = best).</t>
+          <t>Whether the fund is run by a single manager, a team, or a committee.</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr"/>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>Lower = stronger signal</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr"/>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr">
+        <is>
+          <t>Mentioned in column_glossary.md; not in the current export and not used in scoring.</t>
+        </is>
+      </c>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Morningstar (not in current data)</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
@@ -5765,40 +5785,52 @@
           <t>No</t>
         </is>
       </c>
-      <c r="I114" s="2" t="inlineStr"/>
-      <c r="J114" s="2" t="inlineStr"/>
-      <c r="K114" s="2" t="inlineStr"/>
+      <c r="I114" s="2" t="inlineStr">
+        <is>
+          <t>Not found. The closest Morningstar definitions: 'Management Team' is used when more than two people manage the fund together or the fund strongly promotes a team approach; 'Multiple Managers' is used when people manage portions independently. Key facts: When a fund lists only 'Management Team' without names, Morningstar shows manager tenure as a dash.</t>
+        </is>
+      </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>No Morningstar definition found</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>https://awgmain.morningstar.com/webhelp/glossary_definitions/mutual_fund/Manager_Tenure_(Longest).htm</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>Bottom K Cutoff (rows needed)</t>
+          <t>3Y Return Rank in Category</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr"/>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>(Momentum tab) Smallest K such that at least 50 funds are within the worst K funds for BOTH 1W and 1M return.</t>
+          <t>Morningstar's percentile rank of the fund's 3-year return within its category (1 = best).</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>K = smallest number with ≥ 50 funds having 1W position ≤ K AND 1M position ≤ K</t>
+          <t>Morningstar computes this; lower rank = better</t>
         </is>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>Same value on every row.</t>
+          <t>Used by the old single 'Performance' concept, which has since been split into Long-term and Short-term Return. Not in the current export.</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Morningstar (not in current data)</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
@@ -5806,204 +5838,24 @@
           <t>No</t>
         </is>
       </c>
-      <c r="I115" s="2" t="inlineStr"/>
-      <c r="J115" s="2" t="inlineStr"/>
-      <c r="K115" s="2" t="inlineStr"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>Bottom Position</t>
-        </is>
-      </c>
-      <c r="B116" s="2" t="inlineStr">
-        <is>
-          <t>1W, 1M</t>
-        </is>
-      </c>
-      <c r="C116" s="2" t="inlineStr">
-        <is>
-          <t>(Momentum tab) Fund's position counted from the worst 1-week (1W) or 1-month (1M) return (1 = worst).</t>
-        </is>
-      </c>
-      <c r="D116" s="2" t="inlineStr"/>
-      <c r="E116" s="2" t="inlineStr">
-        <is>
-          <t>Lower = stronger signal</t>
-        </is>
-      </c>
-      <c r="F116" s="2" t="inlineStr"/>
-      <c r="G116" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="H116" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I116" s="2" t="inlineStr"/>
-      <c r="J116" s="2" t="inlineStr"/>
-      <c r="K116" s="2" t="inlineStr"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="2" t="inlineStr">
-        <is>
-          <t>Trading Volume</t>
-        </is>
-      </c>
-      <c r="B117" s="2" t="inlineStr"/>
-      <c r="C117" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window.</t>
-        </is>
-      </c>
-      <c r="D117" s="2" t="inlineStr">
-        <is>
-          <t>Reported directly from exchange data</t>
-        </is>
-      </c>
-      <c r="E117" s="2" t="inlineStr">
-        <is>
-          <t>Higher = easier to trade at a fair price</t>
-        </is>
-      </c>
-      <c r="F117" s="2" t="inlineStr">
-        <is>
-          <t>Not in the current eTrade export. The YAML still gives it weight 0.4 in Liquidity/Size; since the column is missing, Fund Size gets the whole Liquidity/Size weight. Add it to the export to use it.</t>
-        </is>
-      </c>
-      <c r="G117" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar (not in current data)</t>
-        </is>
-      </c>
-      <c r="H117" s="2" t="inlineStr">
-        <is>
-          <t>No effect: weighted 0.4 in the YAML, but the column is missing</t>
-        </is>
-      </c>
-      <c r="I117" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window. Key facts: Unit is shares, not dollars. Single-day volume and average volume are distinct fields; which one an export column holds depends on the data point chosen.</t>
-        </is>
-      </c>
-      <c r="J117" s="2" t="inlineStr">
-        <is>
-          <t>Corrected to Morningstar's definition</t>
-        </is>
-      </c>
-      <c r="K117" s="2" t="inlineStr">
-        <is>
-          <t>http://quote.morningstar.com/ETFdefinition.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
-        <is>
-          <t>Management Style</t>
-        </is>
-      </c>
-      <c r="B118" s="2" t="inlineStr"/>
-      <c r="C118" s="2" t="inlineStr">
-        <is>
-          <t>Whether the fund is run by a single manager, a team, or a committee.</t>
-        </is>
-      </c>
-      <c r="D118" s="2" t="inlineStr"/>
-      <c r="E118" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F118" s="2" t="inlineStr">
-        <is>
-          <t>Mentioned in column_glossary.md; not in the current export and not used in scoring.</t>
-        </is>
-      </c>
-      <c r="G118" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar (not in current data)</t>
-        </is>
-      </c>
-      <c r="H118" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I118" s="2" t="inlineStr">
-        <is>
-          <t>Not found. The closest Morningstar definitions: 'Management Team' is used when more than two people manage the fund together or the fund strongly promotes a team approach; 'Multiple Managers' is used when people manage portions independently. Key facts: When a fund lists only 'Management Team' without names, Morningstar shows manager tenure as a dash.</t>
-        </is>
-      </c>
-      <c r="J118" s="2" t="inlineStr">
-        <is>
-          <t>No Morningstar definition found</t>
-        </is>
-      </c>
-      <c r="K118" s="2" t="inlineStr">
-        <is>
-          <t>https://awgmain.morningstar.com/webhelp/glossary_definitions/mutual_fund/Manager_Tenure_(Longest).htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="2" t="inlineStr">
-        <is>
-          <t>3Y Return Rank in Category</t>
-        </is>
-      </c>
-      <c r="B119" s="2" t="inlineStr"/>
-      <c r="C119" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar's percentile rank of the fund's 3-year return within its category (1 = best).</t>
-        </is>
-      </c>
-      <c r="D119" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar computes this; lower rank = better</t>
-        </is>
-      </c>
-      <c r="E119" s="2" t="inlineStr">
-        <is>
-          <t>Lower is better</t>
-        </is>
-      </c>
-      <c r="F119" s="2" t="inlineStr">
-        <is>
-          <t>Used by the old single 'Performance' concept, which has since been split into Long-term and Short-term Return. Not in the current export.</t>
-        </is>
-      </c>
-      <c r="G119" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar (not in current data)</t>
-        </is>
-      </c>
-      <c r="H119" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I119" s="2" t="inlineStr">
+      <c r="I115" s="2" t="inlineStr">
         <is>
           <t>The fund's 3-year total-return percentile rank among all funds in the same Morningstar Category, on a 1-100 scale where 1 is the best (highest return) and 100 the worst. Key facts: Based on total return, not adjusted for sales loads (Morningstar publishes load-adjusted ranks separately). Only funds with a full 3-year history are ranked. Lower = better for returns.</t>
         </is>
       </c>
-      <c r="J119" s="2" t="inlineStr">
+      <c r="J115" s="2" t="inlineStr">
         <is>
           <t>Matches Morningstar</t>
         </is>
       </c>
-      <c r="K119" s="2" t="inlineStr">
+      <c r="K115" s="2" t="inlineStr">
         <is>
           <t>https://awgmain.morningstar.com/webhelp/glossary_definitions/mutual_fund/mfglossary_PercentileRankCategory.html</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K119"/>
+  <autoFilter ref="A1:K115"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6014,7 +5866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G258"/>
+  <dimension ref="A1:G252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -6071,7 +5923,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -6104,7 +5956,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -6137,7 +5989,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -6170,7 +6022,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -6203,7 +6055,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -6236,7 +6088,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -6269,7 +6121,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -6302,7 +6154,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -6335,7 +6187,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -6368,7 +6220,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -6405,7 +6257,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -6442,7 +6294,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -6479,7 +6331,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -6516,7 +6368,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -6553,7 +6405,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -6590,7 +6442,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -6627,7 +6479,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -6664,7 +6516,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -6701,7 +6553,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -6738,7 +6590,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -6775,7 +6627,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -6812,7 +6664,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -6849,7 +6701,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -6886,7 +6738,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -6923,7 +6775,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -6960,7 +6812,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -6997,7 +6849,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -7034,7 +6886,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -7071,7 +6923,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -7108,7 +6960,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -7145,7 +6997,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -7182,7 +7034,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -7219,7 +7071,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -7256,7 +7108,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -7293,7 +7145,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -7330,7 +7182,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -7367,7 +7219,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -7404,7 +7256,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -7441,7 +7293,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -7478,7 +7330,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -7515,7 +7367,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -7548,7 +7400,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -7581,7 +7433,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -7614,7 +7466,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -7647,7 +7499,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -7680,7 +7532,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -7713,7 +7565,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -7750,7 +7602,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -7787,7 +7639,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -7824,7 +7676,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -7861,7 +7713,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -7898,7 +7750,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -7935,7 +7787,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -7972,7 +7824,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -8009,7 +7861,7 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -8046,7 +7898,7 @@
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -8079,7 +7931,7 @@
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -8116,7 +7968,7 @@
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -8153,7 +8005,7 @@
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -8190,7 +8042,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -8227,7 +8079,7 @@
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -8264,7 +8116,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -8301,7 +8153,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -8338,7 +8190,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -8375,7 +8227,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -8412,7 +8264,7 @@
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -8449,7 +8301,7 @@
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -8486,7 +8338,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -8523,7 +8375,7 @@
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -8560,7 +8412,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -8597,7 +8449,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -8634,7 +8486,7 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -8671,7 +8523,7 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -8708,7 +8560,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -8745,7 +8597,7 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -8782,7 +8634,7 @@
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -8819,7 +8671,7 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -8856,7 +8708,7 @@
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -8893,7 +8745,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -8930,7 +8782,7 @@
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -8967,7 +8819,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -9004,7 +8856,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -9041,7 +8893,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -9078,7 +8930,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -9115,7 +8967,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -9152,7 +9004,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -9189,7 +9041,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr">
@@ -9226,7 +9078,7 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr">
@@ -9263,7 +9115,7 @@
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
@@ -9300,7 +9152,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -9337,7 +9189,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -9374,7 +9226,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -9411,7 +9263,7 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
@@ -9444,7 +9296,7 @@
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
@@ -9477,7 +9329,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
@@ -9510,7 +9362,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr">
@@ -9543,7 +9395,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr">
@@ -9576,7 +9428,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
@@ -9609,7 +9461,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C100" s="2" t="inlineStr">
@@ -9646,7 +9498,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C101" s="2" t="inlineStr">
@@ -9683,7 +9535,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C102" s="2" t="inlineStr">
@@ -9720,7 +9572,7 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
@@ -9757,7 +9609,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C104" s="2" t="inlineStr">
@@ -9794,7 +9646,7 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C105" s="2" t="inlineStr">
@@ -9831,7 +9683,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C106" s="2" t="inlineStr">
@@ -9868,7 +9720,7 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C107" s="2" t="inlineStr">
@@ -9905,7 +9757,7 @@
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C108" s="2" t="inlineStr">
@@ -9942,7 +9794,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
@@ -9975,7 +9827,7 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C110" s="2" t="inlineStr">
@@ -10012,7 +9864,7 @@
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
@@ -10049,7 +9901,7 @@
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C112" s="2" t="inlineStr">
@@ -10086,7 +9938,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C113" s="2" t="inlineStr">
@@ -10123,7 +9975,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C114" s="2" t="inlineStr">
@@ -10160,7 +10012,7 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C115" s="2" t="inlineStr">
@@ -10197,7 +10049,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
@@ -10234,7 +10086,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
@@ -10271,7 +10123,7 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C118" s="2" t="inlineStr">
@@ -10304,7 +10156,7 @@
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C119" s="2" t="inlineStr">
@@ -10337,7 +10189,7 @@
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C120" s="2" t="inlineStr">
@@ -10374,7 +10226,7 @@
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C121" s="2" t="inlineStr">
@@ -10411,7 +10263,7 @@
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C122" s="2" t="inlineStr">
@@ -10448,7 +10300,7 @@
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C123" s="2" t="inlineStr">
@@ -10485,7 +10337,7 @@
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C124" s="2" t="inlineStr">
@@ -10522,7 +10374,7 @@
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C125" s="2" t="inlineStr">
@@ -10559,7 +10411,7 @@
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C126" s="2" t="inlineStr">
@@ -10596,7 +10448,7 @@
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C127" s="2" t="inlineStr">
@@ -10633,7 +10485,7 @@
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C128" s="2" t="inlineStr">
@@ -10670,7 +10522,7 @@
       </c>
       <c r="B129" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C129" s="2" t="inlineStr">
@@ -10707,7 +10559,7 @@
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C130" s="2" t="inlineStr">
@@ -10744,7 +10596,7 @@
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C131" s="2" t="inlineStr">
@@ -10781,7 +10633,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -10818,7 +10670,7 @@
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
@@ -10855,7 +10707,7 @@
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
@@ -10892,7 +10744,7 @@
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C135" s="2" t="inlineStr">
@@ -10929,7 +10781,7 @@
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C136" s="2" t="inlineStr">
@@ -10962,7 +10814,7 @@
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
@@ -10999,7 +10851,7 @@
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C138" s="2" t="inlineStr">
@@ -11036,7 +10888,7 @@
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C139" s="2" t="inlineStr">
@@ -11069,7 +10921,7 @@
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C140" s="2" t="inlineStr">
@@ -11102,7 +10954,7 @@
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C141" s="2" t="inlineStr">
@@ -11135,7 +10987,7 @@
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C142" s="2" t="inlineStr">
@@ -11168,7 +11020,7 @@
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
@@ -11201,7 +11053,7 @@
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C144" s="2" t="inlineStr">
@@ -11238,7 +11090,7 @@
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
@@ -11271,7 +11123,7 @@
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C146" s="2" t="inlineStr">
@@ -11304,7 +11156,7 @@
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C147" s="2" t="inlineStr">
@@ -11337,7 +11189,7 @@
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C148" s="2" t="inlineStr">
@@ -11374,7 +11226,7 @@
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C149" s="2" t="inlineStr">
@@ -11411,7 +11263,7 @@
       </c>
       <c r="B150" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C150" s="2" t="inlineStr">
@@ -11448,7 +11300,7 @@
       </c>
       <c r="B151" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C151" s="2" t="inlineStr">
@@ -11481,7 +11333,7 @@
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C152" s="2" t="inlineStr">
@@ -11514,7 +11366,7 @@
       </c>
       <c r="B153" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C153" s="2" t="inlineStr">
@@ -11547,7 +11399,7 @@
       </c>
       <c r="B154" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C154" s="2" t="inlineStr">
@@ -11580,7 +11432,7 @@
       </c>
       <c r="B155" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C155" s="2" t="inlineStr">
@@ -11613,7 +11465,7 @@
       </c>
       <c r="B156" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C156" s="2" t="inlineStr">
@@ -11646,7 +11498,7 @@
       </c>
       <c r="B157" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C157" s="2" t="inlineStr">
@@ -11679,7 +11531,7 @@
       </c>
       <c r="B158" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C158" s="2" t="inlineStr">
@@ -11716,7 +11568,7 @@
       </c>
       <c r="B159" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C159" s="2" t="inlineStr">
@@ -11753,7 +11605,7 @@
       </c>
       <c r="B160" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C160" s="2" t="inlineStr">
@@ -11790,7 +11642,7 @@
       </c>
       <c r="B161" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C161" s="2" t="inlineStr">
@@ -11827,7 +11679,7 @@
       </c>
       <c r="B162" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C162" s="2" t="inlineStr">
@@ -11860,7 +11712,7 @@
       </c>
       <c r="B163" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C163" s="2" t="inlineStr">
@@ -11897,7 +11749,7 @@
       </c>
       <c r="B164" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C164" s="2" t="inlineStr">
@@ -11934,7 +11786,7 @@
       </c>
       <c r="B165" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C165" s="2" t="inlineStr">
@@ -11971,7 +11823,7 @@
       </c>
       <c r="B166" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C166" s="2" t="inlineStr">
@@ -12008,7 +11860,7 @@
       </c>
       <c r="B167" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C167" s="2" t="inlineStr">
@@ -12045,7 +11897,7 @@
       </c>
       <c r="B168" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C168" s="2" t="inlineStr">
@@ -12082,7 +11934,7 @@
       </c>
       <c r="B169" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C169" s="2" t="inlineStr">
@@ -12119,7 +11971,7 @@
       </c>
       <c r="B170" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C170" s="2" t="inlineStr">
@@ -12156,7 +12008,7 @@
       </c>
       <c r="B171" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C171" s="2" t="inlineStr">
@@ -12193,7 +12045,7 @@
       </c>
       <c r="B172" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C172" s="2" t="inlineStr">
@@ -12230,7 +12082,7 @@
       </c>
       <c r="B173" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C173" s="2" t="inlineStr">
@@ -12267,7 +12119,7 @@
       </c>
       <c r="B174" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C174" s="2" t="inlineStr">
@@ -12304,7 +12156,7 @@
       </c>
       <c r="B175" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C175" s="2" t="inlineStr">
@@ -12341,7 +12193,7 @@
       </c>
       <c r="B176" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C176" s="2" t="inlineStr">
@@ -12378,7 +12230,7 @@
       </c>
       <c r="B177" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C177" s="2" t="inlineStr">
@@ -12415,7 +12267,7 @@
       </c>
       <c r="B178" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C178" s="2" t="inlineStr">
@@ -12452,7 +12304,7 @@
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
@@ -12489,7 +12341,7 @@
       </c>
       <c r="B180" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C180" s="2" t="inlineStr">
@@ -12522,7 +12374,7 @@
       </c>
       <c r="B181" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C181" s="2" t="inlineStr">
@@ -12555,7 +12407,7 @@
       </c>
       <c r="B182" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C182" s="2" t="inlineStr">
@@ -12588,7 +12440,7 @@
       </c>
       <c r="B183" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C183" s="2" t="inlineStr">
@@ -12625,7 +12477,7 @@
       </c>
       <c r="B184" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C184" s="2" t="inlineStr">
@@ -12662,7 +12514,7 @@
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
@@ -12699,7 +12551,7 @@
       </c>
       <c r="B186" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C186" s="2" t="inlineStr">
@@ -12736,7 +12588,7 @@
       </c>
       <c r="B187" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C187" s="2" t="inlineStr">
@@ -12769,7 +12621,7 @@
       </c>
       <c r="B188" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C188" s="2" t="inlineStr">
@@ -12802,7 +12654,7 @@
       </c>
       <c r="B189" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C189" s="2" t="inlineStr">
@@ -12835,7 +12687,7 @@
       </c>
       <c r="B190" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C190" s="2" t="inlineStr">
@@ -12868,7 +12720,7 @@
       </c>
       <c r="B191" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C191" s="2" t="inlineStr">
@@ -12901,7 +12753,7 @@
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
@@ -12934,7 +12786,7 @@
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
@@ -12967,7 +12819,7 @@
       </c>
       <c r="B194" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C194" s="2" t="inlineStr">
@@ -13000,7 +12852,7 @@
       </c>
       <c r="B195" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C195" s="2" t="inlineStr">
@@ -13033,7 +12885,7 @@
       </c>
       <c r="B196" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C196" s="2" t="inlineStr">
@@ -13066,7 +12918,7 @@
       </c>
       <c r="B197" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C197" s="2" t="inlineStr">
@@ -13099,7 +12951,7 @@
       </c>
       <c r="B198" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C198" s="2" t="inlineStr">
@@ -13132,7 +12984,7 @@
       </c>
       <c r="B199" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C199" s="2" t="inlineStr">
@@ -13165,7 +13017,7 @@
       </c>
       <c r="B200" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C200" s="2" t="inlineStr">
@@ -13198,7 +13050,7 @@
       </c>
       <c r="B201" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C201" s="2" t="inlineStr">
@@ -13231,7 +13083,7 @@
       </c>
       <c r="B202" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C202" s="2" t="inlineStr">
@@ -13264,7 +13116,7 @@
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C203" s="2" t="inlineStr">
@@ -13297,7 +13149,7 @@
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C204" s="2" t="inlineStr">
@@ -13330,7 +13182,7 @@
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr">
@@ -13363,7 +13215,7 @@
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
@@ -13400,7 +13252,7 @@
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C207" s="2" t="inlineStr">
@@ -13437,7 +13289,7 @@
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
@@ -13474,7 +13326,7 @@
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C209" s="2" t="inlineStr">
@@ -13511,7 +13363,7 @@
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C210" s="2" t="inlineStr">
@@ -13544,7 +13396,7 @@
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C211" s="2" t="inlineStr">
@@ -13577,7 +13429,7 @@
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C212" s="2" t="inlineStr">
@@ -13610,7 +13462,7 @@
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C213" s="2" t="inlineStr">
@@ -13643,7 +13495,7 @@
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C214" s="2" t="inlineStr">
@@ -13676,7 +13528,7 @@
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C215" s="2" t="inlineStr">
@@ -13709,7 +13561,7 @@
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C216" s="2" t="inlineStr">
@@ -13742,7 +13594,7 @@
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C217" s="2" t="inlineStr">
@@ -13775,7 +13627,7 @@
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C218" s="2" t="inlineStr">
@@ -13808,7 +13660,7 @@
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C219" s="2" t="inlineStr">
@@ -13841,7 +13693,7 @@
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C220" s="2" t="inlineStr">
@@ -13874,7 +13726,7 @@
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C221" s="2" t="inlineStr">
@@ -13907,7 +13759,7 @@
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C222" s="2" t="inlineStr">
@@ -13944,7 +13796,7 @@
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C223" s="2" t="inlineStr">
@@ -13981,7 +13833,7 @@
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C224" s="2" t="inlineStr">
@@ -14018,7 +13870,7 @@
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C225" s="2" t="inlineStr">
@@ -14055,7 +13907,7 @@
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C226" s="2" t="inlineStr">
@@ -14092,7 +13944,7 @@
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C227" s="2" t="inlineStr">
@@ -14129,7 +13981,7 @@
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C228" s="2" t="inlineStr">
@@ -14166,7 +14018,7 @@
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C229" s="2" t="inlineStr">
@@ -14203,7 +14055,7 @@
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C230" s="2" t="inlineStr">
@@ -14240,7 +14092,7 @@
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C231" s="2" t="inlineStr">
@@ -14277,7 +14129,7 @@
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C232" s="2" t="inlineStr">
@@ -14314,7 +14166,7 @@
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C233" s="2" t="inlineStr">
@@ -14351,7 +14203,7 @@
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C234" s="2" t="inlineStr">
@@ -14388,7 +14240,7 @@
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C235" s="2" t="inlineStr">
@@ -14425,7 +14277,7 @@
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C236" s="2" t="inlineStr">
@@ -14462,7 +14314,7 @@
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C237" s="2" t="inlineStr">
@@ -14499,7 +14351,7 @@
       </c>
       <c r="B238" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C238" s="2" t="inlineStr">
@@ -14536,7 +14388,7 @@
       </c>
       <c r="B239" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C239" s="2" t="inlineStr">
@@ -14573,7 +14425,7 @@
       </c>
       <c r="B240" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C240" s="2" t="inlineStr">
@@ -14610,7 +14462,7 @@
       </c>
       <c r="B241" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C241" s="2" t="inlineStr">
@@ -14647,7 +14499,7 @@
       </c>
       <c r="B242" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C242" s="2" t="inlineStr">
@@ -14680,7 +14532,7 @@
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
@@ -14713,7 +14565,7 @@
       </c>
       <c r="B244" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C244" s="2" t="inlineStr">
@@ -14746,7 +14598,7 @@
       </c>
       <c r="B245" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C245" s="2" t="inlineStr">
@@ -14779,7 +14631,7 @@
       </c>
       <c r="B246" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C246" s="2" t="inlineStr">
@@ -14812,7 +14664,7 @@
       </c>
       <c r="B247" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C247" s="2" t="inlineStr">
@@ -14845,7 +14697,7 @@
       </c>
       <c r="B248" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C248" s="2" t="inlineStr">
@@ -14878,7 +14730,7 @@
       </c>
       <c r="B249" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C249" s="2" t="inlineStr">
@@ -14911,7 +14763,7 @@
       </c>
       <c r="B250" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C250" s="2" t="inlineStr">
@@ -14944,7 +14796,7 @@
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>Overview (also on the extra tabs)</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
@@ -15002,222 +14854,8 @@
         </is>
       </c>
     </row>
-    <row r="253">
-      <c r="A253" s="2" t="inlineStr">
-        <is>
-          <t>Top K Cutoff (rows needed)</t>
-        </is>
-      </c>
-      <c r="B253" s="2" t="inlineStr">
-        <is>
-          <t>Top 50 / Bottom 50 momentum</t>
-        </is>
-      </c>
-      <c r="C253" s="2" t="inlineStr">
-        <is>
-          <t>Top K Cutoff (rows needed)</t>
-        </is>
-      </c>
-      <c r="D253" s="2" t="inlineStr"/>
-      <c r="E253" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F253" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G253" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" s="2" t="inlineStr">
-        <is>
-          <t>Top Position 1W</t>
-        </is>
-      </c>
-      <c r="B254" s="2" t="inlineStr">
-        <is>
-          <t>Top 50 / Bottom 50 momentum</t>
-        </is>
-      </c>
-      <c r="C254" s="2" t="inlineStr">
-        <is>
-          <t>Top Position</t>
-        </is>
-      </c>
-      <c r="D254" s="2" t="inlineStr">
-        <is>
-          <t>1W</t>
-        </is>
-      </c>
-      <c r="E254" s="2" t="inlineStr">
-        <is>
-          <t>Lower = stronger signal</t>
-        </is>
-      </c>
-      <c r="F254" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G254" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" s="2" t="inlineStr">
-        <is>
-          <t>Top Position 1M</t>
-        </is>
-      </c>
-      <c r="B255" s="2" t="inlineStr">
-        <is>
-          <t>Top 50 / Bottom 50 momentum</t>
-        </is>
-      </c>
-      <c r="C255" s="2" t="inlineStr">
-        <is>
-          <t>Top Position</t>
-        </is>
-      </c>
-      <c r="D255" s="2" t="inlineStr">
-        <is>
-          <t>1M</t>
-        </is>
-      </c>
-      <c r="E255" s="2" t="inlineStr">
-        <is>
-          <t>Lower = stronger signal</t>
-        </is>
-      </c>
-      <c r="F255" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G255" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" s="2" t="inlineStr">
-        <is>
-          <t>Bottom K Cutoff (rows needed)</t>
-        </is>
-      </c>
-      <c r="B256" s="2" t="inlineStr">
-        <is>
-          <t>Top 50 / Bottom 50 momentum</t>
-        </is>
-      </c>
-      <c r="C256" s="2" t="inlineStr">
-        <is>
-          <t>Bottom K Cutoff (rows needed)</t>
-        </is>
-      </c>
-      <c r="D256" s="2" t="inlineStr"/>
-      <c r="E256" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F256" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G256" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" s="2" t="inlineStr">
-        <is>
-          <t>Bottom Position 1W</t>
-        </is>
-      </c>
-      <c r="B257" s="2" t="inlineStr">
-        <is>
-          <t>Top 50 / Bottom 50 momentum</t>
-        </is>
-      </c>
-      <c r="C257" s="2" t="inlineStr">
-        <is>
-          <t>Bottom Position</t>
-        </is>
-      </c>
-      <c r="D257" s="2" t="inlineStr">
-        <is>
-          <t>1W</t>
-        </is>
-      </c>
-      <c r="E257" s="2" t="inlineStr">
-        <is>
-          <t>Lower = stronger signal</t>
-        </is>
-      </c>
-      <c r="F257" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G257" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" s="2" t="inlineStr">
-        <is>
-          <t>Bottom Position 1M</t>
-        </is>
-      </c>
-      <c r="B258" s="2" t="inlineStr">
-        <is>
-          <t>Top 50 / Bottom 50 momentum</t>
-        </is>
-      </c>
-      <c r="C258" s="2" t="inlineStr">
-        <is>
-          <t>Bottom Position</t>
-        </is>
-      </c>
-      <c r="D258" s="2" t="inlineStr">
-        <is>
-          <t>1M</t>
-        </is>
-      </c>
-      <c r="E258" s="2" t="inlineStr">
-        <is>
-          <t>Lower = stronger signal</t>
-        </is>
-      </c>
-      <c r="F258" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G258" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G258"/>
+  <autoFilter ref="A1:G252"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Remove outdated Profile A design doc and column glossary
- report_column_dictionary.xlsx already covers the glossary's definitions,
  formulas and sector-distortion tables; its sector-mix explanation and
  practical takeaway are now notes on the Scoring Concepts tab
- Drop the dictionary rows for Management Style and 3Y Return Rank in
  Category (only listed because the glossary mentioned them)
- Update references in README, scoring.py and the config.py header

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_screener/docs/report_column_dictionary.xlsx
+++ b/etf_screener/docs/report_column_dictionary.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volatile Periods" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$252</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scoring Concepts'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volatile Periods'!$A$1:$H$25</definedName>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K115"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5752,110 +5752,8 @@
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="2" t="inlineStr">
-        <is>
-          <t>Management Style</t>
-        </is>
-      </c>
-      <c r="B114" s="2" t="inlineStr"/>
-      <c r="C114" s="2" t="inlineStr">
-        <is>
-          <t>Whether the fund is run by a single manager, a team, or a committee.</t>
-        </is>
-      </c>
-      <c r="D114" s="2" t="inlineStr"/>
-      <c r="E114" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>Mentioned in column_glossary.md; not in the current export and not used in scoring.</t>
-        </is>
-      </c>
-      <c r="G114" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar (not in current data)</t>
-        </is>
-      </c>
-      <c r="H114" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I114" s="2" t="inlineStr">
-        <is>
-          <t>Not found. The closest Morningstar definitions: 'Management Team' is used when more than two people manage the fund together or the fund strongly promotes a team approach; 'Multiple Managers' is used when people manage portions independently. Key facts: When a fund lists only 'Management Team' without names, Morningstar shows manager tenure as a dash.</t>
-        </is>
-      </c>
-      <c r="J114" s="2" t="inlineStr">
-        <is>
-          <t>No Morningstar definition found</t>
-        </is>
-      </c>
-      <c r="K114" s="2" t="inlineStr">
-        <is>
-          <t>https://awgmain.morningstar.com/webhelp/glossary_definitions/mutual_fund/Manager_Tenure_(Longest).htm</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>3Y Return Rank in Category</t>
-        </is>
-      </c>
-      <c r="B115" s="2" t="inlineStr"/>
-      <c r="C115" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar's percentile rank of the fund's 3-year return within its category (1 = best).</t>
-        </is>
-      </c>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar computes this; lower rank = better</t>
-        </is>
-      </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>Lower is better</t>
-        </is>
-      </c>
-      <c r="F115" s="2" t="inlineStr">
-        <is>
-          <t>Used by the old single 'Performance' concept, which has since been split into Long-term and Short-term Return. Not in the current export.</t>
-        </is>
-      </c>
-      <c r="G115" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar (not in current data)</t>
-        </is>
-      </c>
-      <c r="H115" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I115" s="2" t="inlineStr">
-        <is>
-          <t>The fund's 3-year total-return percentile rank among all funds in the same Morningstar Category, on a 1-100 scale where 1 is the best (highest return) and 100 the worst. Key facts: Based on total return, not adjusted for sales loads (Morningstar publishes load-adjusted ranks separately). Only funds with a full 3-year history are ranked. Lower = better for returns.</t>
-        </is>
-      </c>
-      <c r="J115" s="2" t="inlineStr">
-        <is>
-          <t>Matches Morningstar</t>
-        </is>
-      </c>
-      <c r="K115" s="2" t="inlineStr">
-        <is>
-          <t>https://awgmain.morningstar.com/webhelp/glossary_definitions/mutual_fund/mfglossary_PercentileRankCategory.html</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:K115"/>
+  <autoFilter ref="A1:K113"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14866,7 +14764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -15265,8 +15163,26 @@
         </is>
       </c>
     </row>
+    <row r="13" ht="75" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Why sector mix matters: every score is ranked WITHIN Morningstar Category, but categories are coarse. Morningstar's 'Technology' bundles software (operating systems, applications) with hardware, storage, networking and semiconductors. Two funds in the same category can be semiconductor-heavy (cyclical, capital-intensive) or software-heavy (higher margins, recurring revenue) and still be ranked as direct peers on every score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="75" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Practical takeaway: before trusting a ranking or tuning the Volatility, Quality/Valuation or Return weights in a sector-heavy category like Technology, check the Yahoo Subsector column (or the fund's factsheet holdings) of the top funds. Costs and Liquidity/Size are the least affected; Volatility and Quality/Valuation the most.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G11"/>
+  <mergeCells count="2">
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:G14"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Move sector notes into the column dictionary; add zscore_matrix query
- New Sectors tab: the 11 sectors with their character and sub-sectors
- Z Score row explains reading 1Y and 3Y together (Core / Momentum / Value dip)
- New saved query zscore_matrix lists the funds in each of those groups
- Remove "Financial Sectors and Niche Sub-Sectors.rtf", now covered above

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_screener/docs/report_column_dictionary.xlsx
+++ b/etf_screener/docs/report_column_dictionary.xlsx
@@ -11,12 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Report Columns" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring Concepts" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volatile Periods" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sectors" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$113</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$252</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scoring Concepts'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volatile Periods'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sectors'!$A$1:$D$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -4718,7 +4720,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Peer group = Yahoo Subsector (not Morningstar Category), so a bond fund labelled 'Broad Market Equity' is compared with stock funds.</t>
+          <t>Peer group = Yahoo Subsector (not Morningstar Category), so a bond fund labelled 'Broad Market Equity' is compared with stock funds. Read 1Y and 3Y together: both &gt;= +1 = Core (long-term leader still leading); 1Y &gt;= +1 but 3Y &lt; 0 = Momentum (recent surge, tactical trade, not an anchor); 1Y &lt; 0 but 3Y &gt;= +1 = Value (strong record in a temporary slump, possible buy-the-dip). List them with: python db_access/query.py zscore_matrix</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -16068,4 +16070,289 @@
   <autoFilter ref="A1:H25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Sector</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Character</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Behaviour</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Sub-sectors (example tickers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Growth anchor</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Highest internal dispersion; separating sub-sectors matters most here.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Semiconductors &amp; Equipment (NVDA, AMD, TSM); Software &amp; Services (MSFT, ORCL, CRM); Hardware, Storage &amp; Peripherals (AAPL, HPQ); IT Services &amp; Consulting (ACN, INFY)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Defensive growth</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Defensive stability mixed with volatile, speculative biotech research.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Pharmaceuticals (LLY, JNJ, PFE); Biotechnology (AMGN, VRTX); Equipment &amp; Supplies (MDT, ABT); Providers &amp; Services (UNH, ELV)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Financials</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Interest-rate cyclical</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Sensitive to central-bank rates, credit expansion and the yield curve.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Banks (JPM, BAC, WFC); Financial Services / Capital Markets (V, MA, MS, GS); Insurance (BRK.B, PGR, MET)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Modern media</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Classic telecom combined with digital advertising and entertainment.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Interactive Media (GOOGL, META); Entertainment &amp; Streaming (NFLX, DIS); Telecom Services (T, VZ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Economic pulse</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Relies on disposable income: thrives in expansions, contracts sharply in recessions.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Automobiles (TSLA, F, GM); Broadline Retail &amp; E-Commerce (AMZN); Hotels, Restaurants &amp; Leisure (MCD, SBUX, BKNG); Durables &amp; Apparel (NKE, HD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Recession guard</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Essentials bought in any economy: low volatility, steady dividends.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Beverages &amp; Tobacco (KO, PEP, PM); Food &amp; Staples Retailing (WMT, COST); Household &amp; Personal Products (PG, CL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Commodity cycle</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Tied to oil and gas prices and alternative power.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Oil, Gas &amp; Fuels (XOM, CVX); Equipment &amp; Services (SLB, HAL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Capital expenditure</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Machinery, manufacturing, construction and logistics.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Aerospace &amp; Defense (LMT, RTX); Transportation &amp; Logistics (UPS, FDX, UNP); Machinery &amp; Electrical Equipment (CAT, GE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Materials</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Raw base</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Front of the supply chain: turns raw elements into materials for manufacturers.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Chemicals (LIN, DD); Metals &amp; Mining (FCX, NUE, NEM); Containers &amp; Packaging (IP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Utilities</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Regulated income bond</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Heavily regulated and debt-financed, so they trade like a bond proxy.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Electric, Gas &amp; Water (NEE, DUK, SO); Independent Power &amp; Renewables (CEG)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Hard-asset yield</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Owners and managers of income-producing property.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Equity REITs (PLD, AMT, O); Management &amp; Development (CBRE)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Read filter settings from the YAMLs in the column dictionary; remove unused settings
- Column dictionary: every filter value (expense ratio, loads, minimum
  investment, exclusions, require_*) and the Trading Volume weight now come
  from the profile YAMLs, showing LT and ST values when they differ
- Remove min_3y_return and min_fund_size: listed in the YAMLs and config.py
  but never applied; fix the require_fund_size / expense ratio comments
- query.py: pasted saved-query SQL gets its {name=default} values filled in;
  clearer message for a required value

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_screener/docs/report_column_dictionary.xlsx
+++ b/etf_screener/docs/report_column_dictionary.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Every score and in-category rank compares a fund ONLY with funds in the same category. 132 categories in this report (a few appear twice under ETF vs mutual-fund naming, e.g. 'Mid-Cap Blend' / 'Mid Blend'). Sector caveat: categories are coarse - e.g. 'Technology' mixes semiconductor-heavy and software-heavy funds, which behave very differently; see the Yahoo Subsector column and the 'Scoring Concepts' tab.</t>
+          <t>Filter require_category = OFF (ON = drop funds with no category). Every score and in-category rank compares a fund ONLY with funds in the same category. 132 categories in this report (a few appear twice under ETF vs mutual-fund naming, e.g. 'Mid-Cap Blend' / 'Mid Blend'). Sector caveat: categories are coarse - e.g. 'Technology' mixes semiconductor-heavy and software-heavy funds, which behave very differently; see the Yahoo Subsector column and the 'Scoring Concepts' tab.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Compare within category - a 5% year is great for a bond fund and poor for a tech fund. Blank when the fund is younger than the period. Sector caveat: multi-year returns are strongly driven by sub-sector timing (e.g. AI semiconductors vs software), which within-category ranking does not correct for. 'Since Inception' is not comparable across funds with different start dates.</t>
+          <t>Compare within category - a 5% year is great for a bond fund and poor for a tech fund. Blank when the fund is younger than the period. Sector caveat: multi-year returns are strongly driven by sub-sector timing (e.g. AI semiconductors vs software), which within-category ranking does not correct for. 'Since Inception' is not comparable across funds with different start dates. Filter require_3y_return = LT ON, ST OFF (ON = drop funds with a blank 3Y return, i.e. under 3 years old).</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Waivers can expire. Index ETFs are often &lt; 0.10%, active funds 0.5-1%. The report is filtered to &lt;= 1.75% (max_expense_ratio). Sector-neutral: driven by passive vs active, not holdings.</t>
+          <t>Waivers can expire. Index ETFs are often &lt; 0.10%, active funds 0.5-1%. Filter max_expense_ratio = LT 1.25%, ST 1.75%: funds above it are dropped (a blank ratio is kept). Sector-neutral: driven by passive vs active, not holdings.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Popularity / age driven; little sector link. 'Trading Volume' (YAML weight 0.4) is not in the data, so Fund Size is effectively the whole Liquidity/Size score.</t>
+          <t>Popularity / age driven; little sector link. 'Trading Volume' (YAML weight 0.4) is not in the data, so Fund Size is effectively the whole Liquidity/Size score. Filter require_fund_size = OFF (ON = drop funds with a blank Fund Size).</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Leveraged funds reset daily and lose value in choppy markets ('volatility decay'). Filter exclude_leveraged_funds is currently OFF in the YAML.</t>
+          <t>Leveraged funds reset daily and lose value in choppy markets ('volatility decay'). Filter exclude_leveraged_funds = LT OFF, ST ON (ON = these funds are dropped).</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Filter exclude_interval_funds is currently OFF.</t>
+          <t>Filter exclude_interval_funds = OFF (ON = these funds are dropped).</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>Filter exclude_tender_offer_funds is currently OFF.</t>
+          <t>Filter exclude_tender_offer_funds = OFF (ON = these funds are dropped).</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Hard filter max_deferred_load = 0: funds above it are removed before scoring, so the column is empty in the report.</t>
+          <t>Hard filter max_deferred_load = 0%: funds above it are removed before scoring.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4253,7 +4253,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Hard filter max_front_load = 0 (removed before scoring).</t>
+          <t>Hard filter max_front_load = 0%: funds above it are removed before scoring.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -4302,7 +4302,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Hard filter min_initial_investment = 50,000: funds above it are removed. Blank = no minimum reported (ETFs: one share). Brokers may waive minimums.</t>
+          <t>Hard filter min_initial_investment = $50,000: funds whose minimum is above it are removed. Blank = no minimum reported (ETFs: one share). Brokers may waive minimums.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4351,7 +4351,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Hard filter max_redemption_fee = 0 (removed before scoring).</t>
+          <t>Hard filter max_redemption_fee = 0%: funds above it are removed before scoring.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Profile YAMLs are the only source of profile settings; discover profiles automatically
- Every enabled input_files/profile_*.yaml is a profile (enabled: false skips
  one); run_ci.py, main.py, alerts.py and the column dictionary find them, so a
  new profile needs only a copied YAML with a new `profile:` key
- Remove the per-profile defaults from config.py (thresholds, weights, concept
  weights, top_n, paths, profile list); the YAML must have every key, and a
  missing or unknown key stops the run naming the file and key
- weighted_profile registers any profile key on demand (no PROFILE_KEYS list);
  report headers keep each profile key's spelling (Profile INC Score)
- Yahoo download defaults live only in YahooMetricsConfig; unknown
  yahoo_metrics keys are an error
- Both YAMLs list min_benchmark_beat_pct; drop SEC 7-Day Yield (keep 30-Day)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_screener/docs/report_column_dictionary.xlsx
+++ b/etf_screener/docs/report_column_dictionary.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sectors" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$113</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$252</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$251</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scoring Concepts'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volatile Periods'!$A$1:$H$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sectors'!$A$1:$D$12</definedName>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -3689,18 +3689,22 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>SEC 7-Day Yield</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr"/>
+          <t>Dividend per Share</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Trailing Annual, Forward Annual, 1Y Avg, 3Y Avg</t>
+        </is>
+      </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>The standardized yield used for money market funds, reflecting the fund's income over the most recent seven days, annualized. Morningstar notes it reflects a money fund's current earnings more closely than total return.</t>
+          <t>Dollar dividends per share. Trailing Annual = dividends actually paid over the past 12 months. Forward Annual = the latest declared dividend per share multiplied by how many times a year it is paid (an annualized run rate, not an analyst forecast).</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Morningstar's glossary gives no full formula. Under the SEC money-market method (from fund filings, not Morningstar): base-period return = net change in value of one share over the 7 days, excluding capital changes, divided by starting value; annualized by multiplying by 365/7 (simple). An 'effective' version compounds it.</t>
+          <t>Trailing Annual DPS = sum of dividends per share paid over trailing 12 months. Forward Annual DPS = latest declared dividend per share x payment frequency per year.</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3710,7 +3714,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>Money market funds only.</t>
+          <t>Depends on the share price - compare yields rather than dollars across funds. Forward / 1Y Avg / 3Y Avg are empty in the current export.</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -3720,12 +3724,12 @@
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - Tax/Income has 0 weight in Profile LT (inputs: Trailing Annual: YAML weight 0.1 = 14% of Tax/Income (≈0.0% of Profile LT))</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>The standardized yield used for money market funds, reflecting the fund's income over the most recent seven days, annualized. Morningstar notes it reflects a money fund's current earnings more closely than total return. Key facts: Applies to money market funds only. Reflects income net of expenses, excludes realized/unrealized gains. Changes daily.</t>
+          <t>Dollar dividends per share. Trailing Annual = dividends actually paid over the past 12 months. Forward Annual = the latest declared dividend per share multiplied by how many times a year it is paid (an annualized run rate, not an analyst forecast). Key facts: Forward figure is a mechanical annualization of the most recent (or latest announced) regular payment. Morningstar definitions for the 1Y Avg / 3Y Avg variants were not found.</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
@@ -3735,39 +3739,31 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>https://www.morningstar.com/investing-terms/sec-7-day-yield</t>
+          <t>https://www.morningstar.com/investing-terms/dividend-per-share-forward-annual</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>Dividend per Share</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Trailing Annual, Forward Annual, 1Y Avg, 3Y Avg</t>
-        </is>
-      </c>
+          <t>Leveraged Fund</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr"/>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Dollar dividends per share. Trailing Annual = dividends actually paid over the past 12 months. Forward Annual = the latest declared dividend per share multiplied by how many times a year it is paid (an annualized run rate, not an analyst forecast).</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Trailing Annual DPS = sum of dividends per share paid over trailing 12 months. Forward Annual DPS = latest declared dividend per share x payment frequency per year.</t>
-        </is>
-      </c>
+          <t>A fund that uses leverage to increase its market exposure, typically by borrowing (issuing debt), issuing preferred shares, or using derivatives. For closed-end funds the flag is set if the fund's leverage percentage is above zero.</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr"/>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Higher = more income</t>
+          <t>No for long-term holding</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Depends on the share price - compare yields rather than dollars across funds. Forward / 1Y Avg / 3Y Avg are empty in the current export.</t>
+          <t>Leveraged funds reset daily and lose value in choppy markets ('volatility decay'). Filter exclude_leveraged_funds = LT OFF, ST ON (ON = these funds are dropped).</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -3777,12 +3773,12 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>No - Tax/Income has 0 weight in Profile LT (inputs: Trailing Annual: YAML weight 0.1 = 14% of Tax/Income (≈0.0% of Profile LT))</t>
+          <t>No (optional filter)</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>Dollar dividends per share. Trailing Annual = dividends actually paid over the past 12 months. Forward Annual = the latest declared dividend per share multiplied by how many times a year it is paid (an annualized run rate, not an analyst forecast). Key facts: Forward figure is a mechanical annualization of the most recent (or latest announced) regular payment. Morningstar definitions for the 1Y Avg / 3Y Avg variants were not found.</t>
+          <t>A fund that uses leverage to increase its market exposure, typically by borrowing (issuing debt), issuing preferred shares, or using derivatives. For closed-end funds the flag is set if the fund's leverage percentage is above zero. Key facts: Covers closed-end funds that borrow or issue preferred shares, not just daily-reset 2x/3x/inverse ETFs. A closed-end fund is flagged if leverage % &gt; 0.</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
@@ -3792,31 +3788,31 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>https://www.morningstar.com/investing-terms/dividend-per-share-forward-annual</t>
+          <t>https://www.morningstar.com/investing-terms/leveraged-fund</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Leveraged Fund</t>
+          <t>Interval Fund</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr"/>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>A fund that uses leverage to increase its market exposure, typically by borrowing (issuing debt), issuing preferred shares, or using derivatives. For closed-end funds the flag is set if the fund's leverage percentage is above zero.</t>
+          <t>Yes if the fund only lets you sell at scheduled intervals (e.g. quarterly).</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr"/>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>No for long-term holding</t>
+          <t>No (more liquid)</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Leveraged funds reset daily and lose value in choppy markets ('volatility decay'). Filter exclude_leveraged_funds = LT OFF, ST ON (ON = these funds are dropped).</t>
+          <t>Filter exclude_interval_funds = OFF (ON = these funds are dropped).</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -3831,41 +3827,41 @@
       </c>
       <c r="I68" s="2" t="inlineStr">
         <is>
-          <t>A fund that uses leverage to increase its market exposure, typically by borrowing (issuing debt), issuing preferred shares, or using derivatives. For closed-end funds the flag is set if the fund's leverage percentage is above zero. Key facts: Covers closed-end funds that borrow or issue preferred shares, not just daily-reset 2x/3x/inverse ETFs. A closed-end fund is flagged if leverage % &gt; 0.</t>
+          <t>A semiliquid fund with set repurchase windows: it is not traded on an exchange, and shareholders can only sell shares back to the fund during scheduled periodic repurchase offers (most often quarterly). Key facts: Under SEC Rule 23c-3, repurchase offers happen at least once a year and cover 5%-25% of outstanding shares, at NAV; if requests exceed the offer, shares are bought pro rata, so you may not get out fully. Usually invests in illiquid assets (private credit, real estate).</t>
         </is>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
-          <t>Corrected to Morningstar's definition</t>
+          <t>Matches Morningstar</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>https://www.morningstar.com/investing-terms/leveraged-fund</t>
+          <t>https://www.morningstar.com/alternative-investments/closer-look-semiliquid-funds</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>Interval Fund</t>
+          <t>Fund of Funds</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr"/>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Yes if the fund only lets you sell at scheduled intervals (e.g. quarterly).</t>
+          <t>Yes if the fund invests in other funds (e.g. target-date funds).</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr"/>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>No (more liquid)</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>Filter exclude_interval_funds = OFF (ON = these funds are dropped).</t>
+          <t>Check the total cost including the underlying funds' fees.</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -3875,12 +3871,12 @@
       </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I69" s="2" t="inlineStr">
         <is>
-          <t>A semiliquid fund with set repurchase windows: it is not traded on an exchange, and shareholders can only sell shares back to the fund during scheduled periodic repurchase offers (most often quarterly). Key facts: Under SEC Rule 23c-3, repurchase offers happen at least once a year and cover 5%-25% of outstanding shares, at NAV; if requests exceed the offer, shares are bought pro rata, so you may not get out fully. Usually invests in illiquid assets (private credit, real estate).</t>
+          <t>A fund that invests substantially all of its assets in other pooled vehicles, such as other mutual funds or ETFs, rather than buying individual stocks and bonds directly. Key facts: Target-date and many allocation funds are typical examples.</t>
         </is>
       </c>
       <c r="J69" s="2" t="inlineStr">
@@ -3890,31 +3886,31 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>https://www.morningstar.com/alternative-investments/closer-look-semiliquid-funds</t>
+          <t>https://www.morningstar.com/investing-terms/fund-of-funds</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>Fund of Funds</t>
+          <t>Investment Status</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr"/>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Yes if the fund invests in other funds (e.g. target-date funds).</t>
+          <t>Open, Limited (closed to most new investors) or Closed.</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr"/>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Check the total cost including the underlying funds' fees.</t>
+          <t>You may not be able to buy a Closed / Limited fund.</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -3929,7 +3925,7 @@
       </c>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>A fund that invests substantially all of its assets in other pooled vehicles, such as other mutual funds or ETFs, rather than buying individual stocks and bonds directly. Key facts: Target-date and many allocation funds are typical examples.</t>
+          <t>Whether the fund is accepting money. 'Limited' is how Morningstar displays a fund that is closed to new investors (temporarily or permanently) while existing shareholders may still add to their holdings; 'Closed' means not accepting new purchases; 'Open' means open to all. Key facts: Limited = closed to new investors only; existing shareholders are not restricted from adding money.</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr">
@@ -3939,31 +3935,31 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>https://www.morningstar.com/investing-terms/fund-of-funds</t>
+          <t>https://gladmainnew.morningstar.com/directhelp/Glossary/Operations/Fund/Closed_to_New_Investors.htm</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>Investment Status</t>
+          <t>Strategic Beta Group</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr"/>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Open, Limited (closed to most new investors) or Closed.</t>
+          <t>For 'smart beta' index funds: the factor they tilt to (Value, Dividend, Multi-Factor, ...).</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr"/>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>You may not be able to buy a Closed / Limited fund.</t>
+          <t>'Not Applicable' or blank for regular funds.</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -3978,7 +3974,7 @@
       </c>
       <c r="I71" s="2" t="inlineStr">
         <is>
-          <t>Whether the fund is accepting money. 'Limited' is how Morningstar displays a fund that is closed to new investors (temporarily or permanently) while existing shareholders may still add to their holdings; 'Closed' means not accepting new purchases; 'Open' means open to all. Key facts: Limited = closed to new investors only; existing shareholders are not restricted from adding money.</t>
+          <t>For index-tracking funds whose index is 'strategic beta' (smart beta), the group of funds with a similar objective. Groups: Commodity, Dividend, Fixed Income, Fundamentals, Growth, Momentum, Multifactor, Quality, Risk-Oriented, Value, Other. Key facts: Assigned only to eligible index-tracking ETPs and open-end funds; standard (traditional) index funds get 'Not Applicable'. Blank for actively managed funds, funds tracking blended benchmarks, and leveraged/inverse ('trading' category) funds. Not all groups are factor tilts (e.g. Commodity, Fixed Income, Risk-Oriented such as low-vol/high-beta, Other). Taxonomy updated in 2018 from the older Return-Oriented / Risk-Oriented / Other scheme.</t>
         </is>
       </c>
       <c r="J71" s="2" t="inlineStr">
@@ -3988,31 +3984,31 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>https://gladmainnew.morningstar.com/directhelp/Glossary/Operations/Fund/Closed_to_New_Investors.htm</t>
+          <t>https://advhypo.morningstar.com/Enterprise/VTC/StrategicBetaandIndexStrategyDataMethedologyv2.pdf</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>Strategic Beta Group</t>
+          <t>Share Class Type</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr"/>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>For 'smart beta' index funds: the factor they tilt to (Value, Dividend, Multi-Factor, ...).</t>
+          <t>The sales channel / fee structure of the share class: No Load, Front Load (A), Level Load (C), Deferred Load (B), Institutional, Retirement, Investor, Advisor; this export also uses 'ETF'.</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr"/>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>ETF / No Load / Institutional are usually cheapest</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>'Not Applicable' or blank for regular funds.</t>
+          <t>Retirement and Institutional classes may only be available through employer plans or at high minimums.</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -4027,41 +4023,41 @@
       </c>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>For index-tracking funds whose index is 'strategic beta' (smart beta), the group of funds with a similar objective. Groups: Commodity, Dividend, Fixed Income, Fundamentals, Growth, Momentum, Multifactor, Quality, Risk-Oriented, Value, Other. Key facts: Assigned only to eligible index-tracking ETPs and open-end funds; standard (traditional) index funds get 'Not Applicable'. Blank for actively managed funds, funds tracking blended benchmarks, and leveraged/inverse ('trading' category) funds. Not all groups are factor tilts (e.g. Commodity, Fixed Income, Risk-Oriented such as low-vol/high-beta, Other). Taxonomy updated in 2018 from the older Return-Oriented / Risk-Oriented / Other scheme.</t>
+          <t>The distribution channel or fee structure a share class is sold through. Morningstar's main types are No Load, Front Load (A), Level Load (C), Deferred Load (B), Institutional, Retirement, Investor and Advisor; this export also labels exchange-traded share classes 'ETF'. Key facts: A = front load (typically 4-5.75%); B = deferred load; C = level load (~1% 12b-1); Inst = large institutional buyers, usually $1M+ minimum and lowest expenses; Retirement = retirement-plan classes; Other = not elsewhere classified (&lt;5% of funds).</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>Matches Morningstar</t>
+          <t>Corrected to Morningstar's definition</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>https://advhypo.morningstar.com/Enterprise/VTC/StrategicBetaandIndexStrategyDataMethedologyv2.pdf</t>
+          <t>https://morningstardirect.morningstar.com/clientcomm/Share_Class_Types.pdf</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>Share Class Type</t>
+          <t>Tender Offer</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr"/>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>The sales channel / fee structure of the share class: No Load, Front Load (A), Level Load (C), Deferred Load (B), Institutional, Retirement, Investor, Advisor; this export also uses 'ETF'.</t>
+          <t>Yes if the fund only buys back shares through periodic tender offers (limited liquidity).</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr"/>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>ETF / No Load / Institutional are usually cheapest</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Retirement and Institutional classes may only be available through employer plans or at high minimums.</t>
+          <t>Filter exclude_tender_offer_funds = OFF (ON = these funds are dropped).</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -4071,48 +4067,44 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (optional filter)</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>The distribution channel or fee structure a share class is sold through. Morningstar's main types are No Load, Front Load (A), Level Load (C), Deferred Load (B), Institutional, Retirement, Investor and Advisor; this export also labels exchange-traded share classes 'ETF'. Key facts: A = front load (typically 4-5.75%); B = deferred load; C = level load (~1% 12b-1); Inst = large institutional buyers, usually $1M+ minimum and lowest expenses; Retirement = retirement-plan classes; Other = not elsewhere classified (&lt;5% of funds).</t>
+          <t>A semiliquid (usually closed-end, unlisted) fund whose only exit for investors is periodic offers by the fund to buy back a portion of its shares, typically at or near NAV. Unlike interval funds, the fund and its board decide when, and whether, to make these offers. Key facts: Schedules are usually quarterly or annually but at board discretion; payments can be delayed; if more shares are tendered than offered, purchases are pro rata.</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>Corrected to Morningstar's definition</t>
+          <t>Matches Morningstar</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>https://morningstardirect.morningstar.com/clientcomm/Share_Class_Types.pdf</t>
+          <t>https://www.morningstar.com/funds/semiliquid-funds-are-coming-your-portfolio-are-you-ready-them</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>Tender Offer</t>
+          <t>Index Fund</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr"/>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Yes if the fund only buys back shares through periodic tender offers (limited liquidity).</t>
+          <t>Yes if the fund tracks an index (passive); No = actively managed.</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr"/>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>Filter exclude_tender_offer_funds = OFF (ON = these funds are dropped).</t>
-        </is>
-      </c>
+          <t>Neutral (index funds are usually cheaper)</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
           <t>Morningstar</t>
@@ -4120,12 +4112,12 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>A semiliquid (usually closed-end, unlisted) fund whose only exit for investors is periodic offers by the fund to buy back a portion of its shares, typically at or near NAV. Unlike interval funds, the fund and its board decide when, and whether, to make these offers. Key facts: Schedules are usually quarterly or annually but at board discretion; payments can be delayed; if more shares are tendered than offered, purchases are pro rata.</t>
+          <t>A fund that tracks a particular index and tries to match its returns (passive management). Key facts: Morningstar separately recognizes 'enhanced index' funds; a fund's tracked index is identified from its prospectus.</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr">
@@ -4135,29 +4127,33 @@
       </c>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>https://www.morningstar.com/funds/semiliquid-funds-are-coming-your-portfolio-are-you-ready-them</t>
+          <t>https://www.morningstar.com/investing-terms/index-fund</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>Index Fund</t>
+          <t>Maximum Deferred Load</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr"/>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Yes if the fund tracks an index (passive); No = actively managed.</t>
+          <t>Maximum back-end sales charge (CDSC) when selling, in percent.</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr"/>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Neutral (index funds are usually cheaper)</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr"/>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Hard filter max_deferred_load = 0%: funds above it are removed before scoring.</t>
+        </is>
+      </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
           <t>Morningstar</t>
@@ -4165,12 +4161,12 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (hard filter)</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>A fund that tracks a particular index and tries to match its returns (passive management). Key facts: Morningstar separately recognizes 'enhanced index' funds; a fund's tracked index is identified from its prospectus.</t>
+          <t>The maximum back-end sales charge (deferred load / CDSC) charged when an investor redeems shares; the percentage generally falls the longer the shares are held. Key facts: Often paired with 12b-1 fees as an alternative to a front-end load (typical of B and C shares). Not included in the expense ratio.</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr">
@@ -4180,20 +4176,20 @@
       </c>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>https://www.morningstar.com/investing-terms/index-fund</t>
+          <t>https://advhypo.morningstar.com/Enterprise/VTC/QP_Snapshot_disclosures_Brokerage.pdf</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>Maximum Deferred Load</t>
+          <t>Maximum Front Load</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr"/>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Maximum back-end sales charge (CDSC) when selling, in percent.</t>
+          <t>Maximum sales charge when buying, in percent.</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr"/>
@@ -4204,7 +4200,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Hard filter max_deferred_load = 0%: funds above it are removed before scoring.</t>
+          <t>Hard filter max_front_load = 0%: funds above it are removed before scoring.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4219,7 +4215,7 @@
       </c>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>The maximum back-end sales charge (deferred load / CDSC) charged when an investor redeems shares; the percentage generally falls the longer the shares are held. Key facts: Often paired with 12b-1 fees as an alternative to a front-end load (typical of B and C shares). Not included in the expense ratio.</t>
+          <t>The maximum initial sales charge, deducted from each purchase; the actual charge is generally based on the amount invested (breakpoints lower it for larger purchases). Key facts: Not included in the expense ratio. A shares typically 4%-5.75%. Maximum = rate before any breakpoint discounts.</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr">
@@ -4236,24 +4232,24 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>Maximum Front Load</t>
+          <t>Minimum Initial Investment</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr"/>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Maximum sales charge when buying, in percent.</t>
+          <t>Minimum dollars needed for the first purchase.</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr"/>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Lower is better (must fit your budget)</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Hard filter max_front_load = 0%: funds above it are removed before scoring.</t>
+          <t>Hard filter min_initial_investment = $50,000: funds whose minimum is above it are removed. Blank = no minimum reported (ETFs: one share). Brokers may waive minimums.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -4268,7 +4264,7 @@
       </c>
       <c r="I77" s="2" t="inlineStr">
         <is>
-          <t>The maximum initial sales charge, deducted from each purchase; the actual charge is generally based on the amount invested (breakpoints lower it for larger purchases). Key facts: Not included in the expense ratio. A shares typically 4%-5.75%. Maximum = rate before any breakpoint discounts.</t>
+          <t>The smallest amount the fund will accept to open a new account. Key facts: Separate data points exist for additional purchases, IRA minimums and automatic investment plan minimums, which are often lower.</t>
         </is>
       </c>
       <c r="J77" s="2" t="inlineStr">
@@ -4278,31 +4274,31 @@
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>https://advhypo.morningstar.com/Enterprise/VTC/QP_Snapshot_disclosures_Brokerage.pdf</t>
+          <t>https://www.morningstar.com/investing-terms/minimum-initial-investment</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>Minimum Initial Investment</t>
+          <t>Redemption Fee</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr"/>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Minimum dollars needed for the first purchase.</t>
+          <t>Fee charged when selling within a short holding period, in percent.</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr"/>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (must fit your budget)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Hard filter min_initial_investment = $50,000: funds whose minimum is above it are removed. Blank = no minimum reported (ETFs: one share). Brokers may waive minimums.</t>
+          <t>Hard filter max_redemption_fee = 0%: funds above it are removed before scoring.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4317,7 +4313,7 @@
       </c>
       <c r="I78" s="2" t="inlineStr">
         <is>
-          <t>The smallest amount the fund will accept to open a new account. Key facts: Separate data points exist for additional purchases, IRA minimums and automatic investment plan minimums, which are often lower.</t>
+          <t>Morningstar's 'Maximum Redemption Fee': the most a fund may charge if shares are sold within a specified period after purchase (for example 30, 180 or 365 days). Key facts: Expressed as a percent of the amount redeemed; applies only within the stated holding window; not a sales load.</t>
         </is>
       </c>
       <c r="J78" s="2" t="inlineStr">
@@ -4327,82 +4323,74 @@
       </c>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>https://www.morningstar.com/investing-terms/minimum-initial-investment</t>
+          <t>https://advhypo.morningstar.com/Enterprise/VTC/QP_Snapshot_disclosures_Brokerage.pdf</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>Redemption Fee</t>
+          <t>Risk Label</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr"/>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Fee charged when selling within a short holding period, in percent.</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr"/>
+          <t>Label part of 'Portfolio Risk Score': Conservative, Moderate, Aggressive, Very Aggressive or Extreme Risk.</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Text before the '(' in Portfolio Risk Score</t>
+        </is>
+      </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>Hard filter max_redemption_fee = 0%: funds above it are removed before scoring.</t>
-        </is>
-      </c>
+          <t>Lower risk for low-risk investing</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>No (hard filter)</t>
-        </is>
-      </c>
-      <c r="I79" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar's 'Maximum Redemption Fee': the most a fund may charge if shares are sold within a specified period after purchase (for example 30, 180 or 365 days). Key facts: Expressed as a percent of the amount redeemed; applies only within the stated holding window; not a sales load.</t>
-        </is>
-      </c>
-      <c r="J79" s="2" t="inlineStr">
-        <is>
-          <t>Matches Morningstar</t>
-        </is>
-      </c>
-      <c r="K79" s="2" t="inlineStr">
-        <is>
-          <t>https://advhypo.morningstar.com/Enterprise/VTC/QP_Snapshot_disclosures_Brokerage.pdf</t>
-        </is>
-      </c>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>Risk Label</t>
+          <t>Risk Score Numeric</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr"/>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>Label part of 'Portfolio Risk Score': Conservative, Moderate, Aggressive, Very Aggressive or Extreme Risk.</t>
+          <t>Number part of 'Portfolio Risk Score' (about 100 = as risky as a diversified all-stock portfolio).</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Text before the '(' in Portfolio Risk Score</t>
+          <t>Number inside the '( )' in Portfolio Risk Score</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Lower risk for low-risk investing</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr"/>
+          <t>Lower = less risky</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Above 100 ('Extreme Risk') = riskier than an all-stock portfolio, e.g. leveraged, single-sector or crypto funds (361 funds in this report).</t>
+        </is>
+      </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
           <t>Screener (calculated)</t>
@@ -4420,28 +4408,24 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Risk Score Numeric</t>
+          <t>Flag Leveraged Fund</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr"/>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>Number part of 'Portfolio Risk Score' (about 100 = as risky as a diversified all-stock portfolio).</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>Number inside the '( )' in Portfolio Risk Score</t>
-        </is>
-      </c>
+          <t>1 if 'Leveraged Fund' = Yes, else 0.</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr"/>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Lower = less risky</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Above 100 ('Extreme Risk') = riskier than an all-stock portfolio, e.g. leveraged, single-sector or crypto funds (361 funds in this report).</t>
+          <t>Helper for the structural filters.</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -4461,13 +4445,13 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Flag Leveraged Fund</t>
+          <t>Flag Interval Fund</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr"/>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Leveraged Fund' = Yes, else 0.</t>
+          <t>1 if 'Interval Fund' = Yes, else 0.</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr"/>
@@ -4498,13 +4482,13 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Flag Interval Fund</t>
+          <t>Flag Fund Of Funds</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr"/>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Interval Fund' = Yes, else 0.</t>
+          <t>1 if 'Fund of Funds' = Yes, else 0.</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr"/>
@@ -4535,13 +4519,13 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Flag Fund Of Funds</t>
+          <t>Flag Tender Offer</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr"/>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Fund of Funds' = Yes, else 0.</t>
+          <t>1 if 'Tender offer' = Yes, else 0.</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr"/>
@@ -4572,34 +4556,38 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Flag Tender Offer</t>
+          <t>Yahoo Subsector</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr"/>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Tender offer' = Yes, else 0.</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr"/>
+          <t>Industry group with the most weight among the fund's top 10 holdings (Yahoo), e.g. Semiconductors, Software &amp; Services, Banks. 'Broad Market Equity' when no industry dominates or no holdings data.</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>For each of the top 10 holdings: look up its industry → sub-sector; sum holding weights per sub-sector; pick the largest</t>
+        </is>
+      </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>n/a (grouping)</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Helper for the structural filters.</t>
+          <t>Refreshed about once a year. Diversified funds near a tie (e.g. Nvidia vs Microsoft) can flip between neighbouring labels. Not meaningful for bond / allocation funds. Fills the sector gap of Morningstar Category; used as the peer group for Z-scores.</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Yahoo Finance (calculated by screener)</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Used as peer group for Z Score</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr"/>
@@ -4609,28 +4597,32 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Subsector</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr"/>
+          <t>Sharpe</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>1Y, 3Y</t>
+        </is>
+      </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Industry group with the most weight among the fund's top 10 holdings (Yahoo), e.g. Semiconductors, Software &amp; Services, Banks. 'Broad Market Equity' when no industry dominates or no holdings data.</t>
+          <t>Sharpe ratio computed by the screener from Yahoo daily prices over the last 12 (1Y) or 36 (3Y) months - an independent check of Morningstar's.</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>For each of the top 10 holdings: look up its industry → sub-sector; sum holding weights per sub-sector; pick the largest</t>
+          <t>Monthly return r = month-end Adj Close change; Sharpe = mean(r - 4%/12) / std(r - 4%/12) x sqrt(12). Needs ≥ 11 months (1Y) or ≥ 30 months (3Y)</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>n/a (grouping)</t>
+          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Refreshed about once a year. Diversified funds near a tie (e.g. Nvidia vs Microsoft) can flip between neighbouring labels. Not meaningful for bond / allocation funds. Fills the sector gap of Morningstar Category; used as the peer group for Z-scores.</t>
+          <t>Differences from Morningstar's Sharpe come from price data and the fixed 4% risk-free rate.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -4640,7 +4632,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Used as peer group for Z Score</t>
+          <t>Yes - 3Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 1Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr"/>
@@ -4650,7 +4642,7 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Sharpe</t>
+          <t>Z Score</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -4660,27 +4652,27 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Sharpe ratio computed by the screener from Yahoo daily prices over the last 12 (1Y) or 36 (3Y) months - an independent check of Morningstar's.</t>
+          <t>How many standard deviations the fund's Yahoo Sharpe is above (+) or below (-) the average of all funds with the same Yahoo Subsector.</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Monthly return r = month-end Adj Close change; Sharpe = mean(r - 4%/12) / std(r - 4%/12) x sqrt(12). Needs ≥ 11 months (1Y) or ≥ 30 months (3Y)</t>
+          <t>Z = (fund Sharpe - mean Sharpe of its sub-sector) / std of Sharpe in its sub-sector; 0 if the sub-sector has no spread</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
+          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Differences from Morningstar's Sharpe come from price data and the fixed 4% risk-free rate.</t>
+          <t>Peer group = Yahoo Subsector (not Morningstar Category), so a bond fund labelled 'Broad Market Equity' is compared with stock funds. Read 1Y and 3Y together: both &gt;= +1 = Core (long-term leader still leading); 1Y &gt;= +1 but 3Y &lt; 0 = Momentum (recent surge, tactical trade, not an anchor); 1Y &lt; 0 but 3Y &gt;= +1 = Value (strong record in a temporary slump, possible buy-the-dip). List them with: python db_access/query.py zscore_matrix</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance (calculated by screener)</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -4695,32 +4687,24 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Z Score</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>1Y, 3Y</t>
-        </is>
-      </c>
+          <t>Yahoo Fetch Error</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr"/>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>How many standard deviations the fund's Yahoo Sharpe is above (+) or below (-) the average of all funds with the same Yahoo Subsector.</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>Z = (fund Sharpe - mean Sharpe of its sub-sector) / std of Sharpe in its sub-sector; 0 if the sub-sector has no spread</t>
-        </is>
-      </c>
+          <t>Message when Yahoo returned no data for the fund.</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr"/>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
+          <t>Blank</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Peer group = Yahoo Subsector (not Morningstar Category), so a bond fund labelled 'Broad Market Equity' is compared with stock funds. Read 1Y and 3Y together: both &gt;= +1 = Core (long-term leader still leading); 1Y &gt;= +1 but 3Y &lt; 0 = Momentum (recent surge, tactical trade, not an anchor); 1Y &lt; 0 but 3Y &gt;= +1 = Value (strong record in a temporary slump, possible buy-the-dip). List them with: python db_access/query.py zscore_matrix</t>
+          <t>Funds with no Yahoo prices are moved to the 'No Yahoo Data' tab.</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -4730,7 +4714,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 1Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr"/>
@@ -4740,24 +4724,28 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Fetch Error</t>
+          <t>Yahoo Data Suspect</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr"/>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Message when Yahoo returned no data for the fund.</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr"/>
+          <t>1 if the fund is older than 3 years (per Morningstar) but has no Yahoo 3Y Sharpe / Z-score.</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Inception Date ≤ today - 3 years AND (Sharpe 3Y or Z Score 3Y blank)</t>
+        </is>
+      </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Blank</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Funds with no Yahoo prices are moved to the 'No Yahoo Data' tab.</t>
+          <t>Usually an ETF converted from an older mutual fund (Yahoo only has the new ticker's prices).</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -4777,28 +4765,28 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Data Suspect</t>
+          <t>Long Term Return Performance Score</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr"/>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is older than 3 years (per Morningstar) but has no Yahoo 3Y Sharpe / Z-score.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1Y 3%, Total Return 2Y 4%, Total Return 3Y 8%, Total Return 4Y 8%, Total Return 5Y 15%, Total Return 6Y 7%, Total Return 7Y 7%, Total Return 8Y 7%, Total Return 9Y 7%, Total Return 10Y 15%, Total Return 15Y 12%, Total Return 20Y 7%.</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Inception Date ≤ today - 3 years AND (Sharpe 3Y or Z Score 3Y blank)</t>
+          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Usually an ETF converted from an older mutual fund (Yahoo only has the new ticker's prices).</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Missing periods (young funds) are skipped, not counted as 0.</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -4808,7 +4796,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr"/>
@@ -4818,13 +4806,13 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Long Term Return Performance Score</t>
+          <t>Short Term Return Performance Score</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr"/>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1Y 3%, Total Return 2Y 4%, Total Return 3Y 8%, Total Return 4Y 8%, Total Return 5Y 15%, Total Return 6Y 7%, Total Return 7Y 7%, Total Return 8Y 7%, Total Return 9Y 7%, Total Return 10Y 15%, Total Return 15Y 12%, Total Return 20Y 7%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1W 5%, Total Return 1M 16%, Total Return 2M 16%, Total Return QTD 16%, Total Return 3M 16%, Total Return 6M 13%, Total Return 9M 11%, Total Return YTD 5%.</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -4839,7 +4827,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Missing periods (young funds) are skipped, not counted as 0.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Recent momentum - changes quickly.</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -4849,7 +4837,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr"/>
@@ -4859,13 +4847,13 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Short Term Return Performance Score</t>
+          <t>Risk Adjusted Score</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr"/>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1W 5%, Total Return 1M 16%, Total Return 2M 16%, Total Return QTD 16%, Total Return 3M 16%, Total Return 6M 13%, Total Return 9M 11%, Total Return YTD 5%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Morningstar Sharpe 1Y 5%, Morningstar Sharpe 3Y 20%, Morningstar Sharpe 5Y 15%, Morningstar Sharpe 10Y 10%, Upside Capture 3Y 10%, Downside Capture 3Y 10% (inverted), Downside Capture 5Y 5% (inverted), Downside Capture 10Y 5% (inverted), Yahoo Sharpe 1Y 5%, Yahoo Sharpe 3Y 5%, Z Score 1Y 5%, Z Score 3Y 5%.</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -4880,7 +4868,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Recent momentum - changes quickly.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Missing Yahoo values drop out instead of counting as 0.</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -4890,7 +4878,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr"/>
@@ -4900,13 +4888,13 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Risk Adjusted Score</t>
+          <t>Volatility Score</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr"/>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Morningstar Sharpe 1Y 5%, Morningstar Sharpe 3Y 20%, Morningstar Sharpe 5Y 15%, Morningstar Sharpe 10Y 10%, Upside Capture 3Y 10%, Downside Capture 3Y 10% (inverted), Downside Capture 5Y 5% (inverted), Downside Capture 10Y 5% (inverted), Yahoo Sharpe 1Y 5%, Yahoo Sharpe 3Y 5%, Z Score 1Y 5%, Z Score 3Y 5%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Standard Deviation 3Y 20% (inverted), Standard Deviation 5Y 15% (inverted), Standard Deviation 10Y 5% (inverted), Max Drawdown 3Y 20%, Max Drawdown 5Y 25%, Max Drawdown 10Y 15%.</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -4921,7 +4909,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Missing Yahoo values drop out instead of counting as 0.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Blank for funds younger than 3 years. Max drawdown is negative, so it is NOT inverted: closer to 0 scores higher.</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -4931,7 +4919,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
+          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr"/>
@@ -4941,13 +4929,13 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Volatility Score</t>
+          <t>Resilience Score</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr"/>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Standard Deviation 3Y 20% (inverted), Standard Deviation 5Y 15% (inverted), Standard Deviation 10Y 5% (inverted), Max Drawdown 3Y 20%, Max Drawdown 5Y 25%, Max Drawdown 10Y 15%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Yearly Beat % 25%, Yearly Bottom 10% Count / Yearly Periods With Data 15% (inverted), Volatile Beat % 25%, Volatile Bottom 10% Count / Volatile Periods With Data 15% (inverted), Worst Three Month Return 20%.</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -4962,7 +4950,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Blank for funds younger than 3 years. Max drawdown is negative, so it is NOT inverted: closer to 0 scores higher.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. How consistently the fund beat the indexes: calendar years and the S&amp;P 500's volatile periods (crashes and recoveries). Bottom-10% counts are divided by the periods the fund has data for, so older funds aren't penalized for having more periods.</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -4972,7 +4960,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr"/>
@@ -4982,13 +4970,13 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Resilience Score</t>
+          <t>Tracking Score</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr"/>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Yearly Beat % 25%, Yearly Bottom 10% Count / Yearly Periods With Data 15% (inverted), Volatile Beat % 25%, Volatile Bottom 10% Count / Volatile Periods With Data 15% (inverted), Worst Three Month Return 20%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tracking Error 3Y 55% (inverted), Tracking Error 1Y 45% (inverted).</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -5003,7 +4991,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. How consistently the fund beat the indexes: calendar years and the S&amp;P 500's volatile periods (crashes and recoveries). Bottom-10% counts are divided by the periods the fund has data for, so older funds aren't penalized for having more periods.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Good for index funds; for active funds low tracking error just means 'close to the index'.</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -5013,7 +5001,7 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr"/>
@@ -5023,13 +5011,13 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Tracking Score</t>
+          <t>Liquidity Size Score</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr"/>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tracking Error 3Y 55% (inverted), Tracking Error 1Y 45% (inverted).</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Fund Size with fixed cutoffs ($10M → 0, $500M target, $5B → 100) 100%.</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -5044,7 +5032,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Good for index funds; for active funds low tracking error just means 'close to the index'.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Not within category.</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -5064,13 +5052,13 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Liquidity Size Score</t>
+          <t>Quality Valuation Score</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr"/>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Fund Size with fixed cutoffs ($10M → 0, $500M target, $5B → 100) 100%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Growth Grade 20%, Financial Health 15%, Profitability 15%, Price/Fair Value 15% (inverted), Medalist 15%, Star rating 15%, Wide moat 5%.</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -5085,7 +5073,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Not within category.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Mostly equity data; bond funds rely on Medalist and stars.</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -5095,7 +5083,7 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr"/>
@@ -5105,13 +5093,13 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Quality Valuation Score</t>
+          <t>Costs Score</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr"/>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Growth Grade 20%, Financial Health 15%, Profitability 15%, Price/Fair Value 15% (inverted), Medalist 15%, Star rating 15%, Wide moat 5%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Adjusted Expense Ratio 100% (inverted).</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -5126,7 +5114,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Mostly equity data; bond funds rely on Medalist and stars.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type.</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -5146,13 +5134,13 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Costs Score</t>
+          <t>Tax Income Score</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr"/>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Adjusted Expense Ratio 100% (inverted).</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tax Cost Ratio 1Y 29% (inverted), Tax Cost Ratio 2Y 21% (inverted), Dividend per Share (Trailing) 14%, SEC 30-Day Yield 36%.</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -5177,7 +5165,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>No - 0 weight in Profile LT</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr"/>
@@ -5187,28 +5175,32 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Tax Income Score</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr"/>
+          <t>Return Rank</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>1W, 1M, 2M, QTD, 3M, 6M, 9M, YTD, 1Y, 2Y, 3Y, 4Y, 5Y, 6Y, 7Y, 8Y, 9Y, 10Y, 15Y, 20Y</t>
+        </is>
+      </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tax Cost Ratio 1Y 29% (inverted), Tax Cost Ratio 2Y 21% (inverted), Dividend per Share (Trailing) 14%, SEC 30-Day Yield 36%.</t>
+          <t>Rank of the matching 'Total Return' column across ALL funds in the report (1 = highest return).</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
+          <t>Rank = position when all funds are sorted by that period's return, highest first (ties share the lowest rank)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>Lower is better (1 = best)</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type.</t>
+          <t>Across all categories, not within category - leveraged / sector funds dominate both ends. For momentum lists use python db_access/query.py momentum_top / momentum_bottom.</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -5218,7 +5210,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>No - 0 weight in Profile LT</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr"/>
@@ -5228,32 +5220,28 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Return Rank</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr">
-        <is>
-          <t>1W, 1M, 2M, QTD, 3M, 6M, 9M, YTD, 1Y, 2Y, 3Y, 4Y, 5Y, 6Y, 7Y, 8Y, 9Y, 10Y, 15Y, 20Y</t>
-        </is>
-      </c>
+          <t>Profile LT Score</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr"/>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Rank of the matching 'Total Return' column across ALL funds in the report (1 = highest return).</t>
+          <t>Final 0-100 score combining the concept scores with the weights in profile_long_term.yaml.</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>Rank = position when all funds are sorted by that period's return, highest first (ties share the lowest rank)</t>
+          <t>Profile LT Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Long-term Return 0.25, Short-term Return 0.05, Risk-adjusted 0.2, Volatility 0.15, Resilience 0.1, Tracking 0.05, Liquidity/Size 0.05, Quality/Valuation 0.1, Costs 0.1, Tax/Income 0 (sum 1.05, so each effective share = weight / 1.05)</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (1 = best)</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Across all categories, not within category - leveraged / sector funds dominate both ends. For momentum lists use python db_access/query.py momentum_top / momentum_bottom.</t>
+          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'.</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -5263,7 +5251,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>This IS the Profile LT score</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr"/>
@@ -5273,28 +5261,24 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Score</t>
+          <t>Profile LT Rank In Category</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr"/>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Final 0-100 score combining the concept scores with the weights in profile_long_term.yaml.</t>
-        </is>
-      </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>Profile LT Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Long-term Return 0.25, Short-term Return 0.05, Risk-adjusted 0.2, Volatility 0.15, Resilience 0.1, Tracking 0.05, Liquidity/Size 0.05, Quality/Valuation 0.1, Costs 0.1, Tax/Income 0 (sum 1.05, so each effective share = weight / 1.05)</t>
-        </is>
-      </c>
+          <t>Rank of the Profile LT Score within the fund's Morningstar Category (1 = best).</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr"/>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>Higher is better</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'.</t>
+          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -5304,7 +5288,7 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>This IS the Profile LT score</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I102" s="2" t="inlineStr"/>
@@ -5314,24 +5298,28 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank In Category</t>
+          <t>Profile LT Selected Flag</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr"/>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>Rank of the Profile LT Score within the fund's Morningstar Category (1 = best).</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr"/>
+          <t>1 if the fund is in the top 5 of its Morningstar Category by Profile LT Score.</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Rank In Category ≤ top_n_per_category (5)</t>
+        </is>
+      </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
+          <t>top_n_per_category is set in profile_long_term.yaml.</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -5351,28 +5339,24 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Selected Flag</t>
+          <t>Profile LT Rank Overall</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr"/>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is in the top 5 of its Morningstar Category by Profile LT Score.</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr">
-        <is>
-          <t>Rank In Category ≤ top_n_per_category (5)</t>
-        </is>
-      </c>
+          <t>Rank of the Profile LT Score across all funds (1 = best).</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr"/>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>top_n_per_category is set in profile_long_term.yaml.</t>
+          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -5392,24 +5376,28 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank Overall</t>
+          <t>Profile LT Selected Overall Flag</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr"/>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Rank of the Profile LT Score across all funds (1 = best).</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr"/>
+          <t>1 if the fund is in the top 100 overall.</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>Rank Overall ≤ top_n_overall (100)</t>
+        </is>
+      </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
+          <t>top_n_overall is set in profile_long_term.yaml (if left out, top_n_per_category is used).</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -5429,28 +5417,28 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Selected Overall Flag</t>
+          <t>Profile ST Score</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr"/>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is in the top 100 overall.</t>
+          <t>Final 0-100 score combining the concept scores with the weights in profile_short_term.yaml.</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Rank Overall ≤ top_n_overall (100)</t>
+          <t>Profile ST Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Short-term Return 0.4, Risk-adjusted 0.2, Volatility 0.1, Resilience 0, Liquidity/Size 0.1, Costs 0.1, Long-term Return 0.05, Quality/Valuation 0.05, Tracking 0, Tax/Income 0 (sum 1, so each effective share = weight / 1)</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>top_n_overall is set in profile_long_term.yaml (if left out, top_n_per_category is used).</t>
+          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'. Uses ST's own concept weights, so it can't be recomputed from the concept score columns in this report (those use LT's). Blank for funds profile_short_term.yaml filters out.</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -5460,7 +5448,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - this is the Profile ST score</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr"/>
@@ -5470,28 +5458,24 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Score</t>
+          <t>Profile ST Rank In Category</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr"/>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Final 0-100 score combining the concept scores with the weights in profile_short_term.yaml.</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Long-term Return 0.05, Short-term Return 0.4, Risk-adjusted 0.2, Volatility 0.1, Resilience 0, Tracking 0, Liquidity/Size 0.1, Quality/Valuation 0.05, Costs 0.1, Tax/Income 0 (sum 1, so each effective share = weight / 1)</t>
-        </is>
-      </c>
+          <t>Rank of the Profile ST Score within the fund's Morningstar Category (1 = best).</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr"/>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Higher is better</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'. Uses ST's own concept weights, so it can't be recomputed from the concept score columns in this report (those use LT's). Blank for funds profile_short_term.yaml filters out.</t>
+          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -5501,7 +5485,7 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>No - this is the Profile ST score</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I107" s="2" t="inlineStr"/>
@@ -5511,24 +5495,28 @@
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Rank In Category</t>
+          <t>Profile ST Selected Flag</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr"/>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Rank of the Profile ST Score within the fund's Morningstar Category (1 = best).</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr"/>
+          <t>1 if the fund is in the top 5 of its Morningstar Category by Profile ST Score.</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>Rank In Category ≤ top_n_per_category (5)</t>
+        </is>
+      </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
+          <t>top_n_per_category is set in profile_short_term.yaml.</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -5548,28 +5536,24 @@
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Selected Flag</t>
+          <t>Profile ST Rank Overall</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr"/>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is in the top 5 of its Morningstar Category by Profile ST Score.</t>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>Rank In Category ≤ top_n_per_category (5)</t>
-        </is>
-      </c>
+          <t>Rank of the Profile ST Score across all funds (1 = best).</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr"/>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>top_n_per_category is set in profile_short_term.yaml.</t>
+          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -5589,24 +5573,28 @@
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Rank Overall</t>
+          <t>Profile ST Selected Overall Flag</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr"/>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Rank of the Profile ST Score across all funds (1 = best).</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr"/>
+          <t>1 if the fund is in the top 25 overall.</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>Rank Overall ≤ top_n_overall (25)</t>
+        </is>
+      </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
+          <t>top_n_overall is set in profile_short_term.yaml (if left out, top_n_per_category is used).</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -5626,28 +5614,24 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Selected Overall Flag</t>
+          <t>Missing From Yahoo</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr"/>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is in the top 25 overall.</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr">
-        <is>
-          <t>Rank Overall ≤ top_n_overall (25)</t>
-        </is>
-      </c>
+          <t>('No Yahoo Data' tab only) Which Yahoo-based results are missing: Sharpe / Z-score, yearly returns, volatile periods.</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr"/>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>top_n_overall is set in profile_short_term.yaml (if left out, top_n_per_category is used).</t>
+          <t>These funds are taken off the overview; all their Morningstar columns are still on that tab.</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -5667,95 +5651,58 @@
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>Missing From Yahoo</t>
+          <t>Trading Volume</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr"/>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>('No Yahoo Data' tab only) Which Yahoo-based results are missing: Sharpe / Z-score, yearly returns, volatile periods.</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr"/>
+          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window.</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>Reported directly from exchange data</t>
+        </is>
+      </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Higher = easier to trade at a fair price</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>These funds are taken off the overview; all their Morningstar columns are still on that tab.</t>
+          <t>Not in the current eTrade export. The YAML still gives it weight 0.4 in Liquidity/Size; since the column is missing, Fund Size gets the whole Liquidity/Size weight. Add it to the export to use it.</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Morningstar (not in current data)</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I112" s="2" t="inlineStr"/>
-      <c r="J112" s="2" t="inlineStr"/>
-      <c r="K112" s="2" t="inlineStr"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="2" t="inlineStr">
-        <is>
-          <t>Trading Volume</t>
-        </is>
-      </c>
-      <c r="B113" s="2" t="inlineStr"/>
-      <c r="C113" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window.</t>
-        </is>
-      </c>
-      <c r="D113" s="2" t="inlineStr">
-        <is>
-          <t>Reported directly from exchange data</t>
-        </is>
-      </c>
-      <c r="E113" s="2" t="inlineStr">
-        <is>
-          <t>Higher = easier to trade at a fair price</t>
-        </is>
-      </c>
-      <c r="F113" s="2" t="inlineStr">
-        <is>
-          <t>Not in the current eTrade export. The YAML still gives it weight 0.4 in Liquidity/Size; since the column is missing, Fund Size gets the whole Liquidity/Size weight. Add it to the export to use it.</t>
-        </is>
-      </c>
-      <c r="G113" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar (not in current data)</t>
-        </is>
-      </c>
-      <c r="H113" s="2" t="inlineStr">
-        <is>
           <t>No effect: weighted 0.4 in the YAML, but the column is missing</t>
         </is>
       </c>
-      <c r="I113" s="2" t="inlineStr">
+      <c r="I112" s="2" t="inlineStr">
         <is>
           <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window. Key facts: Unit is shares, not dollars. Single-day volume and average volume are distinct fields; which one an export column holds depends on the data point chosen.</t>
         </is>
       </c>
-      <c r="J113" s="2" t="inlineStr">
+      <c r="J112" s="2" t="inlineStr">
         <is>
           <t>Corrected to Morningstar's definition</t>
         </is>
       </c>
-      <c r="K113" s="2" t="inlineStr">
+      <c r="K112" s="2" t="inlineStr">
         <is>
           <t>http://quote.morningstar.com/ETFdefinition.html</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K113"/>
+  <autoFilter ref="A1:K112"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5766,7 +5713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G252"/>
+  <dimension ref="A1:G251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -12302,7 +12249,7 @@
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>SEC 7-Day Yield</t>
+          <t>Dividend per Share (Trailing Annual)</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -12312,10 +12259,14 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>SEC 7-Day Yield</t>
-        </is>
-      </c>
-      <c r="D182" s="2" t="inlineStr"/>
+          <t>Dividend per Share</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Trailing Annual</t>
+        </is>
+      </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
           <t>Higher = more income</t>
@@ -12328,14 +12279,14 @@
       </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - Tax/Income has 0 weight in Profile LT (inputs: YAML weight 0.1 = 14% of Tax/Income (≈0.0% of Profile LT))</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>Dividend per Share (Trailing Annual)</t>
+          <t>Dividend per Share (Forward Annual)</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
@@ -12350,7 +12301,7 @@
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>Trailing Annual</t>
+          <t>Forward Annual</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr">
@@ -12365,14 +12316,14 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>No - Tax/Income has 0 weight in Profile LT (inputs: YAML weight 0.1 = 14% of Tax/Income (≈0.0% of Profile LT))</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>Dividend per Share (Forward Annual)</t>
+          <t>Dividend per Share (1Y Avg)</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -12387,7 +12338,7 @@
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>Forward Annual</t>
+          <t>1Y Avg</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr">
@@ -12409,7 +12360,7 @@
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>Dividend per Share (1Y Avg)</t>
+          <t>Dividend per Share (3Y Avg)</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
@@ -12424,7 +12375,7 @@
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>1Y Avg</t>
+          <t>3Y Avg</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
@@ -12446,7 +12397,7 @@
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>Dividend per Share (3Y Avg)</t>
+          <t>Leveraged Fund</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -12456,17 +12407,13 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>Dividend per Share</t>
-        </is>
-      </c>
-      <c r="D186" s="2" t="inlineStr">
-        <is>
-          <t>3Y Avg</t>
-        </is>
-      </c>
+          <t>Leveraged Fund</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr"/>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>Higher = more income</t>
+          <t>No for long-term holding</t>
         </is>
       </c>
       <c r="F186" s="2" t="inlineStr">
@@ -12476,14 +12423,14 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (optional filter)</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>Leveraged Fund</t>
+          <t>Interval Fund</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -12493,13 +12440,13 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>Leveraged Fund</t>
+          <t>Interval Fund</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr"/>
       <c r="E187" s="2" t="inlineStr">
         <is>
-          <t>No for long-term holding</t>
+          <t>No (more liquid)</t>
         </is>
       </c>
       <c r="F187" s="2" t="inlineStr">
@@ -12516,7 +12463,7 @@
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>Interval Fund</t>
+          <t>Fund of Funds</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -12526,13 +12473,13 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>Interval Fund</t>
+          <t>Fund of Funds</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr"/>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>No (more liquid)</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="F188" s="2" t="inlineStr">
@@ -12542,14 +12489,14 @@
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>Fund of Funds</t>
+          <t>Investment Status</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -12559,13 +12506,13 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>Fund of Funds</t>
+          <t>Investment Status</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr"/>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Open</t>
         </is>
       </c>
       <c r="F189" s="2" t="inlineStr">
@@ -12582,7 +12529,7 @@
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>Investment Status</t>
+          <t>Strategic Beta Group</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -12592,13 +12539,13 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>Investment Status</t>
+          <t>Strategic Beta Group</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr"/>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
@@ -12615,7 +12562,7 @@
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>Strategic Beta Group</t>
+          <t>Share Class Type</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -12625,13 +12572,13 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>Strategic Beta Group</t>
+          <t>Share Class Type</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr"/>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>ETF / No Load / Institutional are usually cheapest</t>
         </is>
       </c>
       <c r="F191" s="2" t="inlineStr">
@@ -12648,7 +12595,7 @@
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>Share Class Type</t>
+          <t>Tender Offer</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -12658,13 +12605,13 @@
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Share Class Type</t>
+          <t>Tender Offer</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr"/>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>ETF / No Load / Institutional are usually cheapest</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F192" s="2" t="inlineStr">
@@ -12674,14 +12621,14 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (optional filter)</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>Tender Offer</t>
+          <t>Index Fund</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -12691,13 +12638,13 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Tender Offer</t>
+          <t>Index Fund</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr"/>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Neutral (index funds are usually cheaper)</t>
         </is>
       </c>
       <c r="F193" s="2" t="inlineStr">
@@ -12707,14 +12654,14 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>Index Fund</t>
+          <t>Maximum Deferred Load</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -12724,13 +12671,13 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Index Fund</t>
+          <t>Maximum Deferred Load</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr"/>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>Neutral (index funds are usually cheaper)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F194" s="2" t="inlineStr">
@@ -12740,14 +12687,14 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No (hard filter)</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>Maximum Deferred Load</t>
+          <t>Maximum Front Load</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -12757,7 +12704,7 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Maximum Deferred Load</t>
+          <t>Maximum Front Load</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr"/>
@@ -12780,7 +12727,7 @@
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>Maximum Front Load</t>
+          <t>Minimum Initial Investment</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -12790,13 +12737,13 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Maximum Front Load</t>
+          <t>Minimum Initial Investment</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr"/>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Lower is better (must fit your budget)</t>
         </is>
       </c>
       <c r="F196" s="2" t="inlineStr">
@@ -12813,7 +12760,7 @@
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>Minimum Initial Investment</t>
+          <t>Redemption Fee</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -12823,13 +12770,13 @@
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>Minimum Initial Investment</t>
+          <t>Redemption Fee</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr"/>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (must fit your budget)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F197" s="2" t="inlineStr">
@@ -12846,7 +12793,7 @@
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>Redemption Fee</t>
+          <t>Risk Label</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -12856,30 +12803,30 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Redemption Fee</t>
+          <t>Risk Label</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr"/>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Lower risk for low-risk investing</t>
         </is>
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>Morningstar</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
         <is>
-          <t>No (hard filter)</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>Risk Label</t>
+          <t>Risk Score Numeric</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -12889,13 +12836,13 @@
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>Risk Label</t>
+          <t>Risk Score Numeric</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr"/>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>Lower risk for low-risk investing</t>
+          <t>Lower = less risky</t>
         </is>
       </c>
       <c r="F199" s="2" t="inlineStr">
@@ -12912,7 +12859,7 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>Risk Score Numeric</t>
+          <t>Flag Leveraged Fund</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -12922,13 +12869,13 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Risk Score Numeric</t>
+          <t>Flag Leveraged Fund</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr"/>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>Lower = less risky</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F200" s="2" t="inlineStr">
@@ -12945,7 +12892,7 @@
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>Flag Leveraged Fund</t>
+          <t>Flag Interval Fund</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -12955,7 +12902,7 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>Flag Leveraged Fund</t>
+          <t>Flag Interval Fund</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr"/>
@@ -12978,7 +12925,7 @@
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>Flag Interval Fund</t>
+          <t>Flag Fund Of Funds</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -12988,7 +12935,7 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Flag Interval Fund</t>
+          <t>Flag Fund Of Funds</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr"/>
@@ -13011,7 +12958,7 @@
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Flag Fund Of Funds</t>
+          <t>Flag Tender Offer</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -13021,7 +12968,7 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>Flag Fund Of Funds</t>
+          <t>Flag Tender Offer</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr"/>
@@ -13044,7 +12991,7 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Flag Tender Offer</t>
+          <t>Yahoo Subsector</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -13054,30 +13001,30 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Flag Tender Offer</t>
+          <t>Yahoo Subsector</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr"/>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>n/a (grouping)</t>
         </is>
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Yahoo Finance (calculated by screener)</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Used as peer group for Z Score</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Subsector</t>
+          <t>Sharpe 1y</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -13087,13 +13034,17 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Subsector</t>
-        </is>
-      </c>
-      <c r="D205" s="2" t="inlineStr"/>
+          <t>Sharpe</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>1Y</t>
+        </is>
+      </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>n/a (grouping)</t>
+          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
         </is>
       </c>
       <c r="F205" s="2" t="inlineStr">
@@ -13103,14 +13054,14 @@
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>Used as peer group for Z Score</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Sharpe 1y</t>
+          <t>Sharpe 3y</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -13125,7 +13076,7 @@
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>1Y</t>
+          <t>3Y</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
@@ -13147,7 +13098,7 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Sharpe 3y</t>
+          <t>Z Score 1y</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -13157,22 +13108,22 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Sharpe</t>
+          <t>Z Score</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>3Y</t>
+          <t>1Y</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
+          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
         </is>
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance (calculated by screener)</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -13184,7 +13135,7 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>Z Score 1y</t>
+          <t>Z Score 3y</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -13199,7 +13150,7 @@
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>1Y</t>
+          <t>3Y</t>
         </is>
       </c>
       <c r="E208" s="2" t="inlineStr">
@@ -13221,7 +13172,7 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Z Score 3y</t>
+          <t>Yahoo Fetch Error</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -13231,17 +13182,13 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Z Score</t>
-        </is>
-      </c>
-      <c r="D209" s="2" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
+          <t>Yahoo Fetch Error</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr"/>
       <c r="E209" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
+          <t>Blank</t>
         </is>
       </c>
       <c r="F209" s="2" t="inlineStr">
@@ -13251,14 +13198,14 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Fetch Error</t>
+          <t>Yahoo Data Suspect</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -13268,13 +13215,13 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Fetch Error</t>
+          <t>Yahoo Data Suspect</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr"/>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>Blank</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F210" s="2" t="inlineStr">
@@ -13291,7 +13238,7 @@
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Data Suspect</t>
+          <t>Long Term Return Performance Score</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -13301,13 +13248,13 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Data Suspect</t>
+          <t>Long Term Return Performance Score</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr"/>
       <c r="E211" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F211" s="2" t="inlineStr">
@@ -13317,14 +13264,14 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>Long Term Return Performance Score</t>
+          <t>Short Term Return Performance Score</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -13334,7 +13281,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Long Term Return Performance Score</t>
+          <t>Short Term Return Performance Score</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr"/>
@@ -13350,14 +13297,14 @@
       </c>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>Short Term Return Performance Score</t>
+          <t>Risk Adjusted Score</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -13367,7 +13314,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>Short Term Return Performance Score</t>
+          <t>Risk Adjusted Score</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr"/>
@@ -13383,14 +13330,14 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>Risk Adjusted Score</t>
+          <t>Volatility Score</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -13400,7 +13347,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Risk Adjusted Score</t>
+          <t>Volatility Score</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr"/>
@@ -13416,14 +13363,14 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
+          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Volatility Score</t>
+          <t>Resilience Score</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -13433,7 +13380,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>Volatility Score</t>
+          <t>Resilience Score</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr"/>
@@ -13449,14 +13396,14 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Resilience Score</t>
+          <t>Tracking Score</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -13466,7 +13413,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Resilience Score</t>
+          <t>Tracking Score</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr"/>
@@ -13482,14 +13429,14 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Tracking Score</t>
+          <t>Liquidity Size Score</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -13499,7 +13446,7 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>Tracking Score</t>
+          <t>Liquidity Size Score</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr"/>
@@ -13522,7 +13469,7 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Liquidity Size Score</t>
+          <t>Quality Valuation Score</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -13532,7 +13479,7 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Liquidity Size Score</t>
+          <t>Quality Valuation Score</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr"/>
@@ -13548,14 +13495,14 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Quality Valuation Score</t>
+          <t>Costs Score</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -13565,7 +13512,7 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>Quality Valuation Score</t>
+          <t>Costs Score</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr"/>
@@ -13588,7 +13535,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Costs Score</t>
+          <t>Tax Income Score</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -13598,7 +13545,7 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Costs Score</t>
+          <t>Tax Income Score</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr"/>
@@ -13614,14 +13561,14 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>No - 0 weight in Profile LT</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Tax Income Score</t>
+          <t>Return Rank (1W)</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -13631,13 +13578,17 @@
       </c>
       <c r="C221" s="2" t="inlineStr">
         <is>
-          <t>Tax Income Score</t>
-        </is>
-      </c>
-      <c r="D221" s="2" t="inlineStr"/>
+          <t>Return Rank</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
       <c r="E221" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>Lower is better (1 = best)</t>
         </is>
       </c>
       <c r="F221" s="2" t="inlineStr">
@@ -13647,14 +13598,14 @@
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>No - 0 weight in Profile LT</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (1W)</t>
+          <t>Return Rank (1M)</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -13669,7 +13620,7 @@
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>1W</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
@@ -13691,7 +13642,7 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (1M)</t>
+          <t>Return Rank (2M)</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -13706,7 +13657,7 @@
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>2M</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr">
@@ -13728,7 +13679,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (2M)</t>
+          <t>Return Rank (QTD)</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -13743,7 +13694,7 @@
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>2M</t>
+          <t>QTD</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
@@ -13765,7 +13716,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (QTD)</t>
+          <t>Return Rank (3M)</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -13780,7 +13731,7 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>QTD</t>
+          <t>3M</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
@@ -13802,7 +13753,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (3M)</t>
+          <t>Return Rank (6M)</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -13817,7 +13768,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>3M</t>
+          <t>6M</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
@@ -13839,7 +13790,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (6M)</t>
+          <t>Return Rank (9M)</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -13854,7 +13805,7 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>6M</t>
+          <t>9M</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
@@ -13876,7 +13827,7 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (9M)</t>
+          <t>Return Rank (YTD)</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -13891,7 +13842,7 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>9M</t>
+          <t>YTD</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
@@ -13913,7 +13864,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (YTD)</t>
+          <t>Return Rank (1Y)</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -13928,7 +13879,7 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>YTD</t>
+          <t>1Y</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
@@ -13950,7 +13901,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (1Y)</t>
+          <t>Return Rank (2Y)</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -13965,7 +13916,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>1Y</t>
+          <t>2Y</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
@@ -13987,7 +13938,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (2Y)</t>
+          <t>Return Rank (3Y)</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -14002,7 +13953,7 @@
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>2Y</t>
+          <t>3Y</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
@@ -14024,7 +13975,7 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (3Y)</t>
+          <t>Return Rank (4Y)</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -14039,7 +13990,7 @@
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>3Y</t>
+          <t>4Y</t>
         </is>
       </c>
       <c r="E232" s="2" t="inlineStr">
@@ -14061,7 +14012,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (4Y)</t>
+          <t>Return Rank (5Y)</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -14076,7 +14027,7 @@
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>4Y</t>
+          <t>5Y</t>
         </is>
       </c>
       <c r="E233" s="2" t="inlineStr">
@@ -14098,7 +14049,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (5Y)</t>
+          <t>Return Rank (6Y)</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -14113,7 +14064,7 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>5Y</t>
+          <t>6Y</t>
         </is>
       </c>
       <c r="E234" s="2" t="inlineStr">
@@ -14135,7 +14086,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (6Y)</t>
+          <t>Return Rank (7Y)</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -14150,7 +14101,7 @@
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>6Y</t>
+          <t>7Y</t>
         </is>
       </c>
       <c r="E235" s="2" t="inlineStr">
@@ -14172,7 +14123,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (7Y)</t>
+          <t>Return Rank (8Y)</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -14187,7 +14138,7 @@
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>7Y</t>
+          <t>8Y</t>
         </is>
       </c>
       <c r="E236" s="2" t="inlineStr">
@@ -14209,7 +14160,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (8Y)</t>
+          <t>Return Rank (9Y)</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -14224,7 +14175,7 @@
       </c>
       <c r="D237" s="2" t="inlineStr">
         <is>
-          <t>8Y</t>
+          <t>9Y</t>
         </is>
       </c>
       <c r="E237" s="2" t="inlineStr">
@@ -14246,7 +14197,7 @@
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (9Y)</t>
+          <t>Return Rank (10Y)</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -14261,7 +14212,7 @@
       </c>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>9Y</t>
+          <t>10Y</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr">
@@ -14283,7 +14234,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (10Y)</t>
+          <t>Return Rank (15Y)</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -14298,7 +14249,7 @@
       </c>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>10Y</t>
+          <t>15Y</t>
         </is>
       </c>
       <c r="E239" s="2" t="inlineStr">
@@ -14320,7 +14271,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (15Y)</t>
+          <t>Return Rank (20Y)</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -14335,7 +14286,7 @@
       </c>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>15Y</t>
+          <t>20Y</t>
         </is>
       </c>
       <c r="E240" s="2" t="inlineStr">
@@ -14357,7 +14308,7 @@
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (20Y)</t>
+          <t>Profile LT Score</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -14367,17 +14318,13 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Return Rank</t>
-        </is>
-      </c>
-      <c r="D241" s="2" t="inlineStr">
-        <is>
-          <t>20Y</t>
-        </is>
-      </c>
+          <t>Profile LT Score</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr"/>
       <c r="E241" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (1 = best)</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F241" s="2" t="inlineStr">
@@ -14387,14 +14334,14 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>This IS the Profile LT score</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Score</t>
+          <t>Profile LT Rank In Category</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -14404,13 +14351,13 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Score</t>
+          <t>Profile LT Rank In Category</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr"/>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>Higher is better</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F242" s="2" t="inlineStr">
@@ -14420,14 +14367,14 @@
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t>This IS the Profile LT score</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank In Category</t>
+          <t>Profile LT Selected Flag</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
@@ -14437,13 +14384,13 @@
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank In Category</t>
+          <t>Profile LT Selected Flag</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr"/>
       <c r="E243" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F243" s="2" t="inlineStr">
@@ -14460,7 +14407,7 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Selected Flag</t>
+          <t>Profile LT Rank Overall</t>
         </is>
       </c>
       <c r="B244" s="2" t="inlineStr">
@@ -14470,13 +14417,13 @@
       </c>
       <c r="C244" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Selected Flag</t>
+          <t>Profile LT Rank Overall</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr"/>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F244" s="2" t="inlineStr">
@@ -14493,7 +14440,7 @@
     <row r="245">
       <c r="A245" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank Overall</t>
+          <t>Profile LT Selected Overall Flag</t>
         </is>
       </c>
       <c r="B245" s="2" t="inlineStr">
@@ -14503,13 +14450,13 @@
       </c>
       <c r="C245" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank Overall</t>
+          <t>Profile LT Selected Overall Flag</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr"/>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F245" s="2" t="inlineStr">
@@ -14526,7 +14473,7 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Selected Overall Flag</t>
+          <t>Profile ST Score</t>
         </is>
       </c>
       <c r="B246" s="2" t="inlineStr">
@@ -14536,13 +14483,13 @@
       </c>
       <c r="C246" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Selected Overall Flag</t>
+          <t>Profile ST Score</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr"/>
       <c r="E246" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F246" s="2" t="inlineStr">
@@ -14552,14 +14499,14 @@
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - this is the Profile ST score</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Score</t>
+          <t>Profile ST Rank In Category</t>
         </is>
       </c>
       <c r="B247" s="2" t="inlineStr">
@@ -14569,13 +14516,13 @@
       </c>
       <c r="C247" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Score</t>
+          <t>Profile ST Rank In Category</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr"/>
       <c r="E247" s="2" t="inlineStr">
         <is>
-          <t>Higher is better</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F247" s="2" t="inlineStr">
@@ -14585,14 +14532,14 @@
       </c>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>No - this is the Profile ST score</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Rank In Category</t>
+          <t>Profile ST Selected Flag</t>
         </is>
       </c>
       <c r="B248" s="2" t="inlineStr">
@@ -14602,13 +14549,13 @@
       </c>
       <c r="C248" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Rank In Category</t>
+          <t>Profile ST Selected Flag</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr"/>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F248" s="2" t="inlineStr">
@@ -14625,7 +14572,7 @@
     <row r="249">
       <c r="A249" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Selected Flag</t>
+          <t>Profile ST Rank Overall</t>
         </is>
       </c>
       <c r="B249" s="2" t="inlineStr">
@@ -14635,13 +14582,13 @@
       </c>
       <c r="C249" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Selected Flag</t>
+          <t>Profile ST Rank Overall</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr"/>
       <c r="E249" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F249" s="2" t="inlineStr">
@@ -14658,7 +14605,7 @@
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Rank Overall</t>
+          <t>Profile ST Selected Overall Flag</t>
         </is>
       </c>
       <c r="B250" s="2" t="inlineStr">
@@ -14668,13 +14615,13 @@
       </c>
       <c r="C250" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Rank Overall</t>
+          <t>Profile ST Selected Overall Flag</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr"/>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>1 = selected</t>
         </is>
       </c>
       <c r="F250" s="2" t="inlineStr">
@@ -14691,23 +14638,23 @@
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Selected Overall Flag</t>
+          <t>Missing From Yahoo</t>
         </is>
       </c>
       <c r="B251" s="2" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>No Yahoo Data</t>
         </is>
       </c>
       <c r="C251" s="2" t="inlineStr">
         <is>
-          <t>Profile ST Selected Overall Flag</t>
+          <t>Missing From Yahoo</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr"/>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F251" s="2" t="inlineStr">
@@ -14721,41 +14668,8 @@
         </is>
       </c>
     </row>
-    <row r="252">
-      <c r="A252" s="2" t="inlineStr">
-        <is>
-          <t>Missing From Yahoo</t>
-        </is>
-      </c>
-      <c r="B252" s="2" t="inlineStr">
-        <is>
-          <t>No Yahoo Data</t>
-        </is>
-      </c>
-      <c r="C252" s="2" t="inlineStr">
-        <is>
-          <t>Missing From Yahoo</t>
-        </is>
-      </c>
-      <c r="D252" s="2" t="inlineStr"/>
-      <c r="E252" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F252" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G252" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G252"/>
+  <autoFilter ref="A1:G251"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Profile YAMLs only score funds; shared purchase rules are the only filters
- New config.PURCHASE_RULES, applied once for every profile right after
  loading: no front or deferred load, no redemption fee, minimum initial
  investment <= $50,000
- Remove every filter key from the profile YAMLs (expense cap, 3-year history,
  category, fund size, leveraged / interval / tender-offer, benchmark
  outperformance); a weight of 0.0 is how to make something not count
- Every fund now gets a score from every profile, so the report no longer
  depends on profile order; add_profile_columns still adds funds only a later
  profile scores, for profile modules with their own filter
- Column dictionary, README and YAML comments describe the new rules
- Yahoo sub-sector and volatile-period caches gain the newly scored funds

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_screener/docs/report_column_dictionary.xlsx
+++ b/etf_screener/docs/report_column_dictionary.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Filter require_category = OFF (ON = drop funds with no category). Every score and in-category rank compares a fund ONLY with funds in the same category. 132 categories in this report (a few appear twice under ETF vs mutual-fund naming, e.g. 'Mid-Cap Blend' / 'Mid Blend'). Sector caveat: categories are coarse - e.g. 'Technology' mixes semiconductor-heavy and software-heavy funds, which behave very differently; see the Yahoo Subsector column and the 'Scoring Concepts' tab.</t>
+          <t>Every score and in-category rank compares a fund ONLY with funds in the same category. 132 categories in this report (a few appear twice under ETF vs mutual-fund naming, e.g. 'Mid-Cap Blend' / 'Mid Blend'). Sector caveat: categories are coarse - e.g. 'Technology' mixes semiconductor-heavy and software-heavy funds, which behave very differently; see the Yahoo Subsector column and the 'Scoring Concepts' tab.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Compare within category - a 5% year is great for a bond fund and poor for a tech fund. Blank when the fund is younger than the period. Sector caveat: multi-year returns are strongly driven by sub-sector timing (e.g. AI semiconductors vs software), which within-category ranking does not correct for. 'Since Inception' is not comparable across funds with different start dates. Filter require_3y_return = LT ON, ST OFF (ON = drop funds with a blank 3Y return, i.e. under 3 years old).</t>
+          <t>Compare within category - a 5% year is great for a bond fund and poor for a tech fund. Blank when the fund is younger than the period. Sector caveat: multi-year returns are strongly driven by sub-sector timing (e.g. AI semiconductors vs software), which within-category ranking does not correct for. 'Since Inception' is not comparable across funds with different start dates. A fund younger than a period has that return blank, and it simply drops out of the fund's score.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -2418,7 +2418,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Waivers can expire. Index ETFs are often &lt; 0.10%, active funds 0.5-1%. Filter max_expense_ratio = LT 1.25%, ST 1.75%: funds above it are dropped (a blank ratio is kept). Sector-neutral: driven by passive vs active, not holdings.</t>
+          <t>Waivers can expire. Index ETFs are often &lt; 0.10%, active funds 0.5-1%. Sector-neutral: driven by passive vs active, not holdings. Expense counts in the score through the Costs concept (Adjusted Expense Ratio).</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2428,7 +2428,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>No (used as the max_expense_ratio filter)</t>
+          <t>No (Costs uses Adjusted Expense Ratio)</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Popularity / age driven; little sector link. 'Trading Volume' (YAML weight 0.4) is not in the data, so Fund Size is effectively the whole Liquidity/Size score. Filter require_fund_size = OFF (ON = drop funds with a blank Fund Size).</t>
+          <t>Popularity / age driven; little sector link. 'Trading Volume' (YAML weight 0.4) is not in the data, so Fund Size is effectively the whole Liquidity/Size score.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Leveraged funds reset daily and lose value in choppy markets ('volatility decay'). Filter exclude_leveraged_funds = LT OFF, ST ON (ON = these funds are dropped).</t>
+          <t>Leveraged funds reset daily and lose value in choppy markets ('volatility decay'). Kept in every profile (no leveraged filter); compare them with care.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Filter exclude_interval_funds = OFF (ON = these funds are dropped).</t>
+          <t>Kept and scored like other funds; check liquidity before buying.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Filter exclude_tender_offer_funds = OFF (ON = these funds are dropped).</t>
+          <t>Kept and scored like other funds; check liquidity before buying.</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I73" s="2" t="inlineStr">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Hard filter max_deferred_load = 0%: funds above it are removed before scoring.</t>
+          <t>Purchase rule for every profile (max_deferred_load = 0%, config.PURCHASE_RULES): funds above it are removed before scoring.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -4200,7 +4200,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>Hard filter max_front_load = 0%: funds above it are removed before scoring.</t>
+          <t>Purchase rule for every profile (max_front_load = 0%, config.PURCHASE_RULES): funds above it are removed before scoring.</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Hard filter min_initial_investment = $50,000: funds whose minimum is above it are removed. Blank = no minimum reported (ETFs: one share). Brokers may waive minimums.</t>
+          <t>Purchase rule for every profile (min_initial_investment = $50,000, config.PURCHASE_RULES): funds whose minimum is above it are removed. Blank = no minimum reported (ETFs: one share). Brokers may waive minimums.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>Hard filter max_redemption_fee = 0%: funds above it are removed before scoring.</t>
+          <t>Purchase rule for every profile (max_redemption_fee = 0%, config.PURCHASE_RULES): funds above it are removed before scoring.</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -4408,34 +4408,38 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>Flag Leveraged Fund</t>
+          <t>Yahoo Subsector</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr"/>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Leveraged Fund' = Yes, else 0.</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr"/>
+          <t>Industry group with the most weight among the fund's top 10 holdings (Yahoo), e.g. Semiconductors, Software &amp; Services, Banks. 'Broad Market Equity' when no industry dominates or no holdings data.</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>For each of the top 10 holdings: look up its industry → sub-sector; sum holding weights per sub-sector; pick the largest</t>
+        </is>
+      </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>n/a (grouping)</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>Helper for the structural filters.</t>
+          <t>Refreshed about once a year. Diversified funds near a tie (e.g. Nvidia vs Microsoft) can flip between neighbouring labels. Not meaningful for bond / allocation funds. Fills the sector gap of Morningstar Category; used as the peer group for Z-scores.</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Yahoo Finance (calculated by screener)</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Used as peer group for Z Score</t>
         </is>
       </c>
       <c r="I81" s="2" t="inlineStr"/>
@@ -4445,34 +4449,42 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>Flag Interval Fund</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr"/>
+          <t>Sharpe</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>1Y, 3Y</t>
+        </is>
+      </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Interval Fund' = Yes, else 0.</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr"/>
+          <t>Sharpe ratio computed by the screener from Yahoo daily prices over the last 12 (1Y) or 36 (3Y) months - an independent check of Morningstar's.</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Monthly return r = month-end Adj Close change; Sharpe = mean(r - 4%/12) / std(r - 4%/12) x sqrt(12). Needs ≥ 11 months (1Y) or ≥ 30 months (3Y)</t>
+        </is>
+      </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Helper for the structural filters.</t>
+          <t>Differences from Morningstar's Sharpe come from price data and the fixed 4% risk-free rate.</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Yahoo Finance (calculated by screener)</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - 3Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 1Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr"/>
@@ -4482,24 +4494,32 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>Flag Fund Of Funds</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr"/>
+          <t>Z Score</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>1Y, 3Y</t>
+        </is>
+      </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Fund of Funds' = Yes, else 0.</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr"/>
+          <t>How many standard deviations the fund's Yahoo Sharpe is above (+) or below (-) the average of all funds with the same Yahoo Subsector.</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Z = (fund Sharpe - mean Sharpe of its sub-sector) / std of Sharpe in its sub-sector; 0 if the sub-sector has no spread</t>
+        </is>
+      </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Helper for the structural filters.</t>
+          <t>Peer group = Yahoo Subsector (not Morningstar Category), so a bond fund labelled 'Broad Market Equity' is compared with stock funds. Read 1Y and 3Y together: both &gt;= +1 = Core (long-term leader still leading); 1Y &gt;= +1 but 3Y &lt; 0 = Momentum (recent surge, tactical trade, not an anchor); 1Y &lt; 0 but 3Y &gt;= +1 = Value (strong record in a temporary slump, possible buy-the-dip). List them with: python db_access/query.py zscore_matrix</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -4509,7 +4529,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - 3Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 1Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr"/>
@@ -4519,24 +4539,24 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>Flag Tender Offer</t>
+          <t>Yahoo Fetch Error</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr"/>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Tender offer' = Yes, else 0.</t>
+          <t>Message when Yahoo returned no data for the fund.</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr"/>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Blank</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Helper for the structural filters.</t>
+          <t>Funds with no Yahoo prices are moved to the 'No Yahoo Data' tab.</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -4556,38 +4576,38 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Subsector</t>
+          <t>Yahoo Data Suspect</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr"/>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Industry group with the most weight among the fund's top 10 holdings (Yahoo), e.g. Semiconductors, Software &amp; Services, Banks. 'Broad Market Equity' when no industry dominates or no holdings data.</t>
+          <t>1 if the fund is older than 3 years (per Morningstar) but has no Yahoo 3Y Sharpe / Z-score.</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>For each of the top 10 holdings: look up its industry → sub-sector; sum holding weights per sub-sector; pick the largest</t>
+          <t>Inception Date ≤ today - 3 years AND (Sharpe 3Y or Z Score 3Y blank)</t>
         </is>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>n/a (grouping)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>Refreshed about once a year. Diversified funds near a tie (e.g. Nvidia vs Microsoft) can flip between neighbouring labels. Not meaningful for bond / allocation funds. Fills the sector gap of Morningstar Category; used as the peer group for Z-scores.</t>
+          <t>Usually an ETF converted from an older mutual fund (Yahoo only has the new ticker's prices).</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance (calculated by screener)</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>Used as peer group for Z Score</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr"/>
@@ -4597,42 +4617,38 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>Sharpe</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>1Y, 3Y</t>
-        </is>
-      </c>
+          <t>Long Term Return Performance Score</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr"/>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Sharpe ratio computed by the screener from Yahoo daily prices over the last 12 (1Y) or 36 (3Y) months - an independent check of Morningstar's.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1Y 3%, Total Return 2Y 4%, Total Return 3Y 8%, Total Return 4Y 8%, Total Return 5Y 15%, Total Return 6Y 7%, Total Return 7Y 7%, Total Return 8Y 7%, Total Return 9Y 7%, Total Return 10Y 15%, Total Return 15Y 12%, Total Return 20Y 7%.</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Monthly return r = month-end Adj Close change; Sharpe = mean(r - 4%/12) / std(r - 4%/12) x sqrt(12). Needs ≥ 11 months (1Y) or ≥ 30 months (3Y)</t>
+          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>Differences from Morningstar's Sharpe come from price data and the fixed 4% risk-free rate.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Missing periods (young funds) are skipped, not counted as 0.</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance (calculated by screener)</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 1Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
+          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr"/>
@@ -4642,32 +4658,28 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>Z Score</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>1Y, 3Y</t>
-        </is>
-      </c>
+          <t>Short Term Return Performance Score</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr"/>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>How many standard deviations the fund's Yahoo Sharpe is above (+) or below (-) the average of all funds with the same Yahoo Subsector.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1W 5%, Total Return 1M 16%, Total Return 2M 16%, Total Return QTD 16%, Total Return 3M 16%, Total Return 6M 13%, Total Return 9M 11%, Total Return YTD 5%.</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Z = (fund Sharpe - mean Sharpe of its sub-sector) / std of Sharpe in its sub-sector; 0 if the sub-sector has no spread</t>
+          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
         </is>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>Peer group = Yahoo Subsector (not Morningstar Category), so a bond fund labelled 'Broad Market Equity' is compared with stock funds. Read 1Y and 3Y together: both &gt;= +1 = Core (long-term leader still leading); 1Y &gt;= +1 but 3Y &lt; 0 = Momentum (recent surge, tactical trade, not an anchor); 1Y &lt; 0 but 3Y &gt;= +1 = Value (strong record in a temporary slump, possible buy-the-dip). List them with: python db_access/query.py zscore_matrix</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Recent momentum - changes quickly.</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -4677,7 +4689,7 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT); 1Y: YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr"/>
@@ -4687,24 +4699,28 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Fetch Error</t>
+          <t>Risk Adjusted Score</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr"/>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Message when Yahoo returned no data for the fund.</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr"/>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Morningstar Sharpe 1Y 5%, Morningstar Sharpe 3Y 20%, Morningstar Sharpe 5Y 15%, Morningstar Sharpe 10Y 10%, Upside Capture 3Y 10%, Downside Capture 3Y 10% (inverted), Downside Capture 5Y 5% (inverted), Downside Capture 10Y 5% (inverted), Yahoo Sharpe 1Y 5%, Yahoo Sharpe 3Y 5%, Z Score 1Y 5%, Z Score 3Y 5%.</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
+        </is>
+      </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Blank</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>Funds with no Yahoo prices are moved to the 'No Yahoo Data' tab.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Missing Yahoo values drop out instead of counting as 0.</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -4714,7 +4730,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr"/>
@@ -4724,28 +4740,28 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Data Suspect</t>
+          <t>Volatility Score</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr"/>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is older than 3 years (per Morningstar) but has no Yahoo 3Y Sharpe / Z-score.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Standard Deviation 3Y 20% (inverted), Standard Deviation 5Y 15% (inverted), Standard Deviation 10Y 5% (inverted), Max Drawdown 3Y 20%, Max Drawdown 5Y 25%, Max Drawdown 10Y 15%.</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Inception Date ≤ today - 3 years AND (Sharpe 3Y or Z Score 3Y blank)</t>
+          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>Usually an ETF converted from an older mutual fund (Yahoo only has the new ticker's prices).</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Blank for funds younger than 3 years. Max drawdown is negative, so it is NOT inverted: closer to 0 scores higher.</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -4755,7 +4771,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr"/>
@@ -4765,13 +4781,13 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>Long Term Return Performance Score</t>
+          <t>Resilience Score</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr"/>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1Y 3%, Total Return 2Y 4%, Total Return 3Y 8%, Total Return 4Y 8%, Total Return 5Y 15%, Total Return 6Y 7%, Total Return 7Y 7%, Total Return 8Y 7%, Total Return 9Y 7%, Total Return 10Y 15%, Total Return 15Y 12%, Total Return 20Y 7%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Yearly Beat % 25%, Yearly Bottom 10% Count / Yearly Periods With Data 15% (inverted), Volatile Beat % 25%, Volatile Bottom 10% Count / Volatile Periods With Data 15% (inverted), Worst Three Month Return 20%.</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -4786,7 +4802,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Missing periods (young funds) are skipped, not counted as 0.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. How consistently the fund beat the indexes: calendar years and the S&amp;P 500's volatile periods (crashes and recoveries). Bottom-10% counts are divided by the periods the fund has data for, so older funds aren't penalized for having more periods.</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -4796,7 +4812,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr"/>
@@ -4806,13 +4822,13 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>Short Term Return Performance Score</t>
+          <t>Tracking Score</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr"/>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Total Return 1W 5%, Total Return 1M 16%, Total Return 2M 16%, Total Return QTD 16%, Total Return 3M 16%, Total Return 6M 13%, Total Return 9M 11%, Total Return YTD 5%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tracking Error 3Y 55% (inverted), Tracking Error 1Y 45% (inverted).</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -4827,7 +4843,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Recent momentum - changes quickly.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Good for index funds; for active funds low tracking error just means 'close to the index'.</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -4847,13 +4863,13 @@
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>Risk Adjusted Score</t>
+          <t>Liquidity Size Score</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr"/>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Morningstar Sharpe 1Y 5%, Morningstar Sharpe 3Y 20%, Morningstar Sharpe 5Y 15%, Morningstar Sharpe 10Y 10%, Upside Capture 3Y 10%, Downside Capture 3Y 10% (inverted), Downside Capture 5Y 5% (inverted), Downside Capture 10Y 5% (inverted), Yahoo Sharpe 1Y 5%, Yahoo Sharpe 3Y 5%, Z Score 1Y 5%, Z Score 3Y 5%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Fund Size with fixed cutoffs ($10M → 0, $500M target, $5B → 100) 100%.</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -4868,7 +4884,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Missing Yahoo values drop out instead of counting as 0.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Not within category.</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -4878,7 +4894,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr"/>
@@ -4888,13 +4904,13 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>Volatility Score</t>
+          <t>Quality Valuation Score</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr"/>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Standard Deviation 3Y 20% (inverted), Standard Deviation 5Y 15% (inverted), Standard Deviation 10Y 5% (inverted), Max Drawdown 3Y 20%, Max Drawdown 5Y 25%, Max Drawdown 10Y 15%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Growth Grade 20%, Financial Health 15%, Profitability 15%, Price/Fair Value 15% (inverted), Medalist 15%, Star rating 15%, Wide moat 5%.</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -4909,7 +4925,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Blank for funds younger than 3 years. Max drawdown is negative, so it is NOT inverted: closer to 0 scores higher.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Mostly equity data; bond funds rely on Medalist and stars.</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -4919,7 +4935,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr"/>
@@ -4929,13 +4945,13 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>Resilience Score</t>
+          <t>Costs Score</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr"/>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Yearly Beat % 25%, Yearly Bottom 10% Count / Yearly Periods With Data 15% (inverted), Volatile Beat % 25%, Volatile Bottom 10% Count / Volatile Periods With Data 15% (inverted), Worst Three Month Return 20%.</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Adjusted Expense Ratio 100% (inverted).</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -4950,7 +4966,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. How consistently the fund beat the indexes: calendar years and the S&amp;P 500's volatile periods (crashes and recoveries). Bottom-10% counts are divided by the periods the fund has data for, so older funds aren't penalized for having more periods.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type.</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -4970,13 +4986,13 @@
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>Tracking Score</t>
+          <t>Tax Income Score</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr"/>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tracking Error 3Y 55% (inverted), Tracking Error 1Y 45% (inverted).</t>
+          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tax Cost Ratio 1Y 29% (inverted), Tax Cost Ratio 2Y 21% (inverted), Dividend per Share (Trailing) 14%, SEC 30-Day Yield 36%.</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -4991,7 +5007,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Good for index funds; for active funds low tracking error just means 'close to the index'.</t>
+          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type.</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -5001,7 +5017,7 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
+          <t>No - 0 weight in Profile LT</t>
         </is>
       </c>
       <c r="I95" s="2" t="inlineStr"/>
@@ -5011,28 +5027,24 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Liquidity Size Score</t>
+          <t>Flag Leveraged Fund</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr"/>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Fund Size with fixed cutoffs ($10M → 0, $500M target, $5B → 100) 100%.</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
-        </is>
-      </c>
+          <t>1 if 'Leveraged Fund' = Yes, else 0.</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr"/>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Not within category.</t>
+          <t>Helper for the structural filters.</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -5042,7 +5054,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I96" s="2" t="inlineStr"/>
@@ -5052,28 +5064,24 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Quality Valuation Score</t>
+          <t>Flag Interval Fund</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr"/>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Growth Grade 20%, Financial Health 15%, Profitability 15%, Price/Fair Value 15% (inverted), Medalist 15%, Star rating 15%, Wide moat 5%.</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
-        </is>
-      </c>
+          <t>1 if 'Interval Fund' = Yes, else 0.</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr"/>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type. Mostly equity data; bond funds rely on Medalist and stars.</t>
+          <t>Helper for the structural filters.</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -5083,7 +5091,7 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr"/>
@@ -5093,28 +5101,24 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Costs Score</t>
+          <t>Flag Fund Of Funds</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr"/>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Adjusted Expense Ratio 100% (inverted).</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="inlineStr">
-        <is>
-          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
-        </is>
-      </c>
+          <t>1 if 'Fund of Funds' = Yes, else 0.</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr"/>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type.</t>
+          <t>Helper for the structural filters.</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -5124,7 +5128,7 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I98" s="2" t="inlineStr"/>
@@ -5134,28 +5138,24 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Tax Income Score</t>
+          <t>Flag Tender Offer</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr"/>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>0-100 concept score from these inputs (YAML weights, divided by their total): Tax Cost Ratio 1Y 29% (inverted), Tax Cost Ratio 2Y 21% (inverted), Dividend per Share (Trailing) 14%, SEC 30-Day Yield 36%.</t>
-        </is>
-      </c>
-      <c r="D99" s="2" t="inlineStr">
-        <is>
-          <t>Each input is turned into a 0-100 percentile rank within the Morningstar Category (score = rank% x 100; for 'lower is better' inputs score = 100 - rank% x 100), then score = Σ(weight x input score) / Σ(weights of inputs the fund has).</t>
-        </is>
-      </c>
+          <t>1 if 'Tender offer' = Yes, else 0.</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr"/>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Scored as a percentile rank WITHIN the fund's Morningstar Category, so a fund is only compared with funds of the same type.</t>
+          <t>Helper for the structural filters.</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -5165,7 +5165,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>No - 0 weight in Profile LT</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I99" s="2" t="inlineStr"/>
@@ -10756,7 +10756,7 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>No (used as the max_expense_ratio filter)</t>
+          <t>No (Costs uses Adjusted Expense Ratio)</t>
         </is>
       </c>
     </row>
@@ -12423,7 +12423,7 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -12456,7 +12456,7 @@
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -12621,7 +12621,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>No (optional filter)</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -12859,7 +12859,7 @@
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>Flag Leveraged Fund</t>
+          <t>Yahoo Subsector</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -12869,30 +12869,30 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Flag Leveraged Fund</t>
+          <t>Yahoo Subsector</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr"/>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>n/a (grouping)</t>
         </is>
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Yahoo Finance (calculated by screener)</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Used as peer group for Z Score</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
         <is>
-          <t>Flag Interval Fund</t>
+          <t>Sharpe 1y</t>
         </is>
       </c>
       <c r="B201" s="2" t="inlineStr">
@@ -12902,30 +12902,34 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>Flag Interval Fund</t>
-        </is>
-      </c>
-      <c r="D201" s="2" t="inlineStr"/>
+          <t>Sharpe</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>1Y</t>
+        </is>
+      </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
         </is>
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Yahoo Finance (calculated by screener)</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
         <is>
-          <t>Flag Fund Of Funds</t>
+          <t>Sharpe 3y</t>
         </is>
       </c>
       <c r="B202" s="2" t="inlineStr">
@@ -12935,30 +12939,34 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>Flag Fund Of Funds</t>
-        </is>
-      </c>
-      <c r="D202" s="2" t="inlineStr"/>
+          <t>Sharpe</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Yahoo Finance (calculated by screener)</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
         <is>
-          <t>Flag Tender Offer</t>
+          <t>Z Score 1y</t>
         </is>
       </c>
       <c r="B203" s="2" t="inlineStr">
@@ -12968,13 +12976,17 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>Flag Tender Offer</t>
-        </is>
-      </c>
-      <c r="D203" s="2" t="inlineStr"/>
+          <t>Z Score</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>1Y</t>
+        </is>
+      </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
         </is>
       </c>
       <c r="F203" s="2" t="inlineStr">
@@ -12984,14 +12996,14 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Subsector</t>
+          <t>Z Score 3y</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
@@ -13001,30 +13013,34 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Subsector</t>
-        </is>
-      </c>
-      <c r="D204" s="2" t="inlineStr"/>
+          <t>Z Score</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>3Y</t>
+        </is>
+      </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>n/a (grouping)</t>
+          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
         </is>
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance (calculated by screener)</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>Used as peer group for Z Score</t>
+          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>Sharpe 1y</t>
+          <t>Yahoo Fetch Error</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
@@ -13034,34 +13050,30 @@
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Sharpe</t>
-        </is>
-      </c>
-      <c r="D205" s="2" t="inlineStr">
-        <is>
-          <t>1Y</t>
-        </is>
-      </c>
+          <t>Yahoo Fetch Error</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr"/>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
+          <t>Blank</t>
         </is>
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance (calculated by screener)</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>Sharpe 3y</t>
+          <t>Yahoo Data Suspect</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
@@ -13071,34 +13083,30 @@
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>Sharpe</t>
-        </is>
-      </c>
-      <c r="D206" s="2" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
+          <t>Yahoo Data Suspect</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr"/>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; 1 good, &lt; 0 = worse than cash)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Finance (calculated by screener)</t>
+          <t>Screener (calculated)</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>Z Score 1y</t>
+          <t>Long Term Return Performance Score</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
@@ -13108,17 +13116,13 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Z Score</t>
-        </is>
-      </c>
-      <c r="D207" s="2" t="inlineStr">
-        <is>
-          <t>1Y</t>
-        </is>
-      </c>
+          <t>Long Term Return Performance Score</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr"/>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F207" s="2" t="inlineStr">
@@ -13128,14 +13132,14 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
+          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>Z Score 3y</t>
+          <t>Short Term Return Performance Score</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
@@ -13145,17 +13149,13 @@
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>Z Score</t>
-        </is>
-      </c>
-      <c r="D208" s="2" t="inlineStr">
-        <is>
-          <t>3Y</t>
-        </is>
-      </c>
+          <t>Short Term Return Performance Score</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr"/>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (&gt; +1 clearly above peers, &lt; -1 clearly below)</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F208" s="2" t="inlineStr">
@@ -13165,14 +13165,14 @@
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 5% of Risk-adjusted (≈1.0% of Profile LT). Risk-adjusted = 19.0% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Fetch Error</t>
+          <t>Risk Adjusted Score</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
@@ -13182,13 +13182,13 @@
       </c>
       <c r="C209" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Fetch Error</t>
+          <t>Risk Adjusted Score</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr"/>
       <c r="E209" s="2" t="inlineStr">
         <is>
-          <t>Blank</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F209" s="2" t="inlineStr">
@@ -13198,14 +13198,14 @@
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Data Suspect</t>
+          <t>Volatility Score</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
@@ -13215,13 +13215,13 @@
       </c>
       <c r="C210" s="2" t="inlineStr">
         <is>
-          <t>Yahoo Data Suspect</t>
+          <t>Volatility Score</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr"/>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Higher is better (100 = best in category)</t>
         </is>
       </c>
       <c r="F210" s="2" t="inlineStr">
@@ -13231,14 +13231,14 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
         <is>
-          <t>Long Term Return Performance Score</t>
+          <t>Resilience Score</t>
         </is>
       </c>
       <c r="B211" s="2" t="inlineStr">
@@ -13248,7 +13248,7 @@
       </c>
       <c r="C211" s="2" t="inlineStr">
         <is>
-          <t>Long Term Return Performance Score</t>
+          <t>Resilience Score</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr"/>
@@ -13264,14 +13264,14 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
         <is>
-          <t>Short Term Return Performance Score</t>
+          <t>Tracking Score</t>
         </is>
       </c>
       <c r="B212" s="2" t="inlineStr">
@@ -13281,7 +13281,7 @@
       </c>
       <c r="C212" s="2" t="inlineStr">
         <is>
-          <t>Short Term Return Performance Score</t>
+          <t>Tracking Score</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr"/>
@@ -13304,7 +13304,7 @@
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
         <is>
-          <t>Risk Adjusted Score</t>
+          <t>Liquidity Size Score</t>
         </is>
       </c>
       <c r="B213" s="2" t="inlineStr">
@@ -13314,7 +13314,7 @@
       </c>
       <c r="C213" s="2" t="inlineStr">
         <is>
-          <t>Risk Adjusted Score</t>
+          <t>Liquidity Size Score</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr"/>
@@ -13330,14 +13330,14 @@
       </c>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 19.0% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
         <is>
-          <t>Volatility Score</t>
+          <t>Quality Valuation Score</t>
         </is>
       </c>
       <c r="B214" s="2" t="inlineStr">
@@ -13347,7 +13347,7 @@
       </c>
       <c r="C214" s="2" t="inlineStr">
         <is>
-          <t>Volatility Score</t>
+          <t>Quality Valuation Score</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr"/>
@@ -13363,14 +13363,14 @@
       </c>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
         <is>
-          <t>Resilience Score</t>
+          <t>Costs Score</t>
         </is>
       </c>
       <c r="B215" s="2" t="inlineStr">
@@ -13380,7 +13380,7 @@
       </c>
       <c r="C215" s="2" t="inlineStr">
         <is>
-          <t>Resilience Score</t>
+          <t>Costs Score</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr"/>
@@ -13403,7 +13403,7 @@
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
         <is>
-          <t>Tracking Score</t>
+          <t>Tax Income Score</t>
         </is>
       </c>
       <c r="B216" s="2" t="inlineStr">
@@ -13413,7 +13413,7 @@
       </c>
       <c r="C216" s="2" t="inlineStr">
         <is>
-          <t>Tracking Score</t>
+          <t>Tax Income Score</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr"/>
@@ -13429,14 +13429,14 @@
       </c>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
+          <t>No - 0 weight in Profile LT</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Liquidity Size Score</t>
+          <t>Flag Leveraged Fund</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -13446,13 +13446,13 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>Liquidity Size Score</t>
+          <t>Flag Leveraged Fund</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr"/>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F217" s="2" t="inlineStr">
@@ -13462,14 +13462,14 @@
       </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Quality Valuation Score</t>
+          <t>Flag Interval Fund</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -13479,13 +13479,13 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Quality Valuation Score</t>
+          <t>Flag Interval Fund</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr"/>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
@@ -13495,14 +13495,14 @@
       </c>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Costs Score</t>
+          <t>Flag Fund Of Funds</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -13512,13 +13512,13 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>Costs Score</t>
+          <t>Flag Fund Of Funds</t>
         </is>
       </c>
       <c r="D219" s="2" t="inlineStr"/>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F219" s="2" t="inlineStr">
@@ -13528,14 +13528,14 @@
       </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Tax Income Score</t>
+          <t>Flag Tender Offer</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -13545,13 +13545,13 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Tax Income Score</t>
+          <t>Flag Tender Offer</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr"/>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>Higher is better (100 = best in category)</t>
+          <t>0 (except Fund Of Funds: neutral)</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
@@ -13561,7 +13561,7 @@
       </c>
       <c r="G220" s="2" t="inlineStr">
         <is>
-          <t>No - 0 weight in Profile LT</t>
+          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove Selected and structure flag columns; alert on rank cutoffs
- Report: drop Flag Leveraged Fund / Interval Fund / Fund Of Funds / Tender
  Offer and every Profile <key> Selected (Overall) Flag; each profile adds only
  Score, Rank In Category and Rank Overall
- Remove top_n_per_category / top_n_overall from the YAMLs, loader, scorer,
  run recorder and used-weights report, plus the empty flag placeholders
- alerts.py: ALERT_RULES rank cutoffs (LT #1 in category and top 100 overall,
  ST #1 in category and top 50 overall)
- main.py summary prints the top funds by overall rank; top_both and
  ticker_history queries, compare_results.py, dictionary and docs use ranks

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/etf_screener/docs/report_column_dictionary.xlsx
+++ b/etf_screener/docs/report_column_dictionary.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sectors" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$251</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Column Dictionary'!$A$1:$K$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All Report Columns'!$A$1:$G$243</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Scoring Concepts'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Volatile Periods'!$A$1:$H$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Sectors'!$A$1:$D$12</definedName>
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K112"/>
+  <dimension ref="A1:K104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -969,7 +969,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Yes - 1W: YAML weight 0.05 = 5% of Short-term Return (≈0.3% of Profile LT); 1M: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); 2M: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); QTD: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); 3M: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); 6M: YAML weight 0.12 = 13% of Short-term Return (≈0.6% of Profile LT); 9M: YAML weight 0.1 = 11% of Short-term Return (≈0.5% of Profile LT); YTD: YAML weight 0.05 = 5% of Short-term Return (≈0.3% of Profile LT). Short-term Return = 4.8% of Profile LT  |  Yes - 1Y: YAML weight 0.03 = 3% of Long-term Return (≈0.7% of Profile LT); 2Y: YAML weight 0.04 = 4% of Long-term Return (≈1.0% of Profile LT); 3Y: YAML weight 0.08 = 8% of Long-term Return (≈1.9% of Profile LT); 4Y: YAML weight 0.08 = 8% of Long-term Return (≈1.9% of Profile LT); 5Y: YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile LT); 6Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT); 7Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT); 8Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT); 9Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT); 10Y: YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile LT); 15Y: YAML weight 0.12 = 12% of Long-term Return (≈2.9% of Profile LT); 20Y: YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - 1W: YAML weight 0.05 = 5% of Short-term Return (≈0.3% of Profile LT); 1M: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); 2M: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); QTD: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); 3M: YAML weight 0.15 = 16% of Short-term Return (≈0.8% of Profile LT); 6M: YAML weight 0.12 = 13% of Short-term Return (≈0.6% of Profile LT); 9M: YAML weight 0.1 = 11% of Short-term Return (≈0.5% of Profile LT); YTD: YAML weight 0.05 = 5% of Short-term Return (≈0.3% of Profile LT). Short-term Return = 4.8% of Profile LT  |  Yes - 1Y: YAML weight 0.03 = 3% of Long-term Return (≈0.9% of Profile LT); 2Y: YAML weight 0.04 = 4% of Long-term Return (≈1.1% of Profile LT); 3Y: YAML weight 0.08 = 8% of Long-term Return (≈2.3% of Profile LT); 4Y: YAML weight 0.08 = 8% of Long-term Return (≈2.3% of Profile LT); 5Y: YAML weight 0.15 = 15% of Long-term Return (≈4.3% of Profile LT); 6Y: YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT); 7Y: YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT); 8Y: YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT); 9Y: YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT); 10Y: YAML weight 0.15 = 15% of Long-term Return (≈4.3% of Profile LT); 15Y: YAML weight 0.12 = 12% of Long-term Return (≈3.4% of Profile LT); 20Y: YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈2.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈3.6% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈1.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈2.1% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
@@ -1612,7 +1612,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈2.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈3.6% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈1.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈2.1% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr"/>
@@ -1882,7 +1882,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.2 = 20% of Volatility (≈2.9% of Profile LT); 5Y: YAML weight 0.15 = 15% of Volatility (≈2.1% of Profile LT); 10Y: YAML weight 0.05 = 5% of Volatility (≈0.7% of Profile LT). Volatility = 14.3% of Profile LT</t>
+          <t>Yes - 3Y: YAML weight 0.2 = 20% of Volatility (≈1.9% of Profile LT); 5Y: YAML weight 0.15 = 15% of Volatility (≈1.4% of Profile LT); 10Y: YAML weight 0.05 = 5% of Volatility (≈0.5% of Profile LT). Volatility = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 20% of Resilience (≈1.9% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.2 = 20% of Resilience (≈2.9% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2208,7 +2208,7 @@
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>Yes - 3Y: YAML weight 0.2 = 20% of Volatility (≈2.9% of Profile LT); 5Y: YAML weight 0.25 = 25% of Volatility (≈3.6% of Profile LT); 10Y: YAML weight 0.15 = 15% of Volatility (≈2.1% of Profile LT). Volatility = 14.3% of Profile LT</t>
+          <t>Yes - 3Y: YAML weight 0.2 = 20% of Volatility (≈1.9% of Profile LT); 5Y: YAML weight 0.25 = 25% of Volatility (≈2.4% of Profile LT); 10Y: YAML weight 0.15 = 15% of Volatility (≈1.4% of Profile LT). Volatility = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 1 = 100% of Costs (≈9.5% of Profile LT). Costs = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 1 = 100% of Costs (≈4.8% of Profile LT). Costs = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -4648,7 +4648,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.3 = 28.6% of Profile LT</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr"/>
@@ -4771,7 +4771,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr"/>
@@ -4812,7 +4812,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr"/>
@@ -4976,7 +4976,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr"/>
@@ -5027,24 +5027,32 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>Flag Leveraged Fund</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr"/>
+          <t>Return Rank</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>1W, 1M, 2M, QTD, 3M, 6M, 9M, YTD, 1Y, 2Y, 3Y, 4Y, 5Y, 6Y, 7Y, 8Y, 9Y, 10Y, 15Y, 20Y</t>
+        </is>
+      </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Leveraged Fund' = Yes, else 0.</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr"/>
+          <t>Rank of the matching 'Total Return' column across ALL funds in the report (1 = highest return).</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>Rank = position when all funds are sorted by that period's return, highest first (ties share the lowest rank)</t>
+        </is>
+      </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Lower is better (1 = best)</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>Helper for the structural filters.</t>
+          <t>Across all categories, not within category - leveraged / sector funds dominate both ends. For momentum lists use python db_access/query.py momentum_top / momentum_bottom.</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -5064,24 +5072,28 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>Flag Interval Fund</t>
+          <t>Profile LT Score</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr"/>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Interval Fund' = Yes, else 0.</t>
-        </is>
-      </c>
-      <c r="D97" s="2" t="inlineStr"/>
+          <t>Final 0-100 score combining the concept scores with the weights in profile_long_term.yaml.</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Profile LT Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Long-term Return 0.3, Short-term Return 0.05, Risk-adjusted 0.2, Volatility 0.1, Resilience 0.15, Tracking 0.05, Liquidity/Size 0.05, Quality/Valuation 0.1, Costs 0.05, Tax/Income 0 (sum 1.05, so each effective share = weight / 1.05)</t>
+        </is>
+      </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>Helper for the structural filters.</t>
+          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'.</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -5091,7 +5103,7 @@
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>This IS the Profile LT score</t>
         </is>
       </c>
       <c r="I97" s="2" t="inlineStr"/>
@@ -5101,24 +5113,24 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>Flag Fund Of Funds</t>
+          <t>Profile LT Rank In Category</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr"/>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Fund of Funds' = Yes, else 0.</t>
+          <t>Rank of the Profile LT Score within the fund's Morningstar Category (1 = best).</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr"/>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>Helper for the structural filters.</t>
+          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -5138,24 +5150,24 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>Flag Tender Offer</t>
+          <t>Profile LT Rank Overall</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr"/>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>1 if 'Tender offer' = Yes, else 0.</t>
+          <t>Rank of the Profile LT Score across all funds (1 = best).</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr"/>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>Helper for the structural filters.</t>
+          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -5175,32 +5187,28 @@
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>Return Rank</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>1W, 1M, 2M, QTD, 3M, 6M, 9M, YTD, 1Y, 2Y, 3Y, 4Y, 5Y, 6Y, 7Y, 8Y, 9Y, 10Y, 15Y, 20Y</t>
-        </is>
-      </c>
+          <t>Profile ST Score</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr"/>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Rank of the matching 'Total Return' column across ALL funds in the report (1 = highest return).</t>
+          <t>Final 0-100 score combining the concept scores with the weights in profile_short_term.yaml.</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Rank = position when all funds are sorted by that period's return, highest first (ties share the lowest rank)</t>
+          <t>Profile ST Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Short-term Return 0.4, Risk-adjusted 0.2, Volatility 0.1, Resilience 0, Liquidity/Size 0.1, Costs 0.1, Long-term Return 0.05, Quality/Valuation 0.05, Tracking 0, Tax/Income 0 (sum 1, so each effective share = weight / 1)</t>
         </is>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (1 = best)</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>Across all categories, not within category - leveraged / sector funds dominate both ends. For momentum lists use python db_access/query.py momentum_top / momentum_bottom.</t>
+          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'. Uses ST's own concept weights, so it can't be recomputed from the concept score columns in this report (those use LT's). Blank for funds profile_short_term.yaml filters out.</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -5210,7 +5218,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - this is the Profile ST score</t>
         </is>
       </c>
       <c r="I100" s="2" t="inlineStr"/>
@@ -5220,28 +5228,24 @@
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Score</t>
+          <t>Profile ST Rank In Category</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr"/>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Final 0-100 score combining the concept scores with the weights in profile_long_term.yaml.</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>Profile LT Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Long-term Return 0.25, Short-term Return 0.05, Risk-adjusted 0.2, Volatility 0.15, Resilience 0.1, Tracking 0.05, Liquidity/Size 0.05, Quality/Valuation 0.1, Costs 0.1, Tax/Income 0 (sum 1.05, so each effective share = weight / 1.05)</t>
-        </is>
-      </c>
+          <t>Rank of the Profile ST Score within the fund's Morningstar Category (1 = best).</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr"/>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Higher is better</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'.</t>
+          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -5251,7 +5255,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>This IS the Profile LT score</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I101" s="2" t="inlineStr"/>
@@ -5261,13 +5265,13 @@
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank In Category</t>
+          <t>Profile ST Rank Overall</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr"/>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Rank of the Profile LT Score within the fund's Morningstar Category (1 = best).</t>
+          <t>Rank of the Profile ST Score across all funds (1 = best).</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr"/>
@@ -5278,7 +5282,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
+          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -5298,28 +5302,24 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Selected Flag</t>
+          <t>Missing From Yahoo</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr"/>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>1 if the fund is in the top 5 of its Morningstar Category by Profile LT Score.</t>
-        </is>
-      </c>
-      <c r="D103" s="2" t="inlineStr">
-        <is>
-          <t>Rank In Category ≤ top_n_per_category (5)</t>
-        </is>
-      </c>
+          <t>('No Yahoo Data' tab only) Which Yahoo-based results are missing: Sharpe / Z-score, yearly returns, volatile periods.</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr"/>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>top_n_per_category is set in profile_long_term.yaml.</t>
+          <t>These funds are taken off the overview; all their Morningstar columns are still on that tab.</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -5339,370 +5339,58 @@
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank Overall</t>
+          <t>Trading Volume</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr"/>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Rank of the Profile LT Score across all funds (1 = best).</t>
-        </is>
-      </c>
-      <c r="D104" s="2" t="inlineStr"/>
+          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window.</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Reported directly from exchange data</t>
+        </is>
+      </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>Lower is better</t>
+          <t>Higher = easier to trade at a fair price</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
+          <t>Not in the current eTrade export. The YAML still gives it weight 0.4 in Liquidity/Size; since the column is missing, Fund Size gets the whole Liquidity/Size weight. Add it to the export to use it.</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Screener (calculated)</t>
+          <t>Morningstar (not in current data)</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I104" s="2" t="inlineStr"/>
-      <c r="J104" s="2" t="inlineStr"/>
-      <c r="K104" s="2" t="inlineStr"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>Profile LT Selected Overall Flag</t>
-        </is>
-      </c>
-      <c r="B105" s="2" t="inlineStr"/>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>1 if the fund is in the top 100 overall.</t>
-        </is>
-      </c>
-      <c r="D105" s="2" t="inlineStr">
-        <is>
-          <t>Rank Overall ≤ top_n_overall (100)</t>
-        </is>
-      </c>
-      <c r="E105" s="2" t="inlineStr">
-        <is>
-          <t>1 = selected</t>
-        </is>
-      </c>
-      <c r="F105" s="2" t="inlineStr">
-        <is>
-          <t>top_n_overall is set in profile_long_term.yaml (if left out, top_n_per_category is used).</t>
-        </is>
-      </c>
-      <c r="G105" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="H105" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I105" s="2" t="inlineStr"/>
-      <c r="J105" s="2" t="inlineStr"/>
-      <c r="K105" s="2" t="inlineStr"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Score</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="inlineStr"/>
-      <c r="C106" s="2" t="inlineStr">
-        <is>
-          <t>Final 0-100 score combining the concept scores with the weights in profile_short_term.yaml.</t>
-        </is>
-      </c>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Score = Σ(concept weight x concept score) / Σ(weights of concept scores the fund has). YAML weights: Short-term Return 0.4, Risk-adjusted 0.2, Volatility 0.1, Resilience 0, Liquidity/Size 0.1, Costs 0.1, Long-term Return 0.05, Quality/Valuation 0.05, Tracking 0, Tax/Income 0 (sum 1, so each effective share = weight / 1)</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>Higher is better</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>Blank concept scores (e.g. Volatility for young funds) are left out and the rest re-weighted. Because inputs are ranked within category, the score means 'good for its category', not 'better than every other fund'. Uses ST's own concept weights, so it can't be recomputed from the concept score columns in this report (those use LT's). Blank for funds profile_short_term.yaml filters out.</t>
-        </is>
-      </c>
-      <c r="G106" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="H106" s="2" t="inlineStr">
-        <is>
-          <t>No - this is the Profile ST score</t>
-        </is>
-      </c>
-      <c r="I106" s="2" t="inlineStr"/>
-      <c r="J106" s="2" t="inlineStr"/>
-      <c r="K106" s="2" t="inlineStr"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Rank In Category</t>
-        </is>
-      </c>
-      <c r="B107" s="2" t="inlineStr"/>
-      <c r="C107" s="2" t="inlineStr">
-        <is>
-          <t>Rank of the Profile ST Score within the fund's Morningstar Category (1 = best).</t>
-        </is>
-      </c>
-      <c r="D107" s="2" t="inlineStr"/>
-      <c r="E107" s="2" t="inlineStr">
-        <is>
-          <t>Lower is better</t>
-        </is>
-      </c>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>Read with the category size: 5th of 8 is mediocre, 5th of 400 is excellent. The highest numbers are the category's weakest funds for this profile.</t>
-        </is>
-      </c>
-      <c r="G107" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="H107" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I107" s="2" t="inlineStr"/>
-      <c r="J107" s="2" t="inlineStr"/>
-      <c r="K107" s="2" t="inlineStr"/>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Selected Flag</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr"/>
-      <c r="C108" s="2" t="inlineStr">
-        <is>
-          <t>1 if the fund is in the top 5 of its Morningstar Category by Profile ST Score.</t>
-        </is>
-      </c>
-      <c r="D108" s="2" t="inlineStr">
-        <is>
-          <t>Rank In Category ≤ top_n_per_category (5)</t>
-        </is>
-      </c>
-      <c r="E108" s="2" t="inlineStr">
-        <is>
-          <t>1 = selected</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>top_n_per_category is set in profile_short_term.yaml.</t>
-        </is>
-      </c>
-      <c r="G108" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="H108" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I108" s="2" t="inlineStr"/>
-      <c r="J108" s="2" t="inlineStr"/>
-      <c r="K108" s="2" t="inlineStr"/>
-    </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Rank Overall</t>
-        </is>
-      </c>
-      <c r="B109" s="2" t="inlineStr"/>
-      <c r="C109" s="2" t="inlineStr">
-        <is>
-          <t>Rank of the Profile ST Score across all funds (1 = best).</t>
-        </is>
-      </c>
-      <c r="D109" s="2" t="inlineStr"/>
-      <c r="E109" s="2" t="inlineStr">
-        <is>
-          <t>Lower is better</t>
-        </is>
-      </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>Mixes categories; a top bond fund and a top stock fund can both rank high.</t>
-        </is>
-      </c>
-      <c r="G109" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="H109" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I109" s="2" t="inlineStr"/>
-      <c r="J109" s="2" t="inlineStr"/>
-      <c r="K109" s="2" t="inlineStr"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Selected Overall Flag</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr"/>
-      <c r="C110" s="2" t="inlineStr">
-        <is>
-          <t>1 if the fund is in the top 25 overall.</t>
-        </is>
-      </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>Rank Overall ≤ top_n_overall (25)</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>1 = selected</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>top_n_overall is set in profile_short_term.yaml (if left out, top_n_per_category is used).</t>
-        </is>
-      </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="H110" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I110" s="2" t="inlineStr"/>
-      <c r="J110" s="2" t="inlineStr"/>
-      <c r="K110" s="2" t="inlineStr"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>Missing From Yahoo</t>
-        </is>
-      </c>
-      <c r="B111" s="2" t="inlineStr"/>
-      <c r="C111" s="2" t="inlineStr">
-        <is>
-          <t>('No Yahoo Data' tab only) Which Yahoo-based results are missing: Sharpe / Z-score, yearly returns, volatile periods.</t>
-        </is>
-      </c>
-      <c r="D111" s="2" t="inlineStr"/>
-      <c r="E111" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F111" s="2" t="inlineStr">
-        <is>
-          <t>These funds are taken off the overview; all their Morningstar columns are still on that tab.</t>
-        </is>
-      </c>
-      <c r="G111" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="H111" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I111" s="2" t="inlineStr"/>
-      <c r="J111" s="2" t="inlineStr"/>
-      <c r="K111" s="2" t="inlineStr"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>Trading Volume</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr"/>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window.</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>Reported directly from exchange data</t>
-        </is>
-      </c>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>Higher = easier to trade at a fair price</t>
-        </is>
-      </c>
-      <c r="F112" s="2" t="inlineStr">
-        <is>
-          <t>Not in the current eTrade export. The YAML still gives it weight 0.4 in Liquidity/Size; since the column is missing, Fund Size gets the whole Liquidity/Size weight. Add it to the export to use it.</t>
-        </is>
-      </c>
-      <c r="G112" s="2" t="inlineStr">
-        <is>
-          <t>Morningstar (not in current data)</t>
-        </is>
-      </c>
-      <c r="H112" s="2" t="inlineStr">
-        <is>
           <t>No effect: weighted 0.4 in the YAML, but the column is missing</t>
         </is>
       </c>
-      <c r="I112" s="2" t="inlineStr">
+      <c r="I104" s="2" t="inlineStr">
         <is>
           <t>Morningstar's ETF 'Volume' is the number of shares traded on the current (most recent) trading day; 'Average Daily Volume' is a separate data point averaging daily volume over a trailing window. Key facts: Unit is shares, not dollars. Single-day volume and average volume are distinct fields; which one an export column holds depends on the data point chosen.</t>
         </is>
       </c>
-      <c r="J112" s="2" t="inlineStr">
+      <c r="J104" s="2" t="inlineStr">
         <is>
           <t>Corrected to Morningstar's definition</t>
         </is>
       </c>
-      <c r="K112" s="2" t="inlineStr">
+      <c r="K104" s="2" t="inlineStr">
         <is>
           <t>http://quote.morningstar.com/ETFdefinition.html</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K112"/>
+  <autoFilter ref="A1:K104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5713,7 +5401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G251"/>
+  <dimension ref="A1:G243"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -6388,7 +6076,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.03 = 3% of Long-term Return (≈0.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.03 = 3% of Long-term Return (≈0.9% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6425,7 +6113,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.04 = 4% of Long-term Return (≈1.0% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.04 = 4% of Long-term Return (≈1.1% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6462,7 +6150,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.08 = 8% of Long-term Return (≈1.9% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.08 = 8% of Long-term Return (≈2.3% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6499,7 +6187,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.08 = 8% of Long-term Return (≈1.9% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.08 = 8% of Long-term Return (≈2.3% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6536,7 +6224,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.15 = 15% of Long-term Return (≈4.3% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6573,7 +6261,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6610,7 +6298,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6647,7 +6335,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6684,7 +6372,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6721,7 +6409,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Long-term Return (≈3.6% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.15 = 15% of Long-term Return (≈4.3% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6758,7 +6446,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.12 = 12% of Long-term Return (≈2.9% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.12 = 12% of Long-term Return (≈3.4% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -6795,7 +6483,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈1.7% of Profile LT). Long-term Return = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.07 = 7% of Long-term Return (≈2.0% of Profile LT). Long-term Return = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -7334,7 +7022,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈2.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈3.6% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -7766,7 +7454,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈1.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈2.1% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9230,7 +8918,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈2.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.25 = 25% of Resilience (≈3.6% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9662,7 +9350,7 @@
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈1.4% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - As a share of Periods With Data: YAML weight 0.15 = 15% of Resilience (≈2.1% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9884,7 +9572,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 20% of Volatility (≈2.9% of Profile LT). Volatility = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.2 = 20% of Volatility (≈1.9% of Profile LT). Volatility = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9921,7 +9609,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Volatility (≈2.1% of Profile LT). Volatility = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.15 = 15% of Volatility (≈1.4% of Profile LT). Volatility = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9958,7 +9646,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.05 = 5% of Volatility (≈0.7% of Profile LT). Volatility = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 5% of Volatility (≈0.5% of Profile LT). Volatility = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -9991,7 +9679,7 @@
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 20% of Resilience (≈1.9% of Profile LT). Resilience = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.2 = 20% of Resilience (≈2.9% of Profile LT). Resilience = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10542,7 +10230,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.2 = 20% of Volatility (≈2.9% of Profile LT). Volatility = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.2 = 20% of Volatility (≈1.9% of Profile LT). Volatility = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10579,7 +10267,7 @@
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 25% of Volatility (≈3.6% of Profile LT). Volatility = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.25 = 25% of Volatility (≈2.4% of Profile LT). Volatility = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10616,7 +10304,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 15% of Volatility (≈2.1% of Profile LT). Volatility = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.15 = 15% of Volatility (≈1.4% of Profile LT). Volatility = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -10789,7 +10477,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 1 = 100% of Costs (≈9.5% of Profile LT). Costs = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 1 = 100% of Costs (≈4.8% of Profile LT). Costs = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13132,7 +12820,7 @@
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.25 = 23.8% of Profile LT</t>
+          <t>Yes - YAML weight 0.3 = 28.6% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13231,7 +12919,7 @@
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
+          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13264,7 +12952,7 @@
       </c>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.15 = 14.3% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13396,7 +13084,7 @@
       </c>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>Yes - YAML weight 0.1 = 9.5% of Profile LT</t>
+          <t>Yes - YAML weight 0.05 = 4.8% of Profile LT</t>
         </is>
       </c>
     </row>
@@ -13436,7 +13124,7 @@
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
         <is>
-          <t>Flag Leveraged Fund</t>
+          <t>Return Rank (1W)</t>
         </is>
       </c>
       <c r="B217" s="2" t="inlineStr">
@@ -13446,13 +13134,17 @@
       </c>
       <c r="C217" s="2" t="inlineStr">
         <is>
-          <t>Flag Leveraged Fund</t>
-        </is>
-      </c>
-      <c r="D217" s="2" t="inlineStr"/>
+          <t>Return Rank</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>1W</t>
+        </is>
+      </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Lower is better (1 = best)</t>
         </is>
       </c>
       <c r="F217" s="2" t="inlineStr">
@@ -13469,7 +13161,7 @@
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
         <is>
-          <t>Flag Interval Fund</t>
+          <t>Return Rank (1M)</t>
         </is>
       </c>
       <c r="B218" s="2" t="inlineStr">
@@ -13479,13 +13171,17 @@
       </c>
       <c r="C218" s="2" t="inlineStr">
         <is>
-          <t>Flag Interval Fund</t>
-        </is>
-      </c>
-      <c r="D218" s="2" t="inlineStr"/>
+          <t>Return Rank</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>1M</t>
+        </is>
+      </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Lower is better (1 = best)</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
@@ -13502,7 +13198,7 @@
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
         <is>
-          <t>Flag Fund Of Funds</t>
+          <t>Return Rank (2M)</t>
         </is>
       </c>
       <c r="B219" s="2" t="inlineStr">
@@ -13512,13 +13208,17 @@
       </c>
       <c r="C219" s="2" t="inlineStr">
         <is>
-          <t>Flag Fund Of Funds</t>
-        </is>
-      </c>
-      <c r="D219" s="2" t="inlineStr"/>
+          <t>Return Rank</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>2M</t>
+        </is>
+      </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Lower is better (1 = best)</t>
         </is>
       </c>
       <c r="F219" s="2" t="inlineStr">
@@ -13535,7 +13235,7 @@
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
         <is>
-          <t>Flag Tender Offer</t>
+          <t>Return Rank (QTD)</t>
         </is>
       </c>
       <c r="B220" s="2" t="inlineStr">
@@ -13545,13 +13245,17 @@
       </c>
       <c r="C220" s="2" t="inlineStr">
         <is>
-          <t>Flag Tender Offer</t>
-        </is>
-      </c>
-      <c r="D220" s="2" t="inlineStr"/>
+          <t>Return Rank</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>QTD</t>
+        </is>
+      </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>0 (except Fund Of Funds: neutral)</t>
+          <t>Lower is better (1 = best)</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
@@ -13568,7 +13272,7 @@
     <row r="221">
       <c r="A221" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (1W)</t>
+          <t>Return Rank (3M)</t>
         </is>
       </c>
       <c r="B221" s="2" t="inlineStr">
@@ -13583,7 +13287,7 @@
       </c>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>1W</t>
+          <t>3M</t>
         </is>
       </c>
       <c r="E221" s="2" t="inlineStr">
@@ -13605,7 +13309,7 @@
     <row r="222">
       <c r="A222" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (1M)</t>
+          <t>Return Rank (6M)</t>
         </is>
       </c>
       <c r="B222" s="2" t="inlineStr">
@@ -13620,7 +13324,7 @@
       </c>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>6M</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr">
@@ -13642,7 +13346,7 @@
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (2M)</t>
+          <t>Return Rank (9M)</t>
         </is>
       </c>
       <c r="B223" s="2" t="inlineStr">
@@ -13657,7 +13361,7 @@
       </c>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>2M</t>
+          <t>9M</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr">
@@ -13679,7 +13383,7 @@
     <row r="224">
       <c r="A224" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (QTD)</t>
+          <t>Return Rank (YTD)</t>
         </is>
       </c>
       <c r="B224" s="2" t="inlineStr">
@@ -13694,7 +13398,7 @@
       </c>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>QTD</t>
+          <t>YTD</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr">
@@ -13716,7 +13420,7 @@
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (3M)</t>
+          <t>Return Rank (1Y)</t>
         </is>
       </c>
       <c r="B225" s="2" t="inlineStr">
@@ -13731,7 +13435,7 @@
       </c>
       <c r="D225" s="2" t="inlineStr">
         <is>
-          <t>3M</t>
+          <t>1Y</t>
         </is>
       </c>
       <c r="E225" s="2" t="inlineStr">
@@ -13753,7 +13457,7 @@
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (6M)</t>
+          <t>Return Rank (2Y)</t>
         </is>
       </c>
       <c r="B226" s="2" t="inlineStr">
@@ -13768,7 +13472,7 @@
       </c>
       <c r="D226" s="2" t="inlineStr">
         <is>
-          <t>6M</t>
+          <t>2Y</t>
         </is>
       </c>
       <c r="E226" s="2" t="inlineStr">
@@ -13790,7 +13494,7 @@
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (9M)</t>
+          <t>Return Rank (3Y)</t>
         </is>
       </c>
       <c r="B227" s="2" t="inlineStr">
@@ -13805,7 +13509,7 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t>9M</t>
+          <t>3Y</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
@@ -13827,7 +13531,7 @@
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (YTD)</t>
+          <t>Return Rank (4Y)</t>
         </is>
       </c>
       <c r="B228" s="2" t="inlineStr">
@@ -13842,7 +13546,7 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t>YTD</t>
+          <t>4Y</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
@@ -13864,7 +13568,7 @@
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (1Y)</t>
+          <t>Return Rank (5Y)</t>
         </is>
       </c>
       <c r="B229" s="2" t="inlineStr">
@@ -13879,7 +13583,7 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t>1Y</t>
+          <t>5Y</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
@@ -13901,7 +13605,7 @@
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (2Y)</t>
+          <t>Return Rank (6Y)</t>
         </is>
       </c>
       <c r="B230" s="2" t="inlineStr">
@@ -13916,7 +13620,7 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t>2Y</t>
+          <t>6Y</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
@@ -13938,7 +13642,7 @@
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (3Y)</t>
+          <t>Return Rank (7Y)</t>
         </is>
       </c>
       <c r="B231" s="2" t="inlineStr">
@@ -13953,7 +13657,7 @@
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t>3Y</t>
+          <t>7Y</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
@@ -13975,7 +13679,7 @@
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (4Y)</t>
+          <t>Return Rank (8Y)</t>
         </is>
       </c>
       <c r="B232" s="2" t="inlineStr">
@@ -13990,7 +13694,7 @@
       </c>
       <c r="D232" s="2" t="inlineStr">
         <is>
-          <t>4Y</t>
+          <t>8Y</t>
         </is>
       </c>
       <c r="E232" s="2" t="inlineStr">
@@ -14012,7 +13716,7 @@
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (5Y)</t>
+          <t>Return Rank (9Y)</t>
         </is>
       </c>
       <c r="B233" s="2" t="inlineStr">
@@ -14027,7 +13731,7 @@
       </c>
       <c r="D233" s="2" t="inlineStr">
         <is>
-          <t>5Y</t>
+          <t>9Y</t>
         </is>
       </c>
       <c r="E233" s="2" t="inlineStr">
@@ -14049,7 +13753,7 @@
     <row r="234">
       <c r="A234" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (6Y)</t>
+          <t>Return Rank (10Y)</t>
         </is>
       </c>
       <c r="B234" s="2" t="inlineStr">
@@ -14064,7 +13768,7 @@
       </c>
       <c r="D234" s="2" t="inlineStr">
         <is>
-          <t>6Y</t>
+          <t>10Y</t>
         </is>
       </c>
       <c r="E234" s="2" t="inlineStr">
@@ -14086,7 +13790,7 @@
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (7Y)</t>
+          <t>Return Rank (15Y)</t>
         </is>
       </c>
       <c r="B235" s="2" t="inlineStr">
@@ -14101,7 +13805,7 @@
       </c>
       <c r="D235" s="2" t="inlineStr">
         <is>
-          <t>7Y</t>
+          <t>15Y</t>
         </is>
       </c>
       <c r="E235" s="2" t="inlineStr">
@@ -14123,7 +13827,7 @@
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (8Y)</t>
+          <t>Return Rank (20Y)</t>
         </is>
       </c>
       <c r="B236" s="2" t="inlineStr">
@@ -14138,7 +13842,7 @@
       </c>
       <c r="D236" s="2" t="inlineStr">
         <is>
-          <t>8Y</t>
+          <t>20Y</t>
         </is>
       </c>
       <c r="E236" s="2" t="inlineStr">
@@ -14160,7 +13864,7 @@
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (9Y)</t>
+          <t>Profile LT Score</t>
         </is>
       </c>
       <c r="B237" s="2" t="inlineStr">
@@ -14170,17 +13874,13 @@
       </c>
       <c r="C237" s="2" t="inlineStr">
         <is>
-          <t>Return Rank</t>
-        </is>
-      </c>
-      <c r="D237" s="2" t="inlineStr">
-        <is>
-          <t>9Y</t>
-        </is>
-      </c>
+          <t>Profile LT Score</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr"/>
       <c r="E237" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (1 = best)</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F237" s="2" t="inlineStr">
@@ -14190,14 +13890,14 @@
       </c>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>This IS the Profile LT score</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (10Y)</t>
+          <t>Profile LT Rank In Category</t>
         </is>
       </c>
       <c r="B238" s="2" t="inlineStr">
@@ -14207,17 +13907,13 @@
       </c>
       <c r="C238" s="2" t="inlineStr">
         <is>
-          <t>Return Rank</t>
-        </is>
-      </c>
-      <c r="D238" s="2" t="inlineStr">
-        <is>
-          <t>10Y</t>
-        </is>
-      </c>
+          <t>Profile LT Rank In Category</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr"/>
       <c r="E238" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (1 = best)</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F238" s="2" t="inlineStr">
@@ -14234,7 +13930,7 @@
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (15Y)</t>
+          <t>Profile LT Rank Overall</t>
         </is>
       </c>
       <c r="B239" s="2" t="inlineStr">
@@ -14244,17 +13940,13 @@
       </c>
       <c r="C239" s="2" t="inlineStr">
         <is>
-          <t>Return Rank</t>
-        </is>
-      </c>
-      <c r="D239" s="2" t="inlineStr">
-        <is>
-          <t>15Y</t>
-        </is>
-      </c>
+          <t>Profile LT Rank Overall</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr"/>
       <c r="E239" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (1 = best)</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F239" s="2" t="inlineStr">
@@ -14271,7 +13963,7 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>Return Rank (20Y)</t>
+          <t>Profile ST Score</t>
         </is>
       </c>
       <c r="B240" s="2" t="inlineStr">
@@ -14281,17 +13973,13 @@
       </c>
       <c r="C240" s="2" t="inlineStr">
         <is>
-          <t>Return Rank</t>
-        </is>
-      </c>
-      <c r="D240" s="2" t="inlineStr">
-        <is>
-          <t>20Y</t>
-        </is>
-      </c>
+          <t>Profile ST Score</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr"/>
       <c r="E240" s="2" t="inlineStr">
         <is>
-          <t>Lower is better (1 = best)</t>
+          <t>Higher is better</t>
         </is>
       </c>
       <c r="F240" s="2" t="inlineStr">
@@ -14301,14 +13989,14 @@
       </c>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>No - this is the Profile ST score</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Score</t>
+          <t>Profile ST Rank In Category</t>
         </is>
       </c>
       <c r="B241" s="2" t="inlineStr">
@@ -14318,13 +14006,13 @@
       </c>
       <c r="C241" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Score</t>
+          <t>Profile ST Rank In Category</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr"/>
       <c r="E241" s="2" t="inlineStr">
         <is>
-          <t>Higher is better</t>
+          <t>Lower is better</t>
         </is>
       </c>
       <c r="F241" s="2" t="inlineStr">
@@ -14334,14 +14022,14 @@
       </c>
       <c r="G241" s="2" t="inlineStr">
         <is>
-          <t>This IS the Profile LT score</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank In Category</t>
+          <t>Profile ST Rank Overall</t>
         </is>
       </c>
       <c r="B242" s="2" t="inlineStr">
@@ -14351,7 +14039,7 @@
       </c>
       <c r="C242" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Rank In Category</t>
+          <t>Profile ST Rank Overall</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr"/>
@@ -14374,23 +14062,23 @@
     <row r="243">
       <c r="A243" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Selected Flag</t>
+          <t>Missing From Yahoo</t>
         </is>
       </c>
       <c r="B243" s="2" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>No Yahoo Data</t>
         </is>
       </c>
       <c r="C243" s="2" t="inlineStr">
         <is>
-          <t>Profile LT Selected Flag</t>
+          <t>Missing From Yahoo</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr"/>
       <c r="E243" s="2" t="inlineStr">
         <is>
-          <t>1 = selected</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="F243" s="2" t="inlineStr">
@@ -14404,272 +14092,8 @@
         </is>
       </c>
     </row>
-    <row r="244">
-      <c r="A244" s="2" t="inlineStr">
-        <is>
-          <t>Profile LT Rank Overall</t>
-        </is>
-      </c>
-      <c r="B244" s="2" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="C244" s="2" t="inlineStr">
-        <is>
-          <t>Profile LT Rank Overall</t>
-        </is>
-      </c>
-      <c r="D244" s="2" t="inlineStr"/>
-      <c r="E244" s="2" t="inlineStr">
-        <is>
-          <t>Lower is better</t>
-        </is>
-      </c>
-      <c r="F244" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G244" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" s="2" t="inlineStr">
-        <is>
-          <t>Profile LT Selected Overall Flag</t>
-        </is>
-      </c>
-      <c r="B245" s="2" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="C245" s="2" t="inlineStr">
-        <is>
-          <t>Profile LT Selected Overall Flag</t>
-        </is>
-      </c>
-      <c r="D245" s="2" t="inlineStr"/>
-      <c r="E245" s="2" t="inlineStr">
-        <is>
-          <t>1 = selected</t>
-        </is>
-      </c>
-      <c r="F245" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G245" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Score</t>
-        </is>
-      </c>
-      <c r="B246" s="2" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="C246" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Score</t>
-        </is>
-      </c>
-      <c r="D246" s="2" t="inlineStr"/>
-      <c r="E246" s="2" t="inlineStr">
-        <is>
-          <t>Higher is better</t>
-        </is>
-      </c>
-      <c r="F246" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G246" s="2" t="inlineStr">
-        <is>
-          <t>No - this is the Profile ST score</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Rank In Category</t>
-        </is>
-      </c>
-      <c r="B247" s="2" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="C247" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Rank In Category</t>
-        </is>
-      </c>
-      <c r="D247" s="2" t="inlineStr"/>
-      <c r="E247" s="2" t="inlineStr">
-        <is>
-          <t>Lower is better</t>
-        </is>
-      </c>
-      <c r="F247" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G247" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Selected Flag</t>
-        </is>
-      </c>
-      <c r="B248" s="2" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="C248" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Selected Flag</t>
-        </is>
-      </c>
-      <c r="D248" s="2" t="inlineStr"/>
-      <c r="E248" s="2" t="inlineStr">
-        <is>
-          <t>1 = selected</t>
-        </is>
-      </c>
-      <c r="F248" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G248" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Rank Overall</t>
-        </is>
-      </c>
-      <c r="B249" s="2" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="C249" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Rank Overall</t>
-        </is>
-      </c>
-      <c r="D249" s="2" t="inlineStr"/>
-      <c r="E249" s="2" t="inlineStr">
-        <is>
-          <t>Lower is better</t>
-        </is>
-      </c>
-      <c r="F249" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G249" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Selected Overall Flag</t>
-        </is>
-      </c>
-      <c r="B250" s="2" t="inlineStr">
-        <is>
-          <t>Overview</t>
-        </is>
-      </c>
-      <c r="C250" s="2" t="inlineStr">
-        <is>
-          <t>Profile ST Selected Overall Flag</t>
-        </is>
-      </c>
-      <c r="D250" s="2" t="inlineStr"/>
-      <c r="E250" s="2" t="inlineStr">
-        <is>
-          <t>1 = selected</t>
-        </is>
-      </c>
-      <c r="F250" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G250" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" s="2" t="inlineStr">
-        <is>
-          <t>Missing From Yahoo</t>
-        </is>
-      </c>
-      <c r="B251" s="2" t="inlineStr">
-        <is>
-          <t>No Yahoo Data</t>
-        </is>
-      </c>
-      <c r="C251" s="2" t="inlineStr">
-        <is>
-          <t>Missing From Yahoo</t>
-        </is>
-      </c>
-      <c r="D251" s="2" t="inlineStr"/>
-      <c r="E251" s="2" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="F251" s="2" t="inlineStr">
-        <is>
-          <t>Screener (calculated)</t>
-        </is>
-      </c>
-      <c r="G251" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G251"/>
+  <autoFilter ref="A1:G243"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14736,11 +14160,11 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>23.8%</t>
+          <t>28.6%</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -14841,11 +14265,11 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>9.5%</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -14876,11 +14300,11 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -15016,11 +14440,11 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>9.5%</t>
+          <t>4.8%</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">

</xml_diff>